<commit_message>
vault backup: 2026-04-01 11:32:06
</commit_message>
<xml_diff>
--- a/睡眠日记_Sleep_Diary1.xlsx
+++ b/睡眠日记_Sleep_Diary1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\My_lovwly\test\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My_like\My_like\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FD508A6-4D2B-4D17-AE07-FBE81090097E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7C51281-174B-4EA0-96B4-E26F95FB0C9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="睡眠日记 Sleep Diary" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="660" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="688" uniqueCount="175">
   <si>
     <t>睡眠日记 Sleep Diary</t>
   </si>
@@ -614,6 +614,9 @@
   </si>
   <si>
     <t>60 min</t>
+  </si>
+  <si>
+    <t>4点被猫吵醒</t>
   </si>
 </sst>
 </file>
@@ -792,6 +795,9 @@
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="20" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -808,9 +814,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1114,51 +1117,51 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H212"/>
-  <sheetFormatPr defaultColWidth="10" defaultRowHeight="15"/>
+  <dimension ref="A1:H231"/>
+  <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="8" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="22.5">
-      <c r="A1" s="16" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="18"/>
-    </row>
-    <row r="2" spans="1:8" ht="17.25">
-      <c r="A2" s="19" t="s">
+    <row r="1" spans="1:8" ht="23.4">
+      <c r="A1" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="19"/>
+    </row>
+    <row r="2" spans="1:8" ht="17.399999999999999">
+      <c r="A2" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="18"/>
-    </row>
-    <row r="3" spans="1:8" ht="16.5">
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="19"/>
+    </row>
+    <row r="3" spans="1:8" ht="15.6">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14"/>
-      <c r="H3" s="15"/>
-    </row>
-    <row r="4" spans="1:8" ht="54">
+      <c r="C3" s="15"/>
+      <c r="D3" s="15"/>
+      <c r="E3" s="15"/>
+      <c r="F3" s="15"/>
+      <c r="G3" s="15"/>
+      <c r="H3" s="16"/>
+    </row>
+    <row r="4" spans="1:8" ht="34.799999999999997">
       <c r="A4" s="2"/>
       <c r="B4" s="2" t="s">
         <v>20</v>
@@ -1182,7 +1185,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="33">
+    <row r="5" spans="1:8" ht="31.2">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -1208,7 +1211,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="16.5">
+    <row r="6" spans="1:8" ht="15.6">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
@@ -1234,7 +1237,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="16.5">
+    <row r="7" spans="1:8" ht="15.6">
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
@@ -1260,7 +1263,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="16.5">
+    <row r="8" spans="1:8" ht="15.6">
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
@@ -1286,7 +1289,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="49.5">
+    <row r="9" spans="1:8" ht="31.2">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
@@ -1312,7 +1315,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="16.5">
+    <row r="10" spans="1:8" ht="15.6">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
@@ -1338,7 +1341,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="33">
+    <row r="11" spans="1:8" ht="31.2">
       <c r="A11" s="1" t="s">
         <v>9</v>
       </c>
@@ -1364,7 +1367,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="33">
+    <row r="12" spans="1:8" ht="31.2">
       <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
@@ -1390,7 +1393,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="82.5">
+    <row r="13" spans="1:8" ht="62.4">
       <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
@@ -1416,7 +1419,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="66">
+    <row r="14" spans="1:8" ht="62.4">
       <c r="A14" s="1" t="s">
         <v>12</v>
       </c>
@@ -1442,7 +1445,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="49.5">
+    <row r="15" spans="1:8" ht="46.8">
       <c r="A15" s="1" t="s">
         <v>40</v>
       </c>
@@ -1468,7 +1471,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="99">
+    <row r="16" spans="1:8" ht="93.6">
       <c r="A16" s="1" t="s">
         <v>27</v>
       </c>
@@ -1494,7 +1497,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="115.5">
+    <row r="17" spans="1:8" ht="109.2">
       <c r="A17" s="1" t="s">
         <v>28</v>
       </c>
@@ -1520,7 +1523,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="66">
+    <row r="18" spans="1:8" ht="62.4">
       <c r="A18" s="1" t="s">
         <v>13</v>
       </c>
@@ -1549,45 +1552,45 @@
     <row r="20" spans="1:8">
       <c r="A20" s="3"/>
     </row>
-    <row r="21" spans="1:8" ht="22.5">
-      <c r="A21" s="16" t="s">
-        <v>0</v>
-      </c>
-      <c r="B21" s="17"/>
-      <c r="C21" s="17"/>
-      <c r="D21" s="17"/>
-      <c r="E21" s="17"/>
-      <c r="F21" s="17"/>
-      <c r="G21" s="17"/>
-      <c r="H21" s="18"/>
-    </row>
-    <row r="22" spans="1:8" ht="17.25">
-      <c r="A22" s="19" t="s">
+    <row r="21" spans="1:8" ht="23.4">
+      <c r="A21" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="B21" s="18"/>
+      <c r="C21" s="18"/>
+      <c r="D21" s="18"/>
+      <c r="E21" s="18"/>
+      <c r="F21" s="18"/>
+      <c r="G21" s="18"/>
+      <c r="H21" s="19"/>
+    </row>
+    <row r="22" spans="1:8" ht="17.399999999999999">
+      <c r="A22" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B22" s="17"/>
-      <c r="C22" s="17"/>
-      <c r="D22" s="17"/>
-      <c r="E22" s="17"/>
-      <c r="F22" s="17"/>
-      <c r="G22" s="17"/>
-      <c r="H22" s="18"/>
-    </row>
-    <row r="23" spans="1:8" ht="16.5">
+      <c r="B22" s="18"/>
+      <c r="C22" s="18"/>
+      <c r="D22" s="18"/>
+      <c r="E22" s="18"/>
+      <c r="F22" s="18"/>
+      <c r="G22" s="18"/>
+      <c r="H22" s="19"/>
+    </row>
+    <row r="23" spans="1:8" ht="15.6">
       <c r="A23" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B23" s="13" t="s">
+      <c r="B23" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="C23" s="14"/>
-      <c r="D23" s="14"/>
-      <c r="E23" s="14"/>
-      <c r="F23" s="14"/>
-      <c r="G23" s="14"/>
-      <c r="H23" s="15"/>
-    </row>
-    <row r="24" spans="1:8" ht="54">
+      <c r="C23" s="15"/>
+      <c r="D23" s="15"/>
+      <c r="E23" s="15"/>
+      <c r="F23" s="15"/>
+      <c r="G23" s="15"/>
+      <c r="H23" s="16"/>
+    </row>
+    <row r="24" spans="1:8" ht="34.799999999999997">
       <c r="A24" s="2"/>
       <c r="B24" s="2" t="s">
         <v>45</v>
@@ -1611,7 +1614,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="33">
+    <row r="25" spans="1:8" ht="31.2">
       <c r="A25" s="1" t="s">
         <v>3</v>
       </c>
@@ -1637,7 +1640,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="16.5">
+    <row r="26" spans="1:8" ht="15.6">
       <c r="A26" s="1" t="s">
         <v>4</v>
       </c>
@@ -1663,7 +1666,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="16.5">
+    <row r="27" spans="1:8" ht="15.6">
       <c r="A27" s="1" t="s">
         <v>5</v>
       </c>
@@ -1689,7 +1692,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="16.5">
+    <row r="28" spans="1:8" ht="15.6">
       <c r="A28" s="1" t="s">
         <v>6</v>
       </c>
@@ -1715,7 +1718,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="49.5">
+    <row r="29" spans="1:8" ht="31.2">
       <c r="A29" s="1" t="s">
         <v>7</v>
       </c>
@@ -1741,7 +1744,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="16.5">
+    <row r="30" spans="1:8" ht="15.6">
       <c r="A30" s="1" t="s">
         <v>8</v>
       </c>
@@ -1767,7 +1770,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="33">
+    <row r="31" spans="1:8" ht="31.2">
       <c r="A31" s="1" t="s">
         <v>9</v>
       </c>
@@ -1793,7 +1796,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="33">
+    <row r="32" spans="1:8" ht="31.2">
       <c r="A32" s="1" t="s">
         <v>10</v>
       </c>
@@ -1819,7 +1822,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="82.5">
+    <row r="33" spans="1:8" ht="62.4">
       <c r="A33" s="1" t="s">
         <v>11</v>
       </c>
@@ -1845,7 +1848,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="66">
+    <row r="34" spans="1:8" ht="62.4">
       <c r="A34" s="1" t="s">
         <v>12</v>
       </c>
@@ -1871,7 +1874,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="49.5">
+    <row r="35" spans="1:8" ht="46.8">
       <c r="A35" s="1" t="s">
         <v>40</v>
       </c>
@@ -1897,7 +1900,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="99">
+    <row r="36" spans="1:8" ht="93.6">
       <c r="A36" s="1" t="s">
         <v>27</v>
       </c>
@@ -1923,7 +1926,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="115.5">
+    <row r="37" spans="1:8" ht="109.2">
       <c r="A37" s="1" t="s">
         <v>28</v>
       </c>
@@ -1949,7 +1952,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="66">
+    <row r="38" spans="1:8" ht="62.4">
       <c r="A38" s="1" t="s">
         <v>13</v>
       </c>
@@ -1975,45 +1978,45 @@
         <v>77</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="22.5">
-      <c r="A40" s="16" t="s">
-        <v>0</v>
-      </c>
-      <c r="B40" s="17"/>
-      <c r="C40" s="17"/>
-      <c r="D40" s="17"/>
-      <c r="E40" s="17"/>
-      <c r="F40" s="17"/>
-      <c r="G40" s="17"/>
-      <c r="H40" s="18"/>
-    </row>
-    <row r="41" spans="1:8" ht="17.25">
-      <c r="A41" s="19" t="s">
+    <row r="40" spans="1:8" ht="23.4">
+      <c r="A40" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="B40" s="18"/>
+      <c r="C40" s="18"/>
+      <c r="D40" s="18"/>
+      <c r="E40" s="18"/>
+      <c r="F40" s="18"/>
+      <c r="G40" s="18"/>
+      <c r="H40" s="19"/>
+    </row>
+    <row r="41" spans="1:8" ht="17.399999999999999">
+      <c r="A41" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B41" s="17"/>
-      <c r="C41" s="17"/>
-      <c r="D41" s="17"/>
-      <c r="E41" s="17"/>
-      <c r="F41" s="17"/>
-      <c r="G41" s="17"/>
-      <c r="H41" s="18"/>
-    </row>
-    <row r="42" spans="1:8" ht="16.5">
+      <c r="B41" s="18"/>
+      <c r="C41" s="18"/>
+      <c r="D41" s="18"/>
+      <c r="E41" s="18"/>
+      <c r="F41" s="18"/>
+      <c r="G41" s="18"/>
+      <c r="H41" s="19"/>
+    </row>
+    <row r="42" spans="1:8" ht="15.6">
       <c r="A42" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B42" s="13" t="s">
+      <c r="B42" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="C42" s="14"/>
-      <c r="D42" s="14"/>
-      <c r="E42" s="14"/>
-      <c r="F42" s="14"/>
-      <c r="G42" s="14"/>
-      <c r="H42" s="15"/>
-    </row>
-    <row r="43" spans="1:8" ht="54">
+      <c r="C42" s="15"/>
+      <c r="D42" s="15"/>
+      <c r="E42" s="15"/>
+      <c r="F42" s="15"/>
+      <c r="G42" s="15"/>
+      <c r="H42" s="16"/>
+    </row>
+    <row r="43" spans="1:8" ht="34.799999999999997">
       <c r="A43" s="2"/>
       <c r="B43" s="2" t="s">
         <v>53</v>
@@ -2037,7 +2040,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="44" spans="1:8" ht="33">
+    <row r="44" spans="1:8" ht="31.2">
       <c r="A44" s="1" t="s">
         <v>3</v>
       </c>
@@ -2063,7 +2066,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="45" spans="1:8" ht="16.5">
+    <row r="45" spans="1:8" ht="15.6">
       <c r="A45" s="1" t="s">
         <v>4</v>
       </c>
@@ -2089,7 +2092,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="46" spans="1:8" ht="16.5">
+    <row r="46" spans="1:8" ht="15.6">
       <c r="A46" s="1" t="s">
         <v>5</v>
       </c>
@@ -2115,7 +2118,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="47" spans="1:8" ht="16.5">
+    <row r="47" spans="1:8" ht="15.6">
       <c r="A47" s="1" t="s">
         <v>6</v>
       </c>
@@ -2141,7 +2144,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="48" spans="1:8" ht="49.5">
+    <row r="48" spans="1:8" ht="31.2">
       <c r="A48" s="1" t="s">
         <v>7</v>
       </c>
@@ -2167,7 +2170,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="49" spans="1:8" ht="16.5">
+    <row r="49" spans="1:8" ht="15.6">
       <c r="A49" s="1" t="s">
         <v>8</v>
       </c>
@@ -2193,7 +2196,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:8" ht="33">
+    <row r="50" spans="1:8" ht="31.2">
       <c r="A50" s="1" t="s">
         <v>9</v>
       </c>
@@ -2219,7 +2222,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="51" spans="1:8" ht="33">
+    <row r="51" spans="1:8" ht="31.2">
       <c r="A51" s="1" t="s">
         <v>10</v>
       </c>
@@ -2245,7 +2248,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="52" spans="1:8" ht="82.5">
+    <row r="52" spans="1:8" ht="62.4">
       <c r="A52" s="1" t="s">
         <v>11</v>
       </c>
@@ -2271,7 +2274,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="53" spans="1:8" ht="66">
+    <row r="53" spans="1:8" ht="62.4">
       <c r="A53" s="1" t="s">
         <v>12</v>
       </c>
@@ -2297,7 +2300,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="54" spans="1:8" ht="49.5">
+    <row r="54" spans="1:8" ht="46.8">
       <c r="A54" s="1" t="s">
         <v>40</v>
       </c>
@@ -2323,7 +2326,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="55" spans="1:8" ht="99">
+    <row r="55" spans="1:8" ht="93.6">
       <c r="A55" s="1" t="s">
         <v>27</v>
       </c>
@@ -2349,7 +2352,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="56" spans="1:8" ht="115.5">
+    <row r="56" spans="1:8" ht="109.2">
       <c r="A56" s="1" t="s">
         <v>28</v>
       </c>
@@ -2375,7 +2378,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="57" spans="1:8" ht="66">
+    <row r="57" spans="1:8" ht="62.4">
       <c r="A57" s="1" t="s">
         <v>13</v>
       </c>
@@ -2401,45 +2404,45 @@
         <v>26</v>
       </c>
     </row>
-    <row r="59" spans="1:8" ht="22.5">
-      <c r="A59" s="16" t="s">
-        <v>0</v>
-      </c>
-      <c r="B59" s="17"/>
-      <c r="C59" s="17"/>
-      <c r="D59" s="17"/>
-      <c r="E59" s="17"/>
-      <c r="F59" s="17"/>
-      <c r="G59" s="17"/>
-      <c r="H59" s="18"/>
-    </row>
-    <row r="60" spans="1:8" ht="17.25">
-      <c r="A60" s="19" t="s">
+    <row r="59" spans="1:8" ht="23.4">
+      <c r="A59" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="B59" s="18"/>
+      <c r="C59" s="18"/>
+      <c r="D59" s="18"/>
+      <c r="E59" s="18"/>
+      <c r="F59" s="18"/>
+      <c r="G59" s="18"/>
+      <c r="H59" s="19"/>
+    </row>
+    <row r="60" spans="1:8" ht="17.399999999999999">
+      <c r="A60" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B60" s="17"/>
-      <c r="C60" s="17"/>
-      <c r="D60" s="17"/>
-      <c r="E60" s="17"/>
-      <c r="F60" s="17"/>
-      <c r="G60" s="17"/>
-      <c r="H60" s="18"/>
-    </row>
-    <row r="61" spans="1:8" ht="16.5">
+      <c r="B60" s="18"/>
+      <c r="C60" s="18"/>
+      <c r="D60" s="18"/>
+      <c r="E60" s="18"/>
+      <c r="F60" s="18"/>
+      <c r="G60" s="18"/>
+      <c r="H60" s="19"/>
+    </row>
+    <row r="61" spans="1:8" ht="15.6">
       <c r="A61" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B61" s="13" t="s">
+      <c r="B61" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="C61" s="14"/>
-      <c r="D61" s="14"/>
-      <c r="E61" s="14"/>
-      <c r="F61" s="14"/>
-      <c r="G61" s="14"/>
-      <c r="H61" s="15"/>
-    </row>
-    <row r="62" spans="1:8" ht="54">
+      <c r="C61" s="15"/>
+      <c r="D61" s="15"/>
+      <c r="E61" s="15"/>
+      <c r="F61" s="15"/>
+      <c r="G61" s="15"/>
+      <c r="H61" s="16"/>
+    </row>
+    <row r="62" spans="1:8" ht="34.799999999999997">
       <c r="A62" s="2"/>
       <c r="B62" s="2" t="s">
         <v>83</v>
@@ -2463,7 +2466,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="63" spans="1:8" ht="33">
+    <row r="63" spans="1:8" ht="31.2">
       <c r="A63" s="1" t="s">
         <v>3</v>
       </c>
@@ -2489,7 +2492,7 @@
         <v>0.28611111111111109</v>
       </c>
     </row>
-    <row r="64" spans="1:8" ht="16.5">
+    <row r="64" spans="1:8" ht="15.6">
       <c r="A64" s="1" t="s">
         <v>4</v>
       </c>
@@ -2515,7 +2518,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="65" spans="1:8" ht="16.5">
+    <row r="65" spans="1:8" ht="15.6">
       <c r="A65" s="1" t="s">
         <v>5</v>
       </c>
@@ -2541,7 +2544,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="66" spans="1:8" ht="16.5">
+    <row r="66" spans="1:8" ht="15.6">
       <c r="A66" s="1" t="s">
         <v>6</v>
       </c>
@@ -2567,7 +2570,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="67" spans="1:8" ht="49.5">
+    <row r="67" spans="1:8" ht="31.2">
       <c r="A67" s="1" t="s">
         <v>7</v>
       </c>
@@ -2593,7 +2596,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="68" spans="1:8" ht="16.5">
+    <row r="68" spans="1:8" ht="15.6">
       <c r="A68" s="1" t="s">
         <v>8</v>
       </c>
@@ -2619,7 +2622,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:8" ht="33">
+    <row r="69" spans="1:8" ht="31.2">
       <c r="A69" s="1" t="s">
         <v>9</v>
       </c>
@@ -2645,7 +2648,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="70" spans="1:8" ht="33">
+    <row r="70" spans="1:8" ht="31.2">
       <c r="A70" s="1" t="s">
         <v>10</v>
       </c>
@@ -2671,7 +2674,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="71" spans="1:8" ht="82.5">
+    <row r="71" spans="1:8" ht="62.4">
       <c r="A71" s="1" t="s">
         <v>11</v>
       </c>
@@ -2697,7 +2700,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="72" spans="1:8" ht="66">
+    <row r="72" spans="1:8" ht="62.4">
       <c r="A72" s="1" t="s">
         <v>12</v>
       </c>
@@ -2723,7 +2726,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="73" spans="1:8" ht="49.5">
+    <row r="73" spans="1:8" ht="46.8">
       <c r="A73" s="1" t="s">
         <v>40</v>
       </c>
@@ -2749,7 +2752,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="74" spans="1:8" ht="99">
+    <row r="74" spans="1:8" ht="93.6">
       <c r="A74" s="1" t="s">
         <v>27</v>
       </c>
@@ -2775,7 +2778,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="75" spans="1:8" ht="115.5">
+    <row r="75" spans="1:8" ht="109.2">
       <c r="A75" s="1" t="s">
         <v>28</v>
       </c>
@@ -2801,7 +2804,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="76" spans="1:8" ht="66">
+    <row r="76" spans="1:8" ht="62.4">
       <c r="A76" s="1" t="s">
         <v>13</v>
       </c>
@@ -2827,33 +2830,33 @@
         <v>26</v>
       </c>
     </row>
-    <row r="79" spans="1:8" ht="17.25">
-      <c r="A79" s="19" t="s">
+    <row r="79" spans="1:8" ht="17.399999999999999">
+      <c r="A79" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B79" s="17"/>
-      <c r="C79" s="17"/>
-      <c r="D79" s="17"/>
-      <c r="E79" s="17"/>
-      <c r="F79" s="17"/>
-      <c r="G79" s="17"/>
-      <c r="H79" s="18"/>
-    </row>
-    <row r="80" spans="1:8" ht="16.5">
+      <c r="B79" s="18"/>
+      <c r="C79" s="18"/>
+      <c r="D79" s="18"/>
+      <c r="E79" s="18"/>
+      <c r="F79" s="18"/>
+      <c r="G79" s="18"/>
+      <c r="H79" s="19"/>
+    </row>
+    <row r="80" spans="1:8" ht="15.6">
       <c r="A80" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B80" s="13" t="s">
+      <c r="B80" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="C80" s="14"/>
-      <c r="D80" s="14"/>
-      <c r="E80" s="14"/>
-      <c r="F80" s="14"/>
-      <c r="G80" s="14"/>
-      <c r="H80" s="15"/>
-    </row>
-    <row r="81" spans="1:8" ht="54">
+      <c r="C80" s="15"/>
+      <c r="D80" s="15"/>
+      <c r="E80" s="15"/>
+      <c r="F80" s="15"/>
+      <c r="G80" s="15"/>
+      <c r="H80" s="16"/>
+    </row>
+    <row r="81" spans="1:8" ht="34.799999999999997">
       <c r="A81" s="2"/>
       <c r="B81" s="2" t="s">
         <v>97</v>
@@ -2877,7 +2880,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="82" spans="1:8" ht="33">
+    <row r="82" spans="1:8" ht="31.2">
       <c r="A82" s="1" t="s">
         <v>3</v>
       </c>
@@ -2903,7 +2906,7 @@
         <v>0.30069444444444449</v>
       </c>
     </row>
-    <row r="83" spans="1:8" ht="16.5">
+    <row r="83" spans="1:8" ht="15.6">
       <c r="A83" s="1" t="s">
         <v>4</v>
       </c>
@@ -2929,7 +2932,7 @@
         <v>0.30069444444444449</v>
       </c>
     </row>
-    <row r="84" spans="1:8" ht="16.5">
+    <row r="84" spans="1:8" ht="15.6">
       <c r="A84" s="1" t="s">
         <v>5</v>
       </c>
@@ -2955,7 +2958,7 @@
         <v>0.97222222222222221</v>
       </c>
     </row>
-    <row r="85" spans="1:8" ht="16.5">
+    <row r="85" spans="1:8" ht="15.6">
       <c r="A85" s="1" t="s">
         <v>6</v>
       </c>
@@ -2981,7 +2984,7 @@
         <v>0.97222222222222221</v>
       </c>
     </row>
-    <row r="86" spans="1:8" ht="49.5">
+    <row r="86" spans="1:8" ht="31.2">
       <c r="A86" s="1" t="s">
         <v>7</v>
       </c>
@@ -3007,7 +3010,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="87" spans="1:8" ht="16.5">
+    <row r="87" spans="1:8" ht="15.6">
       <c r="A87" s="1" t="s">
         <v>8</v>
       </c>
@@ -3033,7 +3036,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:8" ht="33">
+    <row r="88" spans="1:8" ht="31.2">
       <c r="A88" s="1" t="s">
         <v>9</v>
       </c>
@@ -3059,7 +3062,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:8" ht="33">
+    <row r="89" spans="1:8" ht="31.2">
       <c r="A89" s="1" t="s">
         <v>10</v>
       </c>
@@ -3085,7 +3088,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="90" spans="1:8" ht="82.5">
+    <row r="90" spans="1:8" ht="62.4">
       <c r="A90" s="1" t="s">
         <v>11</v>
       </c>
@@ -3111,7 +3114,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="91" spans="1:8" ht="66">
+    <row r="91" spans="1:8" ht="62.4">
       <c r="A91" s="1" t="s">
         <v>12</v>
       </c>
@@ -3137,7 +3140,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="92" spans="1:8" ht="49.5">
+    <row r="92" spans="1:8" ht="46.8">
       <c r="A92" s="1" t="s">
         <v>40</v>
       </c>
@@ -3163,7 +3166,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="93" spans="1:8" ht="99">
+    <row r="93" spans="1:8" ht="93.6">
       <c r="A93" s="1" t="s">
         <v>27</v>
       </c>
@@ -3189,7 +3192,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="94" spans="1:8" ht="115.5">
+    <row r="94" spans="1:8" ht="109.2">
       <c r="A94" s="1" t="s">
         <v>28</v>
       </c>
@@ -3215,7 +3218,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="95" spans="1:8" ht="66">
+    <row r="95" spans="1:8" ht="62.4">
       <c r="A95" s="1" t="s">
         <v>13</v>
       </c>
@@ -3246,33 +3249,33 @@
         <v>112</v>
       </c>
     </row>
-    <row r="101" spans="1:8" ht="17.25">
-      <c r="A101" s="19" t="s">
+    <row r="101" spans="1:8" ht="17.399999999999999">
+      <c r="A101" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B101" s="17"/>
-      <c r="C101" s="17"/>
-      <c r="D101" s="17"/>
-      <c r="E101" s="17"/>
-      <c r="F101" s="17"/>
-      <c r="G101" s="17"/>
-      <c r="H101" s="18"/>
-    </row>
-    <row r="102" spans="1:8" ht="16.5">
+      <c r="B101" s="18"/>
+      <c r="C101" s="18"/>
+      <c r="D101" s="18"/>
+      <c r="E101" s="18"/>
+      <c r="F101" s="18"/>
+      <c r="G101" s="18"/>
+      <c r="H101" s="19"/>
+    </row>
+    <row r="102" spans="1:8" ht="15.6">
       <c r="A102" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B102" s="13" t="s">
+      <c r="B102" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="C102" s="14"/>
-      <c r="D102" s="14"/>
-      <c r="E102" s="14"/>
-      <c r="F102" s="14"/>
-      <c r="G102" s="14"/>
-      <c r="H102" s="15"/>
-    </row>
-    <row r="103" spans="1:8" ht="54">
+      <c r="C102" s="15"/>
+      <c r="D102" s="15"/>
+      <c r="E102" s="15"/>
+      <c r="F102" s="15"/>
+      <c r="G102" s="15"/>
+      <c r="H102" s="16"/>
+    </row>
+    <row r="103" spans="1:8" ht="34.799999999999997">
       <c r="A103" s="2"/>
       <c r="B103" s="2" t="s">
         <v>113</v>
@@ -3296,7 +3299,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="104" spans="1:8" ht="33">
+    <row r="104" spans="1:8" ht="31.2">
       <c r="A104" s="1" t="s">
         <v>3</v>
       </c>
@@ -3322,7 +3325,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="105" spans="1:8" ht="16.5">
+    <row r="105" spans="1:8" ht="15.6">
       <c r="A105" s="1" t="s">
         <v>4</v>
       </c>
@@ -3348,7 +3351,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="106" spans="1:8" ht="16.5">
+    <row r="106" spans="1:8" ht="15.6">
       <c r="A106" s="1" t="s">
         <v>5</v>
       </c>
@@ -3374,7 +3377,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="107" spans="1:8" ht="16.5">
+    <row r="107" spans="1:8" ht="15.6">
       <c r="A107" s="1" t="s">
         <v>6</v>
       </c>
@@ -3400,7 +3403,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="108" spans="1:8" ht="49.5">
+    <row r="108" spans="1:8" ht="31.2">
       <c r="A108" s="1" t="s">
         <v>7</v>
       </c>
@@ -3426,7 +3429,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="109" spans="1:8" ht="16.5">
+    <row r="109" spans="1:8" ht="15.6">
       <c r="A109" s="1" t="s">
         <v>8</v>
       </c>
@@ -3452,7 +3455,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:8" ht="33">
+    <row r="110" spans="1:8" ht="31.2">
       <c r="A110" s="1" t="s">
         <v>9</v>
       </c>
@@ -3478,7 +3481,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:8" ht="33">
+    <row r="111" spans="1:8" ht="31.2">
       <c r="A111" s="1" t="s">
         <v>10</v>
       </c>
@@ -3504,7 +3507,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="112" spans="1:8" ht="82.5">
+    <row r="112" spans="1:8" ht="62.4">
       <c r="A112" s="1" t="s">
         <v>11</v>
       </c>
@@ -3530,7 +3533,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="113" spans="1:8" ht="66">
+    <row r="113" spans="1:8" ht="62.4">
       <c r="A113" s="1" t="s">
         <v>12</v>
       </c>
@@ -3556,7 +3559,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="114" spans="1:8" ht="49.5">
+    <row r="114" spans="1:8" ht="46.8">
       <c r="A114" s="1" t="s">
         <v>40</v>
       </c>
@@ -3582,7 +3585,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="115" spans="1:8" ht="99">
+    <row r="115" spans="1:8" ht="93.6">
       <c r="A115" s="1" t="s">
         <v>27</v>
       </c>
@@ -3608,7 +3611,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="116" spans="1:8" ht="115.5">
+    <row r="116" spans="1:8" ht="109.2">
       <c r="A116" s="1" t="s">
         <v>28</v>
       </c>
@@ -3634,7 +3637,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="117" spans="1:8" ht="66">
+    <row r="117" spans="1:8" ht="62.4">
       <c r="A117" s="1" t="s">
         <v>13</v>
       </c>
@@ -3660,33 +3663,33 @@
         <v>128</v>
       </c>
     </row>
-    <row r="119" spans="1:8" ht="17.25">
-      <c r="A119" s="19" t="s">
+    <row r="119" spans="1:8" ht="17.399999999999999">
+      <c r="A119" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B119" s="17"/>
-      <c r="C119" s="17"/>
-      <c r="D119" s="17"/>
-      <c r="E119" s="17"/>
-      <c r="F119" s="17"/>
-      <c r="G119" s="17"/>
-      <c r="H119" s="18"/>
-    </row>
-    <row r="120" spans="1:8" ht="16.5">
+      <c r="B119" s="18"/>
+      <c r="C119" s="18"/>
+      <c r="D119" s="18"/>
+      <c r="E119" s="18"/>
+      <c r="F119" s="18"/>
+      <c r="G119" s="18"/>
+      <c r="H119" s="19"/>
+    </row>
+    <row r="120" spans="1:8" ht="15.6">
       <c r="A120" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B120" s="13" t="s">
+      <c r="B120" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="C120" s="14"/>
-      <c r="D120" s="14"/>
-      <c r="E120" s="14"/>
-      <c r="F120" s="14"/>
-      <c r="G120" s="14"/>
-      <c r="H120" s="15"/>
-    </row>
-    <row r="121" spans="1:8" ht="36">
+      <c r="C120" s="15"/>
+      <c r="D120" s="15"/>
+      <c r="E120" s="15"/>
+      <c r="F120" s="15"/>
+      <c r="G120" s="15"/>
+      <c r="H120" s="16"/>
+    </row>
+    <row r="121" spans="1:8" ht="34.799999999999997">
       <c r="A121" s="2"/>
       <c r="B121" s="2" t="s">
         <v>129</v>
@@ -3710,7 +3713,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="122" spans="1:8" ht="33">
+    <row r="122" spans="1:8" ht="31.2">
       <c r="A122" s="1" t="s">
         <v>3</v>
       </c>
@@ -3736,7 +3739,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="123" spans="1:8" ht="16.5">
+    <row r="123" spans="1:8" ht="15.6">
       <c r="A123" s="1" t="s">
         <v>4</v>
       </c>
@@ -3762,7 +3765,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="124" spans="1:8" ht="16.5">
+    <row r="124" spans="1:8" ht="15.6">
       <c r="A124" s="1" t="s">
         <v>5</v>
       </c>
@@ -3788,7 +3791,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="125" spans="1:8" ht="16.5">
+    <row r="125" spans="1:8" ht="15.6">
       <c r="A125" s="1" t="s">
         <v>6</v>
       </c>
@@ -3814,7 +3817,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="126" spans="1:8" ht="49.5">
+    <row r="126" spans="1:8" ht="31.2">
       <c r="A126" s="1" t="s">
         <v>7</v>
       </c>
@@ -3840,7 +3843,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="127" spans="1:8" ht="16.5">
+    <row r="127" spans="1:8" ht="15.6">
       <c r="A127" s="1" t="s">
         <v>8</v>
       </c>
@@ -3866,7 +3869,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:8" ht="33">
+    <row r="128" spans="1:8" ht="31.2">
       <c r="A128" s="1" t="s">
         <v>9</v>
       </c>
@@ -3892,7 +3895,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:8" ht="33">
+    <row r="129" spans="1:8" ht="31.2">
       <c r="A129" s="1" t="s">
         <v>10</v>
       </c>
@@ -3918,7 +3921,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="130" spans="1:8" ht="82.5">
+    <row r="130" spans="1:8" ht="62.4">
       <c r="A130" s="1" t="s">
         <v>11</v>
       </c>
@@ -3944,7 +3947,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="131" spans="1:8" ht="66">
+    <row r="131" spans="1:8" ht="62.4">
       <c r="A131" s="1" t="s">
         <v>12</v>
       </c>
@@ -3970,7 +3973,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="132" spans="1:8" ht="49.5">
+    <row r="132" spans="1:8" ht="46.8">
       <c r="A132" s="1" t="s">
         <v>40</v>
       </c>
@@ -3996,7 +3999,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="133" spans="1:8" ht="99">
+    <row r="133" spans="1:8" ht="93.6">
       <c r="A133" s="1" t="s">
         <v>27</v>
       </c>
@@ -4022,7 +4025,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="134" spans="1:8" ht="115.5">
+    <row r="134" spans="1:8" ht="109.2">
       <c r="A134" s="1" t="s">
         <v>28</v>
       </c>
@@ -4048,7 +4051,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="135" spans="1:8" ht="66">
+    <row r="135" spans="1:8" ht="62.4">
       <c r="A135" s="1" t="s">
         <v>13</v>
       </c>
@@ -4074,33 +4077,33 @@
         <v>26</v>
       </c>
     </row>
-    <row r="138" spans="1:8" ht="17.25">
-      <c r="A138" s="19" t="s">
+    <row r="138" spans="1:8" ht="17.399999999999999">
+      <c r="A138" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B138" s="17"/>
-      <c r="C138" s="17"/>
-      <c r="D138" s="17"/>
-      <c r="E138" s="17"/>
-      <c r="F138" s="17"/>
-      <c r="G138" s="17"/>
-      <c r="H138" s="18"/>
-    </row>
-    <row r="139" spans="1:8" ht="16.5">
+      <c r="B138" s="18"/>
+      <c r="C138" s="18"/>
+      <c r="D138" s="18"/>
+      <c r="E138" s="18"/>
+      <c r="F138" s="18"/>
+      <c r="G138" s="18"/>
+      <c r="H138" s="19"/>
+    </row>
+    <row r="139" spans="1:8" ht="15.6">
       <c r="A139" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B139" s="13" t="s">
+      <c r="B139" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="C139" s="14"/>
-      <c r="D139" s="14"/>
-      <c r="E139" s="14"/>
-      <c r="F139" s="14"/>
-      <c r="G139" s="14"/>
-      <c r="H139" s="15"/>
-    </row>
-    <row r="140" spans="1:8" ht="16.5">
+      <c r="C139" s="15"/>
+      <c r="D139" s="15"/>
+      <c r="E139" s="15"/>
+      <c r="F139" s="15"/>
+      <c r="G139" s="15"/>
+      <c r="H139" s="16"/>
+    </row>
+    <row r="140" spans="1:8" ht="15.6">
       <c r="A140" s="1"/>
       <c r="B140" s="8" t="s">
         <v>147</v>
@@ -4124,7 +4127,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="141" spans="1:8" ht="18">
+    <row r="141" spans="1:8" ht="17.399999999999999">
       <c r="A141" s="2"/>
       <c r="B141" s="11">
         <v>46032</v>
@@ -4154,7 +4157,7 @@
         <v>46038</v>
       </c>
     </row>
-    <row r="142" spans="1:8" ht="33">
+    <row r="142" spans="1:8" ht="31.2">
       <c r="A142" s="1" t="s">
         <v>3</v>
       </c>
@@ -4180,7 +4183,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="143" spans="1:8" ht="16.5">
+    <row r="143" spans="1:8" ht="15.6">
       <c r="A143" s="1" t="s">
         <v>4</v>
       </c>
@@ -4206,7 +4209,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="144" spans="1:8" ht="16.5">
+    <row r="144" spans="1:8" ht="15.6">
       <c r="A144" s="1" t="s">
         <v>5</v>
       </c>
@@ -4232,7 +4235,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="145" spans="1:8" ht="16.5">
+    <row r="145" spans="1:8" ht="15.6">
       <c r="A145" s="1" t="s">
         <v>6</v>
       </c>
@@ -4258,7 +4261,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="146" spans="1:8" ht="49.5">
+    <row r="146" spans="1:8" ht="31.2">
       <c r="A146" s="1" t="s">
         <v>7</v>
       </c>
@@ -4284,7 +4287,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="147" spans="1:8" ht="16.5">
+    <row r="147" spans="1:8" ht="15.6">
       <c r="A147" s="1" t="s">
         <v>8</v>
       </c>
@@ -4310,7 +4313,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="148" spans="1:8" ht="33">
+    <row r="148" spans="1:8" ht="31.2">
       <c r="A148" s="1" t="s">
         <v>9</v>
       </c>
@@ -4336,7 +4339,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="149" spans="1:8" ht="33">
+    <row r="149" spans="1:8" ht="31.2">
       <c r="A149" s="1" t="s">
         <v>10</v>
       </c>
@@ -4362,7 +4365,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="150" spans="1:8" ht="82.5">
+    <row r="150" spans="1:8" ht="62.4">
       <c r="A150" s="1" t="s">
         <v>11</v>
       </c>
@@ -4388,7 +4391,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="151" spans="1:8" ht="66">
+    <row r="151" spans="1:8" ht="62.4">
       <c r="A151" s="1" t="s">
         <v>12</v>
       </c>
@@ -4414,7 +4417,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="152" spans="1:8" ht="49.5">
+    <row r="152" spans="1:8" ht="46.8">
       <c r="A152" s="1" t="s">
         <v>40</v>
       </c>
@@ -4440,7 +4443,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="153" spans="1:8" ht="99">
+    <row r="153" spans="1:8" ht="93.6">
       <c r="A153" s="1" t="s">
         <v>27</v>
       </c>
@@ -4466,7 +4469,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="154" spans="1:8" ht="115.5">
+    <row r="154" spans="1:8" ht="109.2">
       <c r="A154" s="1" t="s">
         <v>28</v>
       </c>
@@ -4492,7 +4495,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="155" spans="1:8" ht="66">
+    <row r="155" spans="1:8" ht="62.4">
       <c r="A155" s="1" t="s">
         <v>13</v>
       </c>
@@ -4523,33 +4526,33 @@
         <v>154</v>
       </c>
     </row>
-    <row r="158" spans="1:8" ht="17.25">
-      <c r="A158" s="19" t="s">
+    <row r="158" spans="1:8" ht="17.399999999999999">
+      <c r="A158" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B158" s="17"/>
-      <c r="C158" s="17"/>
-      <c r="D158" s="17"/>
-      <c r="E158" s="17"/>
-      <c r="F158" s="17"/>
-      <c r="G158" s="17"/>
-      <c r="H158" s="18"/>
-    </row>
-    <row r="159" spans="1:8" ht="16.5">
+      <c r="B158" s="18"/>
+      <c r="C158" s="18"/>
+      <c r="D158" s="18"/>
+      <c r="E158" s="18"/>
+      <c r="F158" s="18"/>
+      <c r="G158" s="18"/>
+      <c r="H158" s="19"/>
+    </row>
+    <row r="159" spans="1:8" ht="15.6">
       <c r="A159" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B159" s="13" t="s">
+      <c r="B159" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="C159" s="14"/>
-      <c r="D159" s="14"/>
-      <c r="E159" s="14"/>
-      <c r="F159" s="14"/>
-      <c r="G159" s="14"/>
-      <c r="H159" s="15"/>
-    </row>
-    <row r="160" spans="1:8" ht="16.5">
+      <c r="C159" s="15"/>
+      <c r="D159" s="15"/>
+      <c r="E159" s="15"/>
+      <c r="F159" s="15"/>
+      <c r="G159" s="15"/>
+      <c r="H159" s="16"/>
+    </row>
+    <row r="160" spans="1:8" ht="15.6">
       <c r="A160" s="1"/>
       <c r="B160" s="8" t="s">
         <v>147</v>
@@ -4573,7 +4576,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="161" spans="1:8" ht="18">
+    <row r="161" spans="1:8" ht="17.399999999999999">
       <c r="A161" s="2"/>
       <c r="B161" s="11">
         <v>46039</v>
@@ -4603,7 +4606,7 @@
         <v>46045</v>
       </c>
     </row>
-    <row r="162" spans="1:8" ht="33">
+    <row r="162" spans="1:8" ht="31.2">
       <c r="A162" s="1" t="s">
         <v>3</v>
       </c>
@@ -4629,7 +4632,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="163" spans="1:8" ht="16.5">
+    <row r="163" spans="1:8" ht="15.6">
       <c r="A163" s="1" t="s">
         <v>4</v>
       </c>
@@ -4655,7 +4658,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="164" spans="1:8" ht="16.5">
+    <row r="164" spans="1:8" ht="15.6">
       <c r="A164" s="1" t="s">
         <v>5</v>
       </c>
@@ -4681,7 +4684,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="165" spans="1:8" ht="16.5">
+    <row r="165" spans="1:8" ht="15.6">
       <c r="A165" s="1" t="s">
         <v>6</v>
       </c>
@@ -4707,7 +4710,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="166" spans="1:8" ht="49.5">
+    <row r="166" spans="1:8" ht="31.2">
       <c r="A166" s="1" t="s">
         <v>7</v>
       </c>
@@ -4733,7 +4736,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="167" spans="1:8" ht="16.5">
+    <row r="167" spans="1:8" ht="15.6">
       <c r="A167" s="1" t="s">
         <v>8</v>
       </c>
@@ -4759,7 +4762,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="168" spans="1:8" ht="33">
+    <row r="168" spans="1:8" ht="31.2">
       <c r="A168" s="1" t="s">
         <v>9</v>
       </c>
@@ -4785,7 +4788,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="169" spans="1:8" ht="33">
+    <row r="169" spans="1:8" ht="31.2">
       <c r="A169" s="1" t="s">
         <v>10</v>
       </c>
@@ -4811,7 +4814,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="170" spans="1:8" ht="82.5">
+    <row r="170" spans="1:8" ht="62.4">
       <c r="A170" s="1" t="s">
         <v>11</v>
       </c>
@@ -4837,7 +4840,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="171" spans="1:8" ht="66">
+    <row r="171" spans="1:8" ht="62.4">
       <c r="A171" s="1" t="s">
         <v>12</v>
       </c>
@@ -4863,7 +4866,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:8" ht="49.5">
+    <row r="172" spans="1:8" ht="46.8">
       <c r="A172" s="1" t="s">
         <v>40</v>
       </c>
@@ -4889,7 +4892,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="173" spans="1:8" ht="99">
+    <row r="173" spans="1:8" ht="93.6">
       <c r="A173" s="1" t="s">
         <v>27</v>
       </c>
@@ -4915,7 +4918,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="174" spans="1:8" ht="115.5">
+    <row r="174" spans="1:8" ht="109.2">
       <c r="A174" s="1" t="s">
         <v>28</v>
       </c>
@@ -4941,7 +4944,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="175" spans="1:8" ht="66">
+    <row r="175" spans="1:8" ht="62.4">
       <c r="A175" s="1" t="s">
         <v>13</v>
       </c>
@@ -4967,21 +4970,21 @@
         <v>26</v>
       </c>
     </row>
-    <row r="177" spans="1:8" ht="16.5">
+    <row r="177" spans="1:8" ht="15.6">
       <c r="A177" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B177" s="13" t="s">
+      <c r="B177" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="C177" s="14"/>
-      <c r="D177" s="14"/>
-      <c r="E177" s="14"/>
-      <c r="F177" s="14"/>
-      <c r="G177" s="14"/>
-      <c r="H177" s="15"/>
-    </row>
-    <row r="178" spans="1:8" ht="16.5">
+      <c r="C177" s="15"/>
+      <c r="D177" s="15"/>
+      <c r="E177" s="15"/>
+      <c r="F177" s="15"/>
+      <c r="G177" s="15"/>
+      <c r="H177" s="16"/>
+    </row>
+    <row r="178" spans="1:8" ht="15.6">
       <c r="A178" s="1"/>
       <c r="B178" s="8" t="s">
         <v>147</v>
@@ -5005,7 +5008,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="179" spans="1:8" ht="18">
+    <row r="179" spans="1:8" ht="17.399999999999999">
       <c r="A179" s="2"/>
       <c r="B179" s="11">
         <v>46046</v>
@@ -5035,7 +5038,7 @@
         <v>46052</v>
       </c>
     </row>
-    <row r="180" spans="1:8" ht="33">
+    <row r="180" spans="1:8" ht="31.2">
       <c r="A180" s="1" t="s">
         <v>3</v>
       </c>
@@ -5061,7 +5064,7 @@
         <v>0.22916666666666666</v>
       </c>
     </row>
-    <row r="181" spans="1:8" ht="16.5">
+    <row r="181" spans="1:8" ht="15.6">
       <c r="A181" s="1" t="s">
         <v>4</v>
       </c>
@@ -5087,7 +5090,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="182" spans="1:8" ht="16.5">
+    <row r="182" spans="1:8" ht="15.6">
       <c r="A182" s="1" t="s">
         <v>5</v>
       </c>
@@ -5111,7 +5114,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="183" spans="1:8" ht="16.5">
+    <row r="183" spans="1:8" ht="15.6">
       <c r="A183" s="1" t="s">
         <v>6</v>
       </c>
@@ -5135,7 +5138,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="184" spans="1:8" ht="49.5">
+    <row r="184" spans="1:8" ht="31.2">
       <c r="A184" s="1" t="s">
         <v>7</v>
       </c>
@@ -5159,7 +5162,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="185" spans="1:8" ht="16.5">
+    <row r="185" spans="1:8" ht="15.6">
       <c r="A185" s="1" t="s">
         <v>8</v>
       </c>
@@ -5181,7 +5184,7 @@
       <c r="G185" s="1"/>
       <c r="H185" s="1"/>
     </row>
-    <row r="186" spans="1:8" ht="33">
+    <row r="186" spans="1:8" ht="31.2">
       <c r="A186" s="1" t="s">
         <v>9</v>
       </c>
@@ -5203,7 +5206,7 @@
       <c r="G186" s="1"/>
       <c r="H186" s="1"/>
     </row>
-    <row r="187" spans="1:8" ht="33">
+    <row r="187" spans="1:8" ht="31.2">
       <c r="A187" s="1" t="s">
         <v>10</v>
       </c>
@@ -5225,7 +5228,7 @@
       <c r="G187" s="1"/>
       <c r="H187" s="6"/>
     </row>
-    <row r="188" spans="1:8" ht="82.5">
+    <row r="188" spans="1:8" ht="62.4">
       <c r="A188" s="1" t="s">
         <v>11</v>
       </c>
@@ -5251,7 +5254,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="189" spans="1:8" ht="66">
+    <row r="189" spans="1:8" ht="62.4">
       <c r="A189" s="1" t="s">
         <v>12</v>
       </c>
@@ -5273,7 +5276,7 @@
       <c r="G189" s="1"/>
       <c r="H189" s="1"/>
     </row>
-    <row r="190" spans="1:8" ht="49.5">
+    <row r="190" spans="1:8" ht="46.8">
       <c r="A190" s="1" t="s">
         <v>40</v>
       </c>
@@ -5295,7 +5298,7 @@
       <c r="G190" s="1"/>
       <c r="H190" s="1"/>
     </row>
-    <row r="191" spans="1:8" ht="99">
+    <row r="191" spans="1:8" ht="93.6">
       <c r="A191" s="1" t="s">
         <v>27</v>
       </c>
@@ -5317,7 +5320,7 @@
       <c r="G191" s="1"/>
       <c r="H191" s="1"/>
     </row>
-    <row r="192" spans="1:8" ht="115.5">
+    <row r="192" spans="1:8" ht="109.2">
       <c r="A192" s="1" t="s">
         <v>28</v>
       </c>
@@ -5339,7 +5342,7 @@
       <c r="G192" s="1"/>
       <c r="H192" s="1"/>
     </row>
-    <row r="193" spans="1:8" ht="66">
+    <row r="193" spans="1:8" ht="62.4">
       <c r="A193" s="1" t="s">
         <v>13</v>
       </c>
@@ -5365,21 +5368,21 @@
         <v>26</v>
       </c>
     </row>
-    <row r="196" spans="1:8" ht="16.5">
+    <row r="196" spans="1:8" ht="15.6">
       <c r="A196" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B196" s="13" t="s">
+      <c r="B196" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="C196" s="14"/>
-      <c r="D196" s="14"/>
-      <c r="E196" s="14"/>
-      <c r="F196" s="14"/>
-      <c r="G196" s="14"/>
-      <c r="H196" s="15"/>
-    </row>
-    <row r="197" spans="1:8" ht="16.5">
+      <c r="C196" s="15"/>
+      <c r="D196" s="15"/>
+      <c r="E196" s="15"/>
+      <c r="F196" s="15"/>
+      <c r="G196" s="15"/>
+      <c r="H196" s="16"/>
+    </row>
+    <row r="197" spans="1:8" ht="15.6">
       <c r="A197" s="1"/>
       <c r="B197" s="8" t="s">
         <v>147</v>
@@ -5403,7 +5406,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="198" spans="1:8" ht="18">
+    <row r="198" spans="1:8" ht="17.399999999999999">
       <c r="A198" s="2"/>
       <c r="B198" s="11">
         <v>46053</v>
@@ -5433,7 +5436,7 @@
         <v>46059</v>
       </c>
     </row>
-    <row r="199" spans="1:8" ht="33">
+    <row r="199" spans="1:8" ht="31.2">
       <c r="A199" s="1" t="s">
         <v>3</v>
       </c>
@@ -5459,7 +5462,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="200" spans="1:8" ht="16.5">
+    <row r="200" spans="1:8" ht="15.6">
       <c r="A200" s="1" t="s">
         <v>4</v>
       </c>
@@ -5481,11 +5484,11 @@
       <c r="G200" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="H200" s="20">
+      <c r="H200" s="13">
         <v>0.39583333333333331</v>
       </c>
     </row>
-    <row r="201" spans="1:8" ht="16.5">
+    <row r="201" spans="1:8" ht="15.6">
       <c r="A201" s="1" t="s">
         <v>5</v>
       </c>
@@ -5507,11 +5510,11 @@
       <c r="G201" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="H201" s="20">
+      <c r="H201" s="13">
         <v>0.91666666666666663</v>
       </c>
     </row>
-    <row r="202" spans="1:8" ht="16.5">
+    <row r="202" spans="1:8" ht="15.6">
       <c r="A202" s="1" t="s">
         <v>6</v>
       </c>
@@ -5533,11 +5536,11 @@
       <c r="G202" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="H202" s="20">
+      <c r="H202" s="13">
         <v>0.91666666666666663</v>
       </c>
     </row>
-    <row r="203" spans="1:8" ht="49.5">
+    <row r="203" spans="1:8" ht="31.2">
       <c r="A203" s="1" t="s">
         <v>7</v>
       </c>
@@ -5563,7 +5566,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="204" spans="1:8" ht="16.5">
+    <row r="204" spans="1:8" ht="15.6">
       <c r="A204" s="1" t="s">
         <v>8</v>
       </c>
@@ -5589,7 +5592,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="205" spans="1:8" ht="33">
+    <row r="205" spans="1:8" ht="31.2">
       <c r="A205" s="1" t="s">
         <v>9</v>
       </c>
@@ -5615,7 +5618,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="206" spans="1:8" ht="33">
+    <row r="206" spans="1:8" ht="31.2">
       <c r="A206" s="1" t="s">
         <v>10</v>
       </c>
@@ -5641,7 +5644,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="207" spans="1:8" ht="82.5">
+    <row r="207" spans="1:8" ht="62.4">
       <c r="A207" s="1" t="s">
         <v>11</v>
       </c>
@@ -5667,7 +5670,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="208" spans="1:8" ht="66">
+    <row r="208" spans="1:8" ht="62.4">
       <c r="A208" s="1" t="s">
         <v>12</v>
       </c>
@@ -5693,7 +5696,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="209" spans="1:8" ht="49.5">
+    <row r="209" spans="1:8" ht="46.8">
       <c r="A209" s="1" t="s">
         <v>40</v>
       </c>
@@ -5719,7 +5722,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="210" spans="1:8" ht="99">
+    <row r="210" spans="1:8" ht="93.6">
       <c r="A210" s="1" t="s">
         <v>27</v>
       </c>
@@ -5745,7 +5748,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="211" spans="1:8" ht="115.5">
+    <row r="211" spans="1:8" ht="109.2">
       <c r="A211" s="1" t="s">
         <v>28</v>
       </c>
@@ -5771,7 +5774,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="212" spans="1:8" ht="66">
+    <row r="212" spans="1:8" ht="62.4">
       <c r="A212" s="1" t="s">
         <v>13</v>
       </c>
@@ -5797,8 +5800,271 @@
         <v>26</v>
       </c>
     </row>
+    <row r="215" spans="1:8" ht="15.6">
+      <c r="A215" s="1"/>
+      <c r="B215" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="C215" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="D215" s="9" t="s">
+        <v>149</v>
+      </c>
+      <c r="E215" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="F215" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="G215" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="H215" s="10" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="216" spans="1:8" ht="17.399999999999999">
+      <c r="A216" s="2"/>
+      <c r="B216" s="11">
+        <v>46111</v>
+      </c>
+      <c r="C216" s="11">
+        <f>B216+1</f>
+        <v>46112</v>
+      </c>
+      <c r="D216" s="11">
+        <f t="shared" ref="D216" si="16">C216+1</f>
+        <v>46113</v>
+      </c>
+      <c r="E216" s="11">
+        <f t="shared" ref="E216" si="17">D216+1</f>
+        <v>46114</v>
+      </c>
+      <c r="F216" s="11">
+        <f t="shared" ref="F216" si="18">E216+1</f>
+        <v>46115</v>
+      </c>
+      <c r="G216" s="11">
+        <f t="shared" ref="G216" si="19">F216+1</f>
+        <v>46116</v>
+      </c>
+      <c r="H216" s="11">
+        <f t="shared" ref="H216" si="20">G216+1</f>
+        <v>46117</v>
+      </c>
+    </row>
+    <row r="217" spans="1:8" ht="31.2">
+      <c r="A217" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B217" s="12"/>
+      <c r="C217" s="6"/>
+      <c r="D217" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="E217" s="6"/>
+      <c r="F217" s="6"/>
+      <c r="G217" s="6"/>
+      <c r="H217" s="6"/>
+    </row>
+    <row r="218" spans="1:8" ht="15.6">
+      <c r="A218" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B218" s="6"/>
+      <c r="C218" s="6"/>
+      <c r="D218" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="E218" s="6"/>
+      <c r="F218" s="6"/>
+      <c r="G218" s="6"/>
+      <c r="H218" s="13"/>
+    </row>
+    <row r="219" spans="1:8" ht="15.6">
+      <c r="A219" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B219" s="6"/>
+      <c r="C219" s="6"/>
+      <c r="D219" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="E219" s="7"/>
+      <c r="F219" s="6"/>
+      <c r="G219" s="6"/>
+      <c r="H219" s="13"/>
+    </row>
+    <row r="220" spans="1:8" ht="15.6">
+      <c r="A220" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B220" s="6"/>
+      <c r="C220" s="6"/>
+      <c r="D220" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="E220" s="7"/>
+      <c r="F220" s="6"/>
+      <c r="G220" s="6"/>
+      <c r="H220" s="13"/>
+    </row>
+    <row r="221" spans="1:8" ht="31.2">
+      <c r="A221" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B221" s="6"/>
+      <c r="C221" s="1"/>
+      <c r="D221" s="7">
+        <v>0</v>
+      </c>
+      <c r="E221" s="1"/>
+      <c r="F221" s="1"/>
+      <c r="G221" s="1"/>
+      <c r="H221" s="1"/>
+    </row>
+    <row r="222" spans="1:8" ht="15.6">
+      <c r="A222" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B222" s="1"/>
+      <c r="C222" s="1"/>
+      <c r="D222" s="1">
+        <v>1</v>
+      </c>
+      <c r="E222" s="1"/>
+      <c r="F222" s="1"/>
+      <c r="G222" s="1"/>
+      <c r="H222" s="1"/>
+    </row>
+    <row r="223" spans="1:8" ht="31.2">
+      <c r="A223" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B223" s="1"/>
+      <c r="C223" s="1"/>
+      <c r="D223" s="1">
+        <v>80</v>
+      </c>
+      <c r="E223" s="1"/>
+      <c r="F223" s="1"/>
+      <c r="G223" s="1"/>
+      <c r="H223" s="1"/>
+    </row>
+    <row r="224" spans="1:8" ht="31.2">
+      <c r="A224" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B224" s="1"/>
+      <c r="C224" s="1"/>
+      <c r="D224" s="1">
+        <v>480</v>
+      </c>
+      <c r="E224" s="1"/>
+      <c r="F224" s="1"/>
+      <c r="G224" s="1"/>
+      <c r="H224" s="6"/>
+    </row>
+    <row r="225" spans="1:8" ht="62.4">
+      <c r="A225" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B225" s="1"/>
+      <c r="C225" s="1"/>
+      <c r="D225" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E225" s="1"/>
+      <c r="F225" s="1"/>
+      <c r="G225" s="1"/>
+      <c r="H225" s="1"/>
+    </row>
+    <row r="226" spans="1:8" ht="62.4">
+      <c r="A226" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B226" s="1"/>
+      <c r="C226" s="1"/>
+      <c r="D226" s="1">
+        <v>30</v>
+      </c>
+      <c r="E226" s="1"/>
+      <c r="F226" s="1"/>
+      <c r="G226" s="1"/>
+      <c r="H226" s="1"/>
+    </row>
+    <row r="227" spans="1:8" ht="46.8">
+      <c r="A227" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B227" s="1"/>
+      <c r="C227" s="1"/>
+      <c r="D227" s="1">
+        <v>3</v>
+      </c>
+      <c r="E227" s="1"/>
+      <c r="F227" s="1"/>
+      <c r="G227" s="1"/>
+      <c r="H227" s="1"/>
+    </row>
+    <row r="228" spans="1:8" ht="93.6">
+      <c r="A228" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B228" s="1"/>
+      <c r="C228" s="1"/>
+      <c r="D228" s="1">
+        <v>2</v>
+      </c>
+      <c r="E228" s="1"/>
+      <c r="F228" s="1"/>
+      <c r="G228" s="1"/>
+      <c r="H228" s="1"/>
+    </row>
+    <row r="229" spans="1:8" ht="109.2">
+      <c r="A229" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B229" s="1"/>
+      <c r="C229" s="1"/>
+      <c r="D229" s="1">
+        <v>4</v>
+      </c>
+      <c r="E229" s="1"/>
+      <c r="F229" s="1"/>
+      <c r="G229" s="1"/>
+      <c r="H229" s="1"/>
+    </row>
+    <row r="230" spans="1:8" ht="62.4">
+      <c r="A230" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B230" s="1"/>
+      <c r="C230" s="1"/>
+      <c r="D230" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E230" s="1"/>
+      <c r="F230" s="1"/>
+      <c r="G230" s="1"/>
+      <c r="H230" s="1"/>
+    </row>
+    <row r="231" spans="1:8">
+      <c r="D231" t="s">
+        <v>174</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="B159:H159"/>
+    <mergeCell ref="A59:H59"/>
+    <mergeCell ref="B102:H102"/>
+    <mergeCell ref="A138:H138"/>
+    <mergeCell ref="B139:H139"/>
+    <mergeCell ref="A101:H101"/>
+    <mergeCell ref="A79:H79"/>
+    <mergeCell ref="B80:H80"/>
     <mergeCell ref="B196:H196"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A60:H60"/>
@@ -5815,14 +6081,6 @@
     <mergeCell ref="B61:H61"/>
     <mergeCell ref="A119:H119"/>
     <mergeCell ref="B120:H120"/>
-    <mergeCell ref="B159:H159"/>
-    <mergeCell ref="A59:H59"/>
-    <mergeCell ref="B102:H102"/>
-    <mergeCell ref="A138:H138"/>
-    <mergeCell ref="B139:H139"/>
-    <mergeCell ref="A101:H101"/>
-    <mergeCell ref="A79:H79"/>
-    <mergeCell ref="B80:H80"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>

</xml_diff>

<commit_message>
vault backup: 2026-04-05 10:55:41
</commit_message>
<xml_diff>
--- a/睡眠日记_Sleep_Diary1.xlsx
+++ b/睡眠日记_Sleep_Diary1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My_like\My_like\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7C51281-174B-4EA0-96B4-E26F95FB0C9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CAA169B-9B34-47A3-BD74-8EC7D14C25E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="睡眠日记 Sleep Diary" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="688" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="701" uniqueCount="178">
   <si>
     <t>睡眠日记 Sleep Diary</t>
   </si>
@@ -617,6 +617,15 @@
   </si>
   <si>
     <t>4点被猫吵醒</t>
+  </si>
+  <si>
+    <t>0：00</t>
+  </si>
+  <si>
+    <t>4：00</t>
+  </si>
+  <si>
+    <t>睡前没有关灯</t>
   </si>
 </sst>
 </file>
@@ -1118,12 +1127,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H231"/>
-  <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="8" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="23.4">
+    <row r="1" spans="1:8" ht="22.5">
       <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
@@ -1135,7 +1144,7 @@
       <c r="G1" s="18"/>
       <c r="H1" s="19"/>
     </row>
-    <row r="2" spans="1:8" ht="17.399999999999999">
+    <row r="2" spans="1:8" ht="17.25">
       <c r="A2" s="20" t="s">
         <v>1</v>
       </c>
@@ -1147,7 +1156,7 @@
       <c r="G2" s="18"/>
       <c r="H2" s="19"/>
     </row>
-    <row r="3" spans="1:8" ht="15.6">
+    <row r="3" spans="1:8" ht="16.5">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -1161,7 +1170,7 @@
       <c r="G3" s="15"/>
       <c r="H3" s="16"/>
     </row>
-    <row r="4" spans="1:8" ht="34.799999999999997">
+    <row r="4" spans="1:8" ht="54">
       <c r="A4" s="2"/>
       <c r="B4" s="2" t="s">
         <v>20</v>
@@ -1185,7 +1194,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="31.2">
+    <row r="5" spans="1:8" ht="33">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -1211,7 +1220,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="15.6">
+    <row r="6" spans="1:8" ht="16.5">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
@@ -1237,7 +1246,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="15.6">
+    <row r="7" spans="1:8" ht="16.5">
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
@@ -1263,7 +1272,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="15.6">
+    <row r="8" spans="1:8" ht="16.5">
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
@@ -1289,7 +1298,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="31.2">
+    <row r="9" spans="1:8" ht="49.5">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
@@ -1315,7 +1324,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="15.6">
+    <row r="10" spans="1:8" ht="16.5">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
@@ -1341,7 +1350,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="31.2">
+    <row r="11" spans="1:8" ht="33">
       <c r="A11" s="1" t="s">
         <v>9</v>
       </c>
@@ -1367,7 +1376,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="31.2">
+    <row r="12" spans="1:8" ht="33">
       <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
@@ -1393,7 +1402,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="62.4">
+    <row r="13" spans="1:8" ht="82.5">
       <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
@@ -1419,7 +1428,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="62.4">
+    <row r="14" spans="1:8" ht="66">
       <c r="A14" s="1" t="s">
         <v>12</v>
       </c>
@@ -1445,7 +1454,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="46.8">
+    <row r="15" spans="1:8" ht="49.5">
       <c r="A15" s="1" t="s">
         <v>40</v>
       </c>
@@ -1471,7 +1480,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="93.6">
+    <row r="16" spans="1:8" ht="99">
       <c r="A16" s="1" t="s">
         <v>27</v>
       </c>
@@ -1497,7 +1506,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="109.2">
+    <row r="17" spans="1:8" ht="115.5">
       <c r="A17" s="1" t="s">
         <v>28</v>
       </c>
@@ -1523,7 +1532,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="62.4">
+    <row r="18" spans="1:8" ht="66">
       <c r="A18" s="1" t="s">
         <v>13</v>
       </c>
@@ -1552,7 +1561,7 @@
     <row r="20" spans="1:8">
       <c r="A20" s="3"/>
     </row>
-    <row r="21" spans="1:8" ht="23.4">
+    <row r="21" spans="1:8" ht="22.5">
       <c r="A21" s="17" t="s">
         <v>0</v>
       </c>
@@ -1564,7 +1573,7 @@
       <c r="G21" s="18"/>
       <c r="H21" s="19"/>
     </row>
-    <row r="22" spans="1:8" ht="17.399999999999999">
+    <row r="22" spans="1:8" ht="17.25">
       <c r="A22" s="20" t="s">
         <v>1</v>
       </c>
@@ -1576,7 +1585,7 @@
       <c r="G22" s="18"/>
       <c r="H22" s="19"/>
     </row>
-    <row r="23" spans="1:8" ht="15.6">
+    <row r="23" spans="1:8" ht="16.5">
       <c r="A23" s="1" t="s">
         <v>2</v>
       </c>
@@ -1590,7 +1599,7 @@
       <c r="G23" s="15"/>
       <c r="H23" s="16"/>
     </row>
-    <row r="24" spans="1:8" ht="34.799999999999997">
+    <row r="24" spans="1:8" ht="54">
       <c r="A24" s="2"/>
       <c r="B24" s="2" t="s">
         <v>45</v>
@@ -1614,7 +1623,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="31.2">
+    <row r="25" spans="1:8" ht="33">
       <c r="A25" s="1" t="s">
         <v>3</v>
       </c>
@@ -1640,7 +1649,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="15.6">
+    <row r="26" spans="1:8" ht="16.5">
       <c r="A26" s="1" t="s">
         <v>4</v>
       </c>
@@ -1666,7 +1675,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="15.6">
+    <row r="27" spans="1:8" ht="16.5">
       <c r="A27" s="1" t="s">
         <v>5</v>
       </c>
@@ -1692,7 +1701,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="15.6">
+    <row r="28" spans="1:8" ht="16.5">
       <c r="A28" s="1" t="s">
         <v>6</v>
       </c>
@@ -1718,7 +1727,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="31.2">
+    <row r="29" spans="1:8" ht="49.5">
       <c r="A29" s="1" t="s">
         <v>7</v>
       </c>
@@ -1744,7 +1753,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="15.6">
+    <row r="30" spans="1:8" ht="16.5">
       <c r="A30" s="1" t="s">
         <v>8</v>
       </c>
@@ -1770,7 +1779,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="31.2">
+    <row r="31" spans="1:8" ht="33">
       <c r="A31" s="1" t="s">
         <v>9</v>
       </c>
@@ -1796,7 +1805,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="31.2">
+    <row r="32" spans="1:8" ht="33">
       <c r="A32" s="1" t="s">
         <v>10</v>
       </c>
@@ -1822,7 +1831,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="62.4">
+    <row r="33" spans="1:8" ht="82.5">
       <c r="A33" s="1" t="s">
         <v>11</v>
       </c>
@@ -1848,7 +1857,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="62.4">
+    <row r="34" spans="1:8" ht="66">
       <c r="A34" s="1" t="s">
         <v>12</v>
       </c>
@@ -1874,7 +1883,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="46.8">
+    <row r="35" spans="1:8" ht="49.5">
       <c r="A35" s="1" t="s">
         <v>40</v>
       </c>
@@ -1900,7 +1909,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="93.6">
+    <row r="36" spans="1:8" ht="99">
       <c r="A36" s="1" t="s">
         <v>27</v>
       </c>
@@ -1926,7 +1935,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="109.2">
+    <row r="37" spans="1:8" ht="115.5">
       <c r="A37" s="1" t="s">
         <v>28</v>
       </c>
@@ -1952,7 +1961,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="62.4">
+    <row r="38" spans="1:8" ht="66">
       <c r="A38" s="1" t="s">
         <v>13</v>
       </c>
@@ -1978,7 +1987,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="23.4">
+    <row r="40" spans="1:8" ht="22.5">
       <c r="A40" s="17" t="s">
         <v>0</v>
       </c>
@@ -1990,7 +1999,7 @@
       <c r="G40" s="18"/>
       <c r="H40" s="19"/>
     </row>
-    <row r="41" spans="1:8" ht="17.399999999999999">
+    <row r="41" spans="1:8" ht="17.25">
       <c r="A41" s="20" t="s">
         <v>1</v>
       </c>
@@ -2002,7 +2011,7 @@
       <c r="G41" s="18"/>
       <c r="H41" s="19"/>
     </row>
-    <row r="42" spans="1:8" ht="15.6">
+    <row r="42" spans="1:8" ht="16.5">
       <c r="A42" s="1" t="s">
         <v>2</v>
       </c>
@@ -2016,7 +2025,7 @@
       <c r="G42" s="15"/>
       <c r="H42" s="16"/>
     </row>
-    <row r="43" spans="1:8" ht="34.799999999999997">
+    <row r="43" spans="1:8" ht="54">
       <c r="A43" s="2"/>
       <c r="B43" s="2" t="s">
         <v>53</v>
@@ -2040,7 +2049,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="44" spans="1:8" ht="31.2">
+    <row r="44" spans="1:8" ht="33">
       <c r="A44" s="1" t="s">
         <v>3</v>
       </c>
@@ -2066,7 +2075,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="45" spans="1:8" ht="15.6">
+    <row r="45" spans="1:8" ht="16.5">
       <c r="A45" s="1" t="s">
         <v>4</v>
       </c>
@@ -2092,7 +2101,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="46" spans="1:8" ht="15.6">
+    <row r="46" spans="1:8" ht="16.5">
       <c r="A46" s="1" t="s">
         <v>5</v>
       </c>
@@ -2118,7 +2127,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="47" spans="1:8" ht="15.6">
+    <row r="47" spans="1:8" ht="16.5">
       <c r="A47" s="1" t="s">
         <v>6</v>
       </c>
@@ -2144,7 +2153,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="48" spans="1:8" ht="31.2">
+    <row r="48" spans="1:8" ht="49.5">
       <c r="A48" s="1" t="s">
         <v>7</v>
       </c>
@@ -2170,7 +2179,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="49" spans="1:8" ht="15.6">
+    <row r="49" spans="1:8" ht="16.5">
       <c r="A49" s="1" t="s">
         <v>8</v>
       </c>
@@ -2196,7 +2205,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:8" ht="31.2">
+    <row r="50" spans="1:8" ht="33">
       <c r="A50" s="1" t="s">
         <v>9</v>
       </c>
@@ -2222,7 +2231,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="51" spans="1:8" ht="31.2">
+    <row r="51" spans="1:8" ht="33">
       <c r="A51" s="1" t="s">
         <v>10</v>
       </c>
@@ -2248,7 +2257,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="52" spans="1:8" ht="62.4">
+    <row r="52" spans="1:8" ht="82.5">
       <c r="A52" s="1" t="s">
         <v>11</v>
       </c>
@@ -2274,7 +2283,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="53" spans="1:8" ht="62.4">
+    <row r="53" spans="1:8" ht="66">
       <c r="A53" s="1" t="s">
         <v>12</v>
       </c>
@@ -2300,7 +2309,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="54" spans="1:8" ht="46.8">
+    <row r="54" spans="1:8" ht="49.5">
       <c r="A54" s="1" t="s">
         <v>40</v>
       </c>
@@ -2326,7 +2335,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="55" spans="1:8" ht="93.6">
+    <row r="55" spans="1:8" ht="99">
       <c r="A55" s="1" t="s">
         <v>27</v>
       </c>
@@ -2352,7 +2361,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="56" spans="1:8" ht="109.2">
+    <row r="56" spans="1:8" ht="115.5">
       <c r="A56" s="1" t="s">
         <v>28</v>
       </c>
@@ -2378,7 +2387,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="57" spans="1:8" ht="62.4">
+    <row r="57" spans="1:8" ht="66">
       <c r="A57" s="1" t="s">
         <v>13</v>
       </c>
@@ -2404,7 +2413,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="59" spans="1:8" ht="23.4">
+    <row r="59" spans="1:8" ht="22.5">
       <c r="A59" s="17" t="s">
         <v>0</v>
       </c>
@@ -2416,7 +2425,7 @@
       <c r="G59" s="18"/>
       <c r="H59" s="19"/>
     </row>
-    <row r="60" spans="1:8" ht="17.399999999999999">
+    <row r="60" spans="1:8" ht="17.25">
       <c r="A60" s="20" t="s">
         <v>1</v>
       </c>
@@ -2428,7 +2437,7 @@
       <c r="G60" s="18"/>
       <c r="H60" s="19"/>
     </row>
-    <row r="61" spans="1:8" ht="15.6">
+    <row r="61" spans="1:8" ht="16.5">
       <c r="A61" s="1" t="s">
         <v>2</v>
       </c>
@@ -2442,7 +2451,7 @@
       <c r="G61" s="15"/>
       <c r="H61" s="16"/>
     </row>
-    <row r="62" spans="1:8" ht="34.799999999999997">
+    <row r="62" spans="1:8" ht="54">
       <c r="A62" s="2"/>
       <c r="B62" s="2" t="s">
         <v>83</v>
@@ -2466,7 +2475,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="63" spans="1:8" ht="31.2">
+    <row r="63" spans="1:8" ht="33">
       <c r="A63" s="1" t="s">
         <v>3</v>
       </c>
@@ -2492,7 +2501,7 @@
         <v>0.28611111111111109</v>
       </c>
     </row>
-    <row r="64" spans="1:8" ht="15.6">
+    <row r="64" spans="1:8" ht="16.5">
       <c r="A64" s="1" t="s">
         <v>4</v>
       </c>
@@ -2518,7 +2527,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="65" spans="1:8" ht="15.6">
+    <row r="65" spans="1:8" ht="16.5">
       <c r="A65" s="1" t="s">
         <v>5</v>
       </c>
@@ -2544,7 +2553,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="66" spans="1:8" ht="15.6">
+    <row r="66" spans="1:8" ht="16.5">
       <c r="A66" s="1" t="s">
         <v>6</v>
       </c>
@@ -2570,7 +2579,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="67" spans="1:8" ht="31.2">
+    <row r="67" spans="1:8" ht="49.5">
       <c r="A67" s="1" t="s">
         <v>7</v>
       </c>
@@ -2596,7 +2605,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="68" spans="1:8" ht="15.6">
+    <row r="68" spans="1:8" ht="16.5">
       <c r="A68" s="1" t="s">
         <v>8</v>
       </c>
@@ -2622,7 +2631,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:8" ht="31.2">
+    <row r="69" spans="1:8" ht="33">
       <c r="A69" s="1" t="s">
         <v>9</v>
       </c>
@@ -2648,7 +2657,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="70" spans="1:8" ht="31.2">
+    <row r="70" spans="1:8" ht="33">
       <c r="A70" s="1" t="s">
         <v>10</v>
       </c>
@@ -2674,7 +2683,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="71" spans="1:8" ht="62.4">
+    <row r="71" spans="1:8" ht="82.5">
       <c r="A71" s="1" t="s">
         <v>11</v>
       </c>
@@ -2700,7 +2709,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="72" spans="1:8" ht="62.4">
+    <row r="72" spans="1:8" ht="66">
       <c r="A72" s="1" t="s">
         <v>12</v>
       </c>
@@ -2726,7 +2735,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="73" spans="1:8" ht="46.8">
+    <row r="73" spans="1:8" ht="49.5">
       <c r="A73" s="1" t="s">
         <v>40</v>
       </c>
@@ -2752,7 +2761,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="74" spans="1:8" ht="93.6">
+    <row r="74" spans="1:8" ht="99">
       <c r="A74" s="1" t="s">
         <v>27</v>
       </c>
@@ -2778,7 +2787,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="75" spans="1:8" ht="109.2">
+    <row r="75" spans="1:8" ht="115.5">
       <c r="A75" s="1" t="s">
         <v>28</v>
       </c>
@@ -2804,7 +2813,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="76" spans="1:8" ht="62.4">
+    <row r="76" spans="1:8" ht="66">
       <c r="A76" s="1" t="s">
         <v>13</v>
       </c>
@@ -2830,7 +2839,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="79" spans="1:8" ht="17.399999999999999">
+    <row r="79" spans="1:8" ht="17.25">
       <c r="A79" s="20" t="s">
         <v>1</v>
       </c>
@@ -2842,7 +2851,7 @@
       <c r="G79" s="18"/>
       <c r="H79" s="19"/>
     </row>
-    <row r="80" spans="1:8" ht="15.6">
+    <row r="80" spans="1:8" ht="16.5">
       <c r="A80" s="1" t="s">
         <v>2</v>
       </c>
@@ -2856,7 +2865,7 @@
       <c r="G80" s="15"/>
       <c r="H80" s="16"/>
     </row>
-    <row r="81" spans="1:8" ht="34.799999999999997">
+    <row r="81" spans="1:8" ht="54">
       <c r="A81" s="2"/>
       <c r="B81" s="2" t="s">
         <v>97</v>
@@ -2880,7 +2889,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="82" spans="1:8" ht="31.2">
+    <row r="82" spans="1:8" ht="33">
       <c r="A82" s="1" t="s">
         <v>3</v>
       </c>
@@ -2906,7 +2915,7 @@
         <v>0.30069444444444449</v>
       </c>
     </row>
-    <row r="83" spans="1:8" ht="15.6">
+    <row r="83" spans="1:8" ht="16.5">
       <c r="A83" s="1" t="s">
         <v>4</v>
       </c>
@@ -2932,7 +2941,7 @@
         <v>0.30069444444444449</v>
       </c>
     </row>
-    <row r="84" spans="1:8" ht="15.6">
+    <row r="84" spans="1:8" ht="16.5">
       <c r="A84" s="1" t="s">
         <v>5</v>
       </c>
@@ -2958,7 +2967,7 @@
         <v>0.97222222222222221</v>
       </c>
     </row>
-    <row r="85" spans="1:8" ht="15.6">
+    <row r="85" spans="1:8" ht="16.5">
       <c r="A85" s="1" t="s">
         <v>6</v>
       </c>
@@ -2984,7 +2993,7 @@
         <v>0.97222222222222221</v>
       </c>
     </row>
-    <row r="86" spans="1:8" ht="31.2">
+    <row r="86" spans="1:8" ht="49.5">
       <c r="A86" s="1" t="s">
         <v>7</v>
       </c>
@@ -3010,7 +3019,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="87" spans="1:8" ht="15.6">
+    <row r="87" spans="1:8" ht="16.5">
       <c r="A87" s="1" t="s">
         <v>8</v>
       </c>
@@ -3036,7 +3045,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:8" ht="31.2">
+    <row r="88" spans="1:8" ht="33">
       <c r="A88" s="1" t="s">
         <v>9</v>
       </c>
@@ -3062,7 +3071,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:8" ht="31.2">
+    <row r="89" spans="1:8" ht="33">
       <c r="A89" s="1" t="s">
         <v>10</v>
       </c>
@@ -3088,7 +3097,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="90" spans="1:8" ht="62.4">
+    <row r="90" spans="1:8" ht="82.5">
       <c r="A90" s="1" t="s">
         <v>11</v>
       </c>
@@ -3114,7 +3123,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="91" spans="1:8" ht="62.4">
+    <row r="91" spans="1:8" ht="66">
       <c r="A91" s="1" t="s">
         <v>12</v>
       </c>
@@ -3140,7 +3149,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="92" spans="1:8" ht="46.8">
+    <row r="92" spans="1:8" ht="49.5">
       <c r="A92" s="1" t="s">
         <v>40</v>
       </c>
@@ -3166,7 +3175,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="93" spans="1:8" ht="93.6">
+    <row r="93" spans="1:8" ht="99">
       <c r="A93" s="1" t="s">
         <v>27</v>
       </c>
@@ -3192,7 +3201,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="94" spans="1:8" ht="109.2">
+    <row r="94" spans="1:8" ht="115.5">
       <c r="A94" s="1" t="s">
         <v>28</v>
       </c>
@@ -3218,7 +3227,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="95" spans="1:8" ht="62.4">
+    <row r="95" spans="1:8" ht="66">
       <c r="A95" s="1" t="s">
         <v>13</v>
       </c>
@@ -3249,7 +3258,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="101" spans="1:8" ht="17.399999999999999">
+    <row r="101" spans="1:8" ht="17.25">
       <c r="A101" s="20" t="s">
         <v>1</v>
       </c>
@@ -3261,7 +3270,7 @@
       <c r="G101" s="18"/>
       <c r="H101" s="19"/>
     </row>
-    <row r="102" spans="1:8" ht="15.6">
+    <row r="102" spans="1:8" ht="16.5">
       <c r="A102" s="1" t="s">
         <v>2</v>
       </c>
@@ -3275,7 +3284,7 @@
       <c r="G102" s="15"/>
       <c r="H102" s="16"/>
     </row>
-    <row r="103" spans="1:8" ht="34.799999999999997">
+    <row r="103" spans="1:8" ht="54">
       <c r="A103" s="2"/>
       <c r="B103" s="2" t="s">
         <v>113</v>
@@ -3299,7 +3308,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="104" spans="1:8" ht="31.2">
+    <row r="104" spans="1:8" ht="33">
       <c r="A104" s="1" t="s">
         <v>3</v>
       </c>
@@ -3325,7 +3334,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="105" spans="1:8" ht="15.6">
+    <row r="105" spans="1:8" ht="16.5">
       <c r="A105" s="1" t="s">
         <v>4</v>
       </c>
@@ -3351,7 +3360,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="106" spans="1:8" ht="15.6">
+    <row r="106" spans="1:8" ht="16.5">
       <c r="A106" s="1" t="s">
         <v>5</v>
       </c>
@@ -3377,7 +3386,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="107" spans="1:8" ht="15.6">
+    <row r="107" spans="1:8" ht="16.5">
       <c r="A107" s="1" t="s">
         <v>6</v>
       </c>
@@ -3403,7 +3412,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="108" spans="1:8" ht="31.2">
+    <row r="108" spans="1:8" ht="49.5">
       <c r="A108" s="1" t="s">
         <v>7</v>
       </c>
@@ -3429,7 +3438,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="109" spans="1:8" ht="15.6">
+    <row r="109" spans="1:8" ht="16.5">
       <c r="A109" s="1" t="s">
         <v>8</v>
       </c>
@@ -3455,7 +3464,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:8" ht="31.2">
+    <row r="110" spans="1:8" ht="33">
       <c r="A110" s="1" t="s">
         <v>9</v>
       </c>
@@ -3481,7 +3490,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:8" ht="31.2">
+    <row r="111" spans="1:8" ht="33">
       <c r="A111" s="1" t="s">
         <v>10</v>
       </c>
@@ -3507,7 +3516,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="112" spans="1:8" ht="62.4">
+    <row r="112" spans="1:8" ht="82.5">
       <c r="A112" s="1" t="s">
         <v>11</v>
       </c>
@@ -3533,7 +3542,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="113" spans="1:8" ht="62.4">
+    <row r="113" spans="1:8" ht="66">
       <c r="A113" s="1" t="s">
         <v>12</v>
       </c>
@@ -3559,7 +3568,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="114" spans="1:8" ht="46.8">
+    <row r="114" spans="1:8" ht="49.5">
       <c r="A114" s="1" t="s">
         <v>40</v>
       </c>
@@ -3585,7 +3594,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="115" spans="1:8" ht="93.6">
+    <row r="115" spans="1:8" ht="99">
       <c r="A115" s="1" t="s">
         <v>27</v>
       </c>
@@ -3611,7 +3620,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="116" spans="1:8" ht="109.2">
+    <row r="116" spans="1:8" ht="115.5">
       <c r="A116" s="1" t="s">
         <v>28</v>
       </c>
@@ -3637,7 +3646,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="117" spans="1:8" ht="62.4">
+    <row r="117" spans="1:8" ht="66">
       <c r="A117" s="1" t="s">
         <v>13</v>
       </c>
@@ -3663,7 +3672,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="119" spans="1:8" ht="17.399999999999999">
+    <row r="119" spans="1:8" ht="17.25">
       <c r="A119" s="20" t="s">
         <v>1</v>
       </c>
@@ -3675,7 +3684,7 @@
       <c r="G119" s="18"/>
       <c r="H119" s="19"/>
     </row>
-    <row r="120" spans="1:8" ht="15.6">
+    <row r="120" spans="1:8" ht="16.5">
       <c r="A120" s="1" t="s">
         <v>2</v>
       </c>
@@ -3689,7 +3698,7 @@
       <c r="G120" s="15"/>
       <c r="H120" s="16"/>
     </row>
-    <row r="121" spans="1:8" ht="34.799999999999997">
+    <row r="121" spans="1:8" ht="36">
       <c r="A121" s="2"/>
       <c r="B121" s="2" t="s">
         <v>129</v>
@@ -3713,7 +3722,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="122" spans="1:8" ht="31.2">
+    <row r="122" spans="1:8" ht="33">
       <c r="A122" s="1" t="s">
         <v>3</v>
       </c>
@@ -3739,7 +3748,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="123" spans="1:8" ht="15.6">
+    <row r="123" spans="1:8" ht="16.5">
       <c r="A123" s="1" t="s">
         <v>4</v>
       </c>
@@ -3765,7 +3774,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="124" spans="1:8" ht="15.6">
+    <row r="124" spans="1:8" ht="16.5">
       <c r="A124" s="1" t="s">
         <v>5</v>
       </c>
@@ -3791,7 +3800,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="125" spans="1:8" ht="15.6">
+    <row r="125" spans="1:8" ht="16.5">
       <c r="A125" s="1" t="s">
         <v>6</v>
       </c>
@@ -3817,7 +3826,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="126" spans="1:8" ht="31.2">
+    <row r="126" spans="1:8" ht="49.5">
       <c r="A126" s="1" t="s">
         <v>7</v>
       </c>
@@ -3843,7 +3852,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="127" spans="1:8" ht="15.6">
+    <row r="127" spans="1:8" ht="16.5">
       <c r="A127" s="1" t="s">
         <v>8</v>
       </c>
@@ -3869,7 +3878,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:8" ht="31.2">
+    <row r="128" spans="1:8" ht="33">
       <c r="A128" s="1" t="s">
         <v>9</v>
       </c>
@@ -3895,7 +3904,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:8" ht="31.2">
+    <row r="129" spans="1:8" ht="33">
       <c r="A129" s="1" t="s">
         <v>10</v>
       </c>
@@ -3921,7 +3930,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="130" spans="1:8" ht="62.4">
+    <row r="130" spans="1:8" ht="82.5">
       <c r="A130" s="1" t="s">
         <v>11</v>
       </c>
@@ -3947,7 +3956,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="131" spans="1:8" ht="62.4">
+    <row r="131" spans="1:8" ht="66">
       <c r="A131" s="1" t="s">
         <v>12</v>
       </c>
@@ -3973,7 +3982,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="132" spans="1:8" ht="46.8">
+    <row r="132" spans="1:8" ht="49.5">
       <c r="A132" s="1" t="s">
         <v>40</v>
       </c>
@@ -3999,7 +4008,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="133" spans="1:8" ht="93.6">
+    <row r="133" spans="1:8" ht="99">
       <c r="A133" s="1" t="s">
         <v>27</v>
       </c>
@@ -4025,7 +4034,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="134" spans="1:8" ht="109.2">
+    <row r="134" spans="1:8" ht="115.5">
       <c r="A134" s="1" t="s">
         <v>28</v>
       </c>
@@ -4051,7 +4060,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="135" spans="1:8" ht="62.4">
+    <row r="135" spans="1:8" ht="66">
       <c r="A135" s="1" t="s">
         <v>13</v>
       </c>
@@ -4077,7 +4086,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="138" spans="1:8" ht="17.399999999999999">
+    <row r="138" spans="1:8" ht="17.25">
       <c r="A138" s="20" t="s">
         <v>1</v>
       </c>
@@ -4089,7 +4098,7 @@
       <c r="G138" s="18"/>
       <c r="H138" s="19"/>
     </row>
-    <row r="139" spans="1:8" ht="15.6">
+    <row r="139" spans="1:8" ht="16.5">
       <c r="A139" s="1" t="s">
         <v>2</v>
       </c>
@@ -4103,7 +4112,7 @@
       <c r="G139" s="15"/>
       <c r="H139" s="16"/>
     </row>
-    <row r="140" spans="1:8" ht="15.6">
+    <row r="140" spans="1:8" ht="16.5">
       <c r="A140" s="1"/>
       <c r="B140" s="8" t="s">
         <v>147</v>
@@ -4127,7 +4136,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="141" spans="1:8" ht="17.399999999999999">
+    <row r="141" spans="1:8" ht="18">
       <c r="A141" s="2"/>
       <c r="B141" s="11">
         <v>46032</v>
@@ -4157,7 +4166,7 @@
         <v>46038</v>
       </c>
     </row>
-    <row r="142" spans="1:8" ht="31.2">
+    <row r="142" spans="1:8" ht="33">
       <c r="A142" s="1" t="s">
         <v>3</v>
       </c>
@@ -4183,7 +4192,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="143" spans="1:8" ht="15.6">
+    <row r="143" spans="1:8" ht="16.5">
       <c r="A143" s="1" t="s">
         <v>4</v>
       </c>
@@ -4209,7 +4218,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="144" spans="1:8" ht="15.6">
+    <row r="144" spans="1:8" ht="16.5">
       <c r="A144" s="1" t="s">
         <v>5</v>
       </c>
@@ -4235,7 +4244,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="145" spans="1:8" ht="15.6">
+    <row r="145" spans="1:8" ht="16.5">
       <c r="A145" s="1" t="s">
         <v>6</v>
       </c>
@@ -4261,7 +4270,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="146" spans="1:8" ht="31.2">
+    <row r="146" spans="1:8" ht="49.5">
       <c r="A146" s="1" t="s">
         <v>7</v>
       </c>
@@ -4287,7 +4296,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="147" spans="1:8" ht="15.6">
+    <row r="147" spans="1:8" ht="16.5">
       <c r="A147" s="1" t="s">
         <v>8</v>
       </c>
@@ -4313,7 +4322,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="148" spans="1:8" ht="31.2">
+    <row r="148" spans="1:8" ht="33">
       <c r="A148" s="1" t="s">
         <v>9</v>
       </c>
@@ -4339,7 +4348,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="149" spans="1:8" ht="31.2">
+    <row r="149" spans="1:8" ht="33">
       <c r="A149" s="1" t="s">
         <v>10</v>
       </c>
@@ -4365,7 +4374,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="150" spans="1:8" ht="62.4">
+    <row r="150" spans="1:8" ht="82.5">
       <c r="A150" s="1" t="s">
         <v>11</v>
       </c>
@@ -4391,7 +4400,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="151" spans="1:8" ht="62.4">
+    <row r="151" spans="1:8" ht="66">
       <c r="A151" s="1" t="s">
         <v>12</v>
       </c>
@@ -4417,7 +4426,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="152" spans="1:8" ht="46.8">
+    <row r="152" spans="1:8" ht="49.5">
       <c r="A152" s="1" t="s">
         <v>40</v>
       </c>
@@ -4443,7 +4452,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="153" spans="1:8" ht="93.6">
+    <row r="153" spans="1:8" ht="99">
       <c r="A153" s="1" t="s">
         <v>27</v>
       </c>
@@ -4469,7 +4478,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="154" spans="1:8" ht="109.2">
+    <row r="154" spans="1:8" ht="115.5">
       <c r="A154" s="1" t="s">
         <v>28</v>
       </c>
@@ -4495,7 +4504,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="155" spans="1:8" ht="62.4">
+    <row r="155" spans="1:8" ht="66">
       <c r="A155" s="1" t="s">
         <v>13</v>
       </c>
@@ -4526,7 +4535,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="158" spans="1:8" ht="17.399999999999999">
+    <row r="158" spans="1:8" ht="17.25">
       <c r="A158" s="20" t="s">
         <v>1</v>
       </c>
@@ -4538,7 +4547,7 @@
       <c r="G158" s="18"/>
       <c r="H158" s="19"/>
     </row>
-    <row r="159" spans="1:8" ht="15.6">
+    <row r="159" spans="1:8" ht="16.5">
       <c r="A159" s="1" t="s">
         <v>2</v>
       </c>
@@ -4552,7 +4561,7 @@
       <c r="G159" s="15"/>
       <c r="H159" s="16"/>
     </row>
-    <row r="160" spans="1:8" ht="15.6">
+    <row r="160" spans="1:8" ht="16.5">
       <c r="A160" s="1"/>
       <c r="B160" s="8" t="s">
         <v>147</v>
@@ -4576,7 +4585,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="161" spans="1:8" ht="17.399999999999999">
+    <row r="161" spans="1:8" ht="18">
       <c r="A161" s="2"/>
       <c r="B161" s="11">
         <v>46039</v>
@@ -4606,7 +4615,7 @@
         <v>46045</v>
       </c>
     </row>
-    <row r="162" spans="1:8" ht="31.2">
+    <row r="162" spans="1:8" ht="33">
       <c r="A162" s="1" t="s">
         <v>3</v>
       </c>
@@ -4632,7 +4641,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="163" spans="1:8" ht="15.6">
+    <row r="163" spans="1:8" ht="16.5">
       <c r="A163" s="1" t="s">
         <v>4</v>
       </c>
@@ -4658,7 +4667,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="164" spans="1:8" ht="15.6">
+    <row r="164" spans="1:8" ht="16.5">
       <c r="A164" s="1" t="s">
         <v>5</v>
       </c>
@@ -4684,7 +4693,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="165" spans="1:8" ht="15.6">
+    <row r="165" spans="1:8" ht="16.5">
       <c r="A165" s="1" t="s">
         <v>6</v>
       </c>
@@ -4710,7 +4719,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="166" spans="1:8" ht="31.2">
+    <row r="166" spans="1:8" ht="49.5">
       <c r="A166" s="1" t="s">
         <v>7</v>
       </c>
@@ -4736,7 +4745,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="167" spans="1:8" ht="15.6">
+    <row r="167" spans="1:8" ht="16.5">
       <c r="A167" s="1" t="s">
         <v>8</v>
       </c>
@@ -4762,7 +4771,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="168" spans="1:8" ht="31.2">
+    <row r="168" spans="1:8" ht="33">
       <c r="A168" s="1" t="s">
         <v>9</v>
       </c>
@@ -4788,7 +4797,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="169" spans="1:8" ht="31.2">
+    <row r="169" spans="1:8" ht="33">
       <c r="A169" s="1" t="s">
         <v>10</v>
       </c>
@@ -4814,7 +4823,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="170" spans="1:8" ht="62.4">
+    <row r="170" spans="1:8" ht="82.5">
       <c r="A170" s="1" t="s">
         <v>11</v>
       </c>
@@ -4840,7 +4849,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="171" spans="1:8" ht="62.4">
+    <row r="171" spans="1:8" ht="66">
       <c r="A171" s="1" t="s">
         <v>12</v>
       </c>
@@ -4866,7 +4875,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:8" ht="46.8">
+    <row r="172" spans="1:8" ht="49.5">
       <c r="A172" s="1" t="s">
         <v>40</v>
       </c>
@@ -4892,7 +4901,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="173" spans="1:8" ht="93.6">
+    <row r="173" spans="1:8" ht="99">
       <c r="A173" s="1" t="s">
         <v>27</v>
       </c>
@@ -4918,7 +4927,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="174" spans="1:8" ht="109.2">
+    <row r="174" spans="1:8" ht="115.5">
       <c r="A174" s="1" t="s">
         <v>28</v>
       </c>
@@ -4944,7 +4953,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="175" spans="1:8" ht="62.4">
+    <row r="175" spans="1:8" ht="66">
       <c r="A175" s="1" t="s">
         <v>13</v>
       </c>
@@ -4970,7 +4979,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="177" spans="1:8" ht="15.6">
+    <row r="177" spans="1:8" ht="16.5">
       <c r="A177" s="1" t="s">
         <v>2</v>
       </c>
@@ -4984,7 +4993,7 @@
       <c r="G177" s="15"/>
       <c r="H177" s="16"/>
     </row>
-    <row r="178" spans="1:8" ht="15.6">
+    <row r="178" spans="1:8" ht="16.5">
       <c r="A178" s="1"/>
       <c r="B178" s="8" t="s">
         <v>147</v>
@@ -5008,7 +5017,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="179" spans="1:8" ht="17.399999999999999">
+    <row r="179" spans="1:8" ht="18">
       <c r="A179" s="2"/>
       <c r="B179" s="11">
         <v>46046</v>
@@ -5038,7 +5047,7 @@
         <v>46052</v>
       </c>
     </row>
-    <row r="180" spans="1:8" ht="31.2">
+    <row r="180" spans="1:8" ht="33">
       <c r="A180" s="1" t="s">
         <v>3</v>
       </c>
@@ -5064,7 +5073,7 @@
         <v>0.22916666666666666</v>
       </c>
     </row>
-    <row r="181" spans="1:8" ht="15.6">
+    <row r="181" spans="1:8" ht="16.5">
       <c r="A181" s="1" t="s">
         <v>4</v>
       </c>
@@ -5090,7 +5099,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="182" spans="1:8" ht="15.6">
+    <row r="182" spans="1:8" ht="16.5">
       <c r="A182" s="1" t="s">
         <v>5</v>
       </c>
@@ -5114,7 +5123,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="183" spans="1:8" ht="15.6">
+    <row r="183" spans="1:8" ht="16.5">
       <c r="A183" s="1" t="s">
         <v>6</v>
       </c>
@@ -5138,7 +5147,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="184" spans="1:8" ht="31.2">
+    <row r="184" spans="1:8" ht="49.5">
       <c r="A184" s="1" t="s">
         <v>7</v>
       </c>
@@ -5162,7 +5171,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="185" spans="1:8" ht="15.6">
+    <row r="185" spans="1:8" ht="16.5">
       <c r="A185" s="1" t="s">
         <v>8</v>
       </c>
@@ -5184,7 +5193,7 @@
       <c r="G185" s="1"/>
       <c r="H185" s="1"/>
     </row>
-    <row r="186" spans="1:8" ht="31.2">
+    <row r="186" spans="1:8" ht="33">
       <c r="A186" s="1" t="s">
         <v>9</v>
       </c>
@@ -5206,7 +5215,7 @@
       <c r="G186" s="1"/>
       <c r="H186" s="1"/>
     </row>
-    <row r="187" spans="1:8" ht="31.2">
+    <row r="187" spans="1:8" ht="33">
       <c r="A187" s="1" t="s">
         <v>10</v>
       </c>
@@ -5228,7 +5237,7 @@
       <c r="G187" s="1"/>
       <c r="H187" s="6"/>
     </row>
-    <row r="188" spans="1:8" ht="62.4">
+    <row r="188" spans="1:8" ht="82.5">
       <c r="A188" s="1" t="s">
         <v>11</v>
       </c>
@@ -5254,7 +5263,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="189" spans="1:8" ht="62.4">
+    <row r="189" spans="1:8" ht="66">
       <c r="A189" s="1" t="s">
         <v>12</v>
       </c>
@@ -5276,7 +5285,7 @@
       <c r="G189" s="1"/>
       <c r="H189" s="1"/>
     </row>
-    <row r="190" spans="1:8" ht="46.8">
+    <row r="190" spans="1:8" ht="49.5">
       <c r="A190" s="1" t="s">
         <v>40</v>
       </c>
@@ -5298,7 +5307,7 @@
       <c r="G190" s="1"/>
       <c r="H190" s="1"/>
     </row>
-    <row r="191" spans="1:8" ht="93.6">
+    <row r="191" spans="1:8" ht="99">
       <c r="A191" s="1" t="s">
         <v>27</v>
       </c>
@@ -5320,7 +5329,7 @@
       <c r="G191" s="1"/>
       <c r="H191" s="1"/>
     </row>
-    <row r="192" spans="1:8" ht="109.2">
+    <row r="192" spans="1:8" ht="115.5">
       <c r="A192" s="1" t="s">
         <v>28</v>
       </c>
@@ -5342,7 +5351,7 @@
       <c r="G192" s="1"/>
       <c r="H192" s="1"/>
     </row>
-    <row r="193" spans="1:8" ht="62.4">
+    <row r="193" spans="1:8" ht="66">
       <c r="A193" s="1" t="s">
         <v>13</v>
       </c>
@@ -5368,7 +5377,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="196" spans="1:8" ht="15.6">
+    <row r="196" spans="1:8" ht="16.5">
       <c r="A196" s="1" t="s">
         <v>2</v>
       </c>
@@ -5382,7 +5391,7 @@
       <c r="G196" s="15"/>
       <c r="H196" s="16"/>
     </row>
-    <row r="197" spans="1:8" ht="15.6">
+    <row r="197" spans="1:8" ht="16.5">
       <c r="A197" s="1"/>
       <c r="B197" s="8" t="s">
         <v>147</v>
@@ -5406,7 +5415,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="198" spans="1:8" ht="17.399999999999999">
+    <row r="198" spans="1:8" ht="18">
       <c r="A198" s="2"/>
       <c r="B198" s="11">
         <v>46053</v>
@@ -5436,7 +5445,7 @@
         <v>46059</v>
       </c>
     </row>
-    <row r="199" spans="1:8" ht="31.2">
+    <row r="199" spans="1:8" ht="33">
       <c r="A199" s="1" t="s">
         <v>3</v>
       </c>
@@ -5462,7 +5471,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="200" spans="1:8" ht="15.6">
+    <row r="200" spans="1:8" ht="16.5">
       <c r="A200" s="1" t="s">
         <v>4</v>
       </c>
@@ -5488,7 +5497,7 @@
         <v>0.39583333333333331</v>
       </c>
     </row>
-    <row r="201" spans="1:8" ht="15.6">
+    <row r="201" spans="1:8" ht="16.5">
       <c r="A201" s="1" t="s">
         <v>5</v>
       </c>
@@ -5514,7 +5523,7 @@
         <v>0.91666666666666663</v>
       </c>
     </row>
-    <row r="202" spans="1:8" ht="15.6">
+    <row r="202" spans="1:8" ht="16.5">
       <c r="A202" s="1" t="s">
         <v>6</v>
       </c>
@@ -5540,7 +5549,7 @@
         <v>0.91666666666666663</v>
       </c>
     </row>
-    <row r="203" spans="1:8" ht="31.2">
+    <row r="203" spans="1:8" ht="49.5">
       <c r="A203" s="1" t="s">
         <v>7</v>
       </c>
@@ -5566,7 +5575,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="204" spans="1:8" ht="15.6">
+    <row r="204" spans="1:8" ht="16.5">
       <c r="A204" s="1" t="s">
         <v>8</v>
       </c>
@@ -5592,7 +5601,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="205" spans="1:8" ht="31.2">
+    <row r="205" spans="1:8" ht="33">
       <c r="A205" s="1" t="s">
         <v>9</v>
       </c>
@@ -5618,7 +5627,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="206" spans="1:8" ht="31.2">
+    <row r="206" spans="1:8" ht="33">
       <c r="A206" s="1" t="s">
         <v>10</v>
       </c>
@@ -5644,7 +5653,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="207" spans="1:8" ht="62.4">
+    <row r="207" spans="1:8" ht="82.5">
       <c r="A207" s="1" t="s">
         <v>11</v>
       </c>
@@ -5670,7 +5679,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="208" spans="1:8" ht="62.4">
+    <row r="208" spans="1:8" ht="66">
       <c r="A208" s="1" t="s">
         <v>12</v>
       </c>
@@ -5696,7 +5705,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="209" spans="1:8" ht="46.8">
+    <row r="209" spans="1:8" ht="49.5">
       <c r="A209" s="1" t="s">
         <v>40</v>
       </c>
@@ -5722,7 +5731,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="210" spans="1:8" ht="93.6">
+    <row r="210" spans="1:8" ht="99">
       <c r="A210" s="1" t="s">
         <v>27</v>
       </c>
@@ -5748,7 +5757,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="211" spans="1:8" ht="109.2">
+    <row r="211" spans="1:8" ht="115.5">
       <c r="A211" s="1" t="s">
         <v>28</v>
       </c>
@@ -5774,7 +5783,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="212" spans="1:8" ht="62.4">
+    <row r="212" spans="1:8" ht="66">
       <c r="A212" s="1" t="s">
         <v>13</v>
       </c>
@@ -5800,7 +5809,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="215" spans="1:8" ht="15.6">
+    <row r="215" spans="1:8" ht="16.5">
       <c r="A215" s="1"/>
       <c r="B215" s="8" t="s">
         <v>147</v>
@@ -5824,7 +5833,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="216" spans="1:8" ht="17.399999999999999">
+    <row r="216" spans="1:8" ht="18">
       <c r="A216" s="2"/>
       <c r="B216" s="11">
         <v>46111</v>
@@ -5854,7 +5863,7 @@
         <v>46117</v>
       </c>
     </row>
-    <row r="217" spans="1:8" ht="31.2">
+    <row r="217" spans="1:8" ht="33">
       <c r="A217" s="1" t="s">
         <v>3</v>
       </c>
@@ -5865,10 +5874,14 @@
       </c>
       <c r="E217" s="6"/>
       <c r="F217" s="6"/>
-      <c r="G217" s="6"/>
-      <c r="H217" s="6"/>
-    </row>
-    <row r="218" spans="1:8" ht="15.6">
+      <c r="G217" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="H217" s="6" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="218" spans="1:8" ht="16.5">
       <c r="A218" s="1" t="s">
         <v>4</v>
       </c>
@@ -5879,10 +5892,14 @@
       </c>
       <c r="E218" s="6"/>
       <c r="F218" s="6"/>
-      <c r="G218" s="6"/>
-      <c r="H218" s="13"/>
-    </row>
-    <row r="219" spans="1:8" ht="15.6">
+      <c r="G218" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H218" s="13" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="219" spans="1:8" ht="16.5">
       <c r="A219" s="1" t="s">
         <v>5</v>
       </c>
@@ -5893,10 +5910,14 @@
       </c>
       <c r="E219" s="7"/>
       <c r="F219" s="6"/>
-      <c r="G219" s="6"/>
-      <c r="H219" s="13"/>
-    </row>
-    <row r="220" spans="1:8" ht="15.6">
+      <c r="G219" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="H219" s="13" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="220" spans="1:8" ht="16.5">
       <c r="A220" s="1" t="s">
         <v>6</v>
       </c>
@@ -5907,10 +5928,14 @@
       </c>
       <c r="E220" s="7"/>
       <c r="F220" s="6"/>
-      <c r="G220" s="6"/>
-      <c r="H220" s="13"/>
-    </row>
-    <row r="221" spans="1:8" ht="31.2">
+      <c r="G220" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="H220" s="13" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="221" spans="1:8" ht="49.5">
       <c r="A221" s="1" t="s">
         <v>7</v>
       </c>
@@ -5921,10 +5946,14 @@
       </c>
       <c r="E221" s="1"/>
       <c r="F221" s="1"/>
-      <c r="G221" s="1"/>
-      <c r="H221" s="1"/>
-    </row>
-    <row r="222" spans="1:8" ht="15.6">
+      <c r="G221" s="1">
+        <v>0</v>
+      </c>
+      <c r="H221" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="222" spans="1:8" ht="16.5">
       <c r="A222" s="1" t="s">
         <v>8</v>
       </c>
@@ -5935,10 +5964,14 @@
       </c>
       <c r="E222" s="1"/>
       <c r="F222" s="1"/>
-      <c r="G222" s="1"/>
-      <c r="H222" s="1"/>
-    </row>
-    <row r="223" spans="1:8" ht="31.2">
+      <c r="G222" s="1">
+        <v>0</v>
+      </c>
+      <c r="H222" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="223" spans="1:8" ht="33">
       <c r="A223" s="1" t="s">
         <v>9</v>
       </c>
@@ -5949,10 +5982,14 @@
       </c>
       <c r="E223" s="1"/>
       <c r="F223" s="1"/>
-      <c r="G223" s="1"/>
-      <c r="H223" s="1"/>
-    </row>
-    <row r="224" spans="1:8" ht="31.2">
+      <c r="G223" s="1">
+        <v>0</v>
+      </c>
+      <c r="H223" s="1">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="224" spans="1:8" ht="33">
       <c r="A224" s="1" t="s">
         <v>10</v>
       </c>
@@ -5963,10 +6000,14 @@
       </c>
       <c r="E224" s="1"/>
       <c r="F224" s="1"/>
-      <c r="G224" s="1"/>
-      <c r="H224" s="6"/>
-    </row>
-    <row r="225" spans="1:8" ht="62.4">
+      <c r="G224" s="1">
+        <v>420</v>
+      </c>
+      <c r="H224" s="6">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="225" spans="1:8" ht="82.5">
       <c r="A225" s="1" t="s">
         <v>11</v>
       </c>
@@ -5977,10 +6018,14 @@
       </c>
       <c r="E225" s="1"/>
       <c r="F225" s="1"/>
-      <c r="G225" s="1"/>
-      <c r="H225" s="1"/>
-    </row>
-    <row r="226" spans="1:8" ht="62.4">
+      <c r="G225" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="H225" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="226" spans="1:8" ht="66">
       <c r="A226" s="1" t="s">
         <v>12</v>
       </c>
@@ -5991,10 +6036,14 @@
       </c>
       <c r="E226" s="1"/>
       <c r="F226" s="1"/>
-      <c r="G226" s="1"/>
-      <c r="H226" s="1"/>
-    </row>
-    <row r="227" spans="1:8" ht="46.8">
+      <c r="G226" s="1">
+        <v>60</v>
+      </c>
+      <c r="H226" s="1">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="227" spans="1:8" ht="49.5">
       <c r="A227" s="1" t="s">
         <v>40</v>
       </c>
@@ -6005,10 +6054,14 @@
       </c>
       <c r="E227" s="1"/>
       <c r="F227" s="1"/>
-      <c r="G227" s="1"/>
-      <c r="H227" s="1"/>
-    </row>
-    <row r="228" spans="1:8" ht="93.6">
+      <c r="G227" s="1">
+        <v>3</v>
+      </c>
+      <c r="H227" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="228" spans="1:8" ht="99">
       <c r="A228" s="1" t="s">
         <v>27</v>
       </c>
@@ -6019,10 +6072,14 @@
       </c>
       <c r="E228" s="1"/>
       <c r="F228" s="1"/>
-      <c r="G228" s="1"/>
-      <c r="H228" s="1"/>
-    </row>
-    <row r="229" spans="1:8" ht="109.2">
+      <c r="G228" s="1">
+        <v>4</v>
+      </c>
+      <c r="H228" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="229" spans="1:8" ht="115.5">
       <c r="A229" s="1" t="s">
         <v>28</v>
       </c>
@@ -6033,10 +6090,14 @@
       </c>
       <c r="E229" s="1"/>
       <c r="F229" s="1"/>
-      <c r="G229" s="1"/>
-      <c r="H229" s="1"/>
-    </row>
-    <row r="230" spans="1:8" ht="62.4">
+      <c r="G229" s="1">
+        <v>4</v>
+      </c>
+      <c r="H229" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="230" spans="1:8" ht="66">
       <c r="A230" s="1" t="s">
         <v>13</v>
       </c>
@@ -6047,12 +6108,19 @@
       </c>
       <c r="E230" s="1"/>
       <c r="F230" s="1"/>
-      <c r="G230" s="1"/>
-      <c r="H230" s="1"/>
+      <c r="G230" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="H230" s="1" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="231" spans="1:8">
       <c r="D231" t="s">
         <v>174</v>
+      </c>
+      <c r="H231" t="s">
+        <v>177</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
vault backup: 2026-04-07 09:31:05
</commit_message>
<xml_diff>
--- a/睡眠日记_Sleep_Diary1.xlsx
+++ b/睡眠日记_Sleep_Diary1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My_like\My_like\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CAA169B-9B34-47A3-BD74-8EC7D14C25E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C667A250-766A-43BC-9019-7539F96E1AB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="701" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="731" uniqueCount="178">
   <si>
     <t>睡眠日记 Sleep Diary</t>
   </si>
@@ -1126,7 +1126,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H231"/>
+  <dimension ref="A1:H247"/>
   <sheetFormatPr defaultColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="8" width="20" customWidth="1"/>
@@ -6123,16 +6123,264 @@
         <v>177</v>
       </c>
     </row>
+    <row r="232" spans="1:8" ht="16.5">
+      <c r="A232" s="1"/>
+      <c r="B232" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="C232" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="D232" s="9" t="s">
+        <v>149</v>
+      </c>
+      <c r="E232" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="F232" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="G232" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="H232" s="10" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="233" spans="1:8" ht="18">
+      <c r="A233" s="2"/>
+      <c r="B233" s="11">
+        <v>46118</v>
+      </c>
+      <c r="C233" s="11">
+        <f>B233+1</f>
+        <v>46119</v>
+      </c>
+      <c r="D233" s="11">
+        <f t="shared" ref="D233" si="21">C233+1</f>
+        <v>46120</v>
+      </c>
+      <c r="E233" s="11">
+        <f t="shared" ref="E233" si="22">D233+1</f>
+        <v>46121</v>
+      </c>
+      <c r="F233" s="11">
+        <f t="shared" ref="F233" si="23">E233+1</f>
+        <v>46122</v>
+      </c>
+      <c r="G233" s="11">
+        <f t="shared" ref="G233" si="24">F233+1</f>
+        <v>46123</v>
+      </c>
+      <c r="H233" s="11">
+        <f t="shared" ref="H233" si="25">G233+1</f>
+        <v>46124</v>
+      </c>
+    </row>
+    <row r="234" spans="1:8" ht="33">
+      <c r="A234" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B234" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="C234" s="6"/>
+      <c r="D234" s="6"/>
+      <c r="E234" s="6"/>
+      <c r="F234" s="6"/>
+      <c r="G234" s="6"/>
+      <c r="H234" s="6"/>
+    </row>
+    <row r="235" spans="1:8" ht="16.5">
+      <c r="A235" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B235" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C235" s="6"/>
+      <c r="D235" s="6"/>
+      <c r="E235" s="6"/>
+      <c r="F235" s="6"/>
+      <c r="G235" s="6"/>
+      <c r="H235" s="13"/>
+    </row>
+    <row r="236" spans="1:8" ht="16.5">
+      <c r="A236" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B236" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C236" s="6"/>
+      <c r="D236" s="6"/>
+      <c r="E236" s="7"/>
+      <c r="F236" s="6"/>
+      <c r="G236" s="6"/>
+      <c r="H236" s="13"/>
+    </row>
+    <row r="237" spans="1:8" ht="16.5">
+      <c r="A237" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B237" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C237" s="6"/>
+      <c r="D237" s="6"/>
+      <c r="E237" s="7"/>
+      <c r="F237" s="6"/>
+      <c r="G237" s="6"/>
+      <c r="H237" s="13"/>
+    </row>
+    <row r="238" spans="1:8" ht="49.5">
+      <c r="A238" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B238" s="6">
+        <v>10</v>
+      </c>
+      <c r="C238" s="1"/>
+      <c r="D238" s="7"/>
+      <c r="E238" s="1"/>
+      <c r="F238" s="1"/>
+      <c r="G238" s="1"/>
+      <c r="H238" s="1"/>
+    </row>
+    <row r="239" spans="1:8" ht="16.5">
+      <c r="A239" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B239" s="1">
+        <v>1</v>
+      </c>
+      <c r="C239" s="1"/>
+      <c r="D239" s="1"/>
+      <c r="E239" s="1"/>
+      <c r="F239" s="1"/>
+      <c r="G239" s="1"/>
+      <c r="H239" s="1"/>
+    </row>
+    <row r="240" spans="1:8" ht="33">
+      <c r="A240" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B240" s="1">
+        <v>5</v>
+      </c>
+      <c r="C240" s="1"/>
+      <c r="D240" s="1"/>
+      <c r="E240" s="1"/>
+      <c r="F240" s="1"/>
+      <c r="G240" s="1"/>
+      <c r="H240" s="1"/>
+    </row>
+    <row r="241" spans="1:8" ht="33">
+      <c r="A241" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B241" s="1">
+        <v>480</v>
+      </c>
+      <c r="C241" s="1"/>
+      <c r="D241" s="1"/>
+      <c r="E241" s="1"/>
+      <c r="F241" s="1"/>
+      <c r="G241" s="1"/>
+      <c r="H241" s="6"/>
+    </row>
+    <row r="242" spans="1:8" ht="82.5">
+      <c r="A242" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B242" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C242" s="1"/>
+      <c r="D242" s="1"/>
+      <c r="E242" s="1"/>
+      <c r="F242" s="1"/>
+      <c r="G242" s="1"/>
+      <c r="H242" s="1"/>
+    </row>
+    <row r="243" spans="1:8" ht="66">
+      <c r="A243" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B243" s="1">
+        <v>20</v>
+      </c>
+      <c r="C243" s="1"/>
+      <c r="D243" s="1"/>
+      <c r="E243" s="1"/>
+      <c r="F243" s="1"/>
+      <c r="G243" s="1"/>
+      <c r="H243" s="1"/>
+    </row>
+    <row r="244" spans="1:8" ht="49.5">
+      <c r="A244" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B244" s="1">
+        <v>4</v>
+      </c>
+      <c r="C244" s="1"/>
+      <c r="D244" s="1"/>
+      <c r="E244" s="1"/>
+      <c r="F244" s="1"/>
+      <c r="G244" s="1"/>
+      <c r="H244" s="1"/>
+    </row>
+    <row r="245" spans="1:8" ht="99">
+      <c r="A245" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B245" s="1">
+        <v>4</v>
+      </c>
+      <c r="C245" s="1"/>
+      <c r="D245" s="1"/>
+      <c r="E245" s="1"/>
+      <c r="F245" s="1"/>
+      <c r="G245" s="1"/>
+      <c r="H245" s="1"/>
+    </row>
+    <row r="246" spans="1:8" ht="115.5">
+      <c r="A246" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B246" s="1">
+        <v>4</v>
+      </c>
+      <c r="C246" s="1"/>
+      <c r="D246" s="1"/>
+      <c r="E246" s="1"/>
+      <c r="F246" s="1"/>
+      <c r="G246" s="1"/>
+      <c r="H246" s="1"/>
+    </row>
+    <row r="247" spans="1:8" ht="66">
+      <c r="A247" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B247" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C247" s="1"/>
+      <c r="D247" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E247" s="1"/>
+      <c r="F247" s="1"/>
+      <c r="G247" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="H247" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="B159:H159"/>
-    <mergeCell ref="A59:H59"/>
-    <mergeCell ref="B102:H102"/>
-    <mergeCell ref="A138:H138"/>
-    <mergeCell ref="B139:H139"/>
-    <mergeCell ref="A101:H101"/>
-    <mergeCell ref="A79:H79"/>
-    <mergeCell ref="B80:H80"/>
     <mergeCell ref="B196:H196"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A60:H60"/>
@@ -6149,6 +6397,14 @@
     <mergeCell ref="B61:H61"/>
     <mergeCell ref="A119:H119"/>
     <mergeCell ref="B120:H120"/>
+    <mergeCell ref="B159:H159"/>
+    <mergeCell ref="A59:H59"/>
+    <mergeCell ref="B102:H102"/>
+    <mergeCell ref="A138:H138"/>
+    <mergeCell ref="B139:H139"/>
+    <mergeCell ref="A101:H101"/>
+    <mergeCell ref="A79:H79"/>
+    <mergeCell ref="B80:H80"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>

</xml_diff>

<commit_message>
vault backup: 2026-04-07 09:44:11
</commit_message>
<xml_diff>
--- a/睡眠日记_Sleep_Diary1.xlsx
+++ b/睡眠日记_Sleep_Diary1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My_like\My_like\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C667A250-766A-43BC-9019-7539F96E1AB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE08AC17-4437-43DB-9926-217369407001}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="731" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="737" uniqueCount="178">
   <si>
     <t>睡眠日记 Sleep Diary</t>
   </si>
@@ -6184,7 +6184,9 @@
       <c r="B234" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="C234" s="6"/>
+      <c r="C234" s="6" t="s">
+        <v>78</v>
+      </c>
       <c r="D234" s="6"/>
       <c r="E234" s="6"/>
       <c r="F234" s="6"/>
@@ -6198,7 +6200,9 @@
       <c r="B235" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="C235" s="6"/>
+      <c r="C235" s="6" t="s">
+        <v>78</v>
+      </c>
       <c r="D235" s="6"/>
       <c r="E235" s="6"/>
       <c r="F235" s="6"/>
@@ -6212,7 +6216,9 @@
       <c r="B236" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="C236" s="6"/>
+      <c r="C236" s="6" t="s">
+        <v>38</v>
+      </c>
       <c r="D236" s="6"/>
       <c r="E236" s="7"/>
       <c r="F236" s="6"/>
@@ -6226,7 +6232,9 @@
       <c r="B237" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="C237" s="6"/>
+      <c r="C237" s="6" t="s">
+        <v>38</v>
+      </c>
       <c r="D237" s="6"/>
       <c r="E237" s="7"/>
       <c r="F237" s="6"/>
@@ -6240,7 +6248,9 @@
       <c r="B238" s="6">
         <v>10</v>
       </c>
-      <c r="C238" s="1"/>
+      <c r="C238" s="1">
+        <v>15</v>
+      </c>
       <c r="D238" s="7"/>
       <c r="E238" s="1"/>
       <c r="F238" s="1"/>
@@ -6254,7 +6264,9 @@
       <c r="B239" s="1">
         <v>1</v>
       </c>
-      <c r="C239" s="1"/>
+      <c r="C239" s="1">
+        <v>1</v>
+      </c>
       <c r="D239" s="1"/>
       <c r="E239" s="1"/>
       <c r="F239" s="1"/>
@@ -6268,7 +6280,9 @@
       <c r="B240" s="1">
         <v>5</v>
       </c>
-      <c r="C240" s="1"/>
+      <c r="C240" s="1">
+        <v>40</v>
+      </c>
       <c r="D240" s="1"/>
       <c r="E240" s="1"/>
       <c r="F240" s="1"/>
@@ -6282,7 +6296,9 @@
       <c r="B241" s="1">
         <v>480</v>
       </c>
-      <c r="C241" s="1"/>
+      <c r="C241" s="1">
+        <v>480</v>
+      </c>
       <c r="D241" s="1"/>
       <c r="E241" s="1"/>
       <c r="F241" s="1"/>
@@ -6296,7 +6312,9 @@
       <c r="B242" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C242" s="1"/>
+      <c r="C242" s="1" t="s">
+        <v>26</v>
+      </c>
       <c r="D242" s="1"/>
       <c r="E242" s="1"/>
       <c r="F242" s="1"/>
@@ -6310,7 +6328,9 @@
       <c r="B243" s="1">
         <v>20</v>
       </c>
-      <c r="C243" s="1"/>
+      <c r="C243" s="1">
+        <v>20</v>
+      </c>
       <c r="D243" s="1"/>
       <c r="E243" s="1"/>
       <c r="F243" s="1"/>
@@ -6324,7 +6344,9 @@
       <c r="B244" s="1">
         <v>4</v>
       </c>
-      <c r="C244" s="1"/>
+      <c r="C244" s="1">
+        <v>3</v>
+      </c>
       <c r="D244" s="1"/>
       <c r="E244" s="1"/>
       <c r="F244" s="1"/>
@@ -6338,7 +6360,9 @@
       <c r="B245" s="1">
         <v>4</v>
       </c>
-      <c r="C245" s="1"/>
+      <c r="C245" s="1">
+        <v>4</v>
+      </c>
       <c r="D245" s="1"/>
       <c r="E245" s="1"/>
       <c r="F245" s="1"/>
@@ -6352,7 +6376,9 @@
       <c r="B246" s="1">
         <v>4</v>
       </c>
-      <c r="C246" s="1"/>
+      <c r="C246" s="1">
+        <v>3</v>
+      </c>
       <c r="D246" s="1"/>
       <c r="E246" s="1"/>
       <c r="F246" s="1"/>
@@ -6366,7 +6392,9 @@
       <c r="B247" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C247" s="1"/>
+      <c r="C247" s="1" t="s">
+        <v>26</v>
+      </c>
       <c r="D247" s="1" t="s">
         <v>26</v>
       </c>
@@ -6381,6 +6409,14 @@
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="B159:H159"/>
+    <mergeCell ref="A59:H59"/>
+    <mergeCell ref="B102:H102"/>
+    <mergeCell ref="A138:H138"/>
+    <mergeCell ref="B139:H139"/>
+    <mergeCell ref="A101:H101"/>
+    <mergeCell ref="A79:H79"/>
+    <mergeCell ref="B80:H80"/>
     <mergeCell ref="B196:H196"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A60:H60"/>
@@ -6397,14 +6433,6 @@
     <mergeCell ref="B61:H61"/>
     <mergeCell ref="A119:H119"/>
     <mergeCell ref="B120:H120"/>
-    <mergeCell ref="B159:H159"/>
-    <mergeCell ref="A59:H59"/>
-    <mergeCell ref="B102:H102"/>
-    <mergeCell ref="A138:H138"/>
-    <mergeCell ref="B139:H139"/>
-    <mergeCell ref="A101:H101"/>
-    <mergeCell ref="A79:H79"/>
-    <mergeCell ref="B80:H80"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>

</xml_diff>

<commit_message>
vault backup: 2026-04-08 10:35:31
</commit_message>
<xml_diff>
--- a/睡眠日记_Sleep_Diary1.xlsx
+++ b/睡眠日记_Sleep_Diary1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My_like\My_like\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\My_lovwly\test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE08AC17-4437-43DB-9926-217369407001}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F04A2B78-2264-42AC-90C3-1A5C718A334A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="737" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="739" uniqueCount="178">
   <si>
     <t>睡眠日记 Sleep Diary</t>
   </si>
@@ -6187,7 +6187,9 @@
       <c r="C234" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="D234" s="6"/>
+      <c r="D234" s="6">
+        <v>0.2590277777777778</v>
+      </c>
       <c r="E234" s="6"/>
       <c r="F234" s="6"/>
       <c r="G234" s="6"/>
@@ -6203,7 +6205,9 @@
       <c r="C235" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="D235" s="6"/>
+      <c r="D235" s="6">
+        <v>0.28472222222222221</v>
+      </c>
       <c r="E235" s="6"/>
       <c r="F235" s="6"/>
       <c r="G235" s="6"/>
@@ -6219,7 +6223,9 @@
       <c r="C236" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="D236" s="6"/>
+      <c r="D236" s="6">
+        <v>0.95833333333333337</v>
+      </c>
       <c r="E236" s="7"/>
       <c r="F236" s="6"/>
       <c r="G236" s="6"/>
@@ -6235,7 +6241,9 @@
       <c r="C237" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="D237" s="6"/>
+      <c r="D237" s="6">
+        <v>0.95833333333333337</v>
+      </c>
       <c r="E237" s="7"/>
       <c r="F237" s="6"/>
       <c r="G237" s="6"/>
@@ -6251,7 +6259,9 @@
       <c r="C238" s="1">
         <v>15</v>
       </c>
-      <c r="D238" s="7"/>
+      <c r="D238" s="7" t="s">
+        <v>139</v>
+      </c>
       <c r="E238" s="1"/>
       <c r="F238" s="1"/>
       <c r="G238" s="1"/>
@@ -6267,7 +6277,9 @@
       <c r="C239" s="1">
         <v>1</v>
       </c>
-      <c r="D239" s="1"/>
+      <c r="D239" s="1">
+        <v>0</v>
+      </c>
       <c r="E239" s="1"/>
       <c r="F239" s="1"/>
       <c r="G239" s="1"/>
@@ -6283,7 +6295,9 @@
       <c r="C240" s="1">
         <v>40</v>
       </c>
-      <c r="D240" s="1"/>
+      <c r="D240" s="1">
+        <v>0</v>
+      </c>
       <c r="E240" s="1"/>
       <c r="F240" s="1"/>
       <c r="G240" s="1"/>
@@ -6299,7 +6313,9 @@
       <c r="C241" s="1">
         <v>480</v>
       </c>
-      <c r="D241" s="1"/>
+      <c r="D241" s="1">
+        <v>480</v>
+      </c>
       <c r="E241" s="1"/>
       <c r="F241" s="1"/>
       <c r="G241" s="1"/>
@@ -6315,7 +6331,9 @@
       <c r="C242" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D242" s="1"/>
+      <c r="D242" s="1" t="s">
+        <v>26</v>
+      </c>
       <c r="E242" s="1"/>
       <c r="F242" s="1"/>
       <c r="G242" s="1"/>
@@ -6331,7 +6349,9 @@
       <c r="C243" s="1">
         <v>20</v>
       </c>
-      <c r="D243" s="1"/>
+      <c r="D243" s="1">
+        <v>25</v>
+      </c>
       <c r="E243" s="1"/>
       <c r="F243" s="1"/>
       <c r="G243" s="1"/>
@@ -6347,7 +6367,9 @@
       <c r="C244" s="1">
         <v>3</v>
       </c>
-      <c r="D244" s="1"/>
+      <c r="D244" s="1">
+        <v>4</v>
+      </c>
       <c r="E244" s="1"/>
       <c r="F244" s="1"/>
       <c r="G244" s="1"/>
@@ -6363,7 +6385,9 @@
       <c r="C245" s="1">
         <v>4</v>
       </c>
-      <c r="D245" s="1"/>
+      <c r="D245" s="1">
+        <v>4</v>
+      </c>
       <c r="E245" s="1"/>
       <c r="F245" s="1"/>
       <c r="G245" s="1"/>
@@ -6379,7 +6403,9 @@
       <c r="C246" s="1">
         <v>3</v>
       </c>
-      <c r="D246" s="1"/>
+      <c r="D246" s="1">
+        <v>4</v>
+      </c>
       <c r="E246" s="1"/>
       <c r="F246" s="1"/>
       <c r="G246" s="1"/>
@@ -6409,14 +6435,6 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="B159:H159"/>
-    <mergeCell ref="A59:H59"/>
-    <mergeCell ref="B102:H102"/>
-    <mergeCell ref="A138:H138"/>
-    <mergeCell ref="B139:H139"/>
-    <mergeCell ref="A101:H101"/>
-    <mergeCell ref="A79:H79"/>
-    <mergeCell ref="B80:H80"/>
     <mergeCell ref="B196:H196"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A60:H60"/>
@@ -6433,6 +6451,14 @@
     <mergeCell ref="B61:H61"/>
     <mergeCell ref="A119:H119"/>
     <mergeCell ref="B120:H120"/>
+    <mergeCell ref="B159:H159"/>
+    <mergeCell ref="A59:H59"/>
+    <mergeCell ref="B102:H102"/>
+    <mergeCell ref="A138:H138"/>
+    <mergeCell ref="B139:H139"/>
+    <mergeCell ref="A101:H101"/>
+    <mergeCell ref="A79:H79"/>
+    <mergeCell ref="B80:H80"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>

</xml_diff>

<commit_message>
vault backup: 2026-04-09 08:22:52
</commit_message>
<xml_diff>
--- a/睡眠日记_Sleep_Diary1.xlsx
+++ b/睡眠日记_Sleep_Diary1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\My_lovwly\test\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My_like\My_like\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F04A2B78-2264-42AC-90C3-1A5C718A334A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E534FA5B-942F-4861-B279-9AA1E98EA56A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="739" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="746" uniqueCount="179">
   <si>
     <t>睡眠日记 Sleep Diary</t>
   </si>
@@ -626,6 +626,9 @@
   </si>
   <si>
     <t>睡前没有关灯</t>
+  </si>
+  <si>
+    <t>6：00</t>
   </si>
 </sst>
 </file>
@@ -6190,7 +6193,9 @@
       <c r="D234" s="6">
         <v>0.2590277777777778</v>
       </c>
-      <c r="E234" s="6"/>
+      <c r="E234" s="6" t="s">
+        <v>178</v>
+      </c>
       <c r="F234" s="6"/>
       <c r="G234" s="6"/>
       <c r="H234" s="6"/>
@@ -6208,7 +6213,9 @@
       <c r="D235" s="6">
         <v>0.28472222222222221</v>
       </c>
-      <c r="E235" s="6"/>
+      <c r="E235" s="6" t="s">
+        <v>24</v>
+      </c>
       <c r="F235" s="6"/>
       <c r="G235" s="6"/>
       <c r="H235" s="13"/>
@@ -6226,7 +6233,9 @@
       <c r="D236" s="6">
         <v>0.95833333333333337</v>
       </c>
-      <c r="E236" s="7"/>
+      <c r="E236" s="7" t="s">
+        <v>30</v>
+      </c>
       <c r="F236" s="6"/>
       <c r="G236" s="6"/>
       <c r="H236" s="13"/>
@@ -6244,7 +6253,9 @@
       <c r="D237" s="6">
         <v>0.95833333333333337</v>
       </c>
-      <c r="E237" s="7"/>
+      <c r="E237" s="7" t="s">
+        <v>30</v>
+      </c>
       <c r="F237" s="6"/>
       <c r="G237" s="6"/>
       <c r="H237" s="13"/>
@@ -6262,7 +6273,9 @@
       <c r="D238" s="7" t="s">
         <v>139</v>
       </c>
-      <c r="E238" s="1"/>
+      <c r="E238" s="1" t="s">
+        <v>139</v>
+      </c>
       <c r="F238" s="1"/>
       <c r="G238" s="1"/>
       <c r="H238" s="1"/>
@@ -6280,7 +6293,9 @@
       <c r="D239" s="1">
         <v>0</v>
       </c>
-      <c r="E239" s="1"/>
+      <c r="E239" s="1">
+        <v>0</v>
+      </c>
       <c r="F239" s="1"/>
       <c r="G239" s="1"/>
       <c r="H239" s="1"/>
@@ -6298,7 +6313,9 @@
       <c r="D240" s="1">
         <v>0</v>
       </c>
-      <c r="E240" s="1"/>
+      <c r="E240" s="1">
+        <v>0</v>
+      </c>
       <c r="F240" s="1"/>
       <c r="G240" s="1"/>
       <c r="H240" s="1"/>
@@ -6316,7 +6333,9 @@
       <c r="D241" s="1">
         <v>480</v>
       </c>
-      <c r="E241" s="1"/>
+      <c r="E241" s="1">
+        <v>480</v>
+      </c>
       <c r="F241" s="1"/>
       <c r="G241" s="1"/>
       <c r="H241" s="6"/>
@@ -6334,7 +6353,9 @@
       <c r="D242" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="E242" s="1"/>
+      <c r="E242" s="1" t="s">
+        <v>26</v>
+      </c>
       <c r="F242" s="1"/>
       <c r="G242" s="1"/>
       <c r="H242" s="1"/>
@@ -6352,7 +6373,9 @@
       <c r="D243" s="1">
         <v>25</v>
       </c>
-      <c r="E243" s="1"/>
+      <c r="E243" s="1">
+        <v>60</v>
+      </c>
       <c r="F243" s="1"/>
       <c r="G243" s="1"/>
       <c r="H243" s="1"/>
@@ -6370,7 +6393,9 @@
       <c r="D244" s="1">
         <v>4</v>
       </c>
-      <c r="E244" s="1"/>
+      <c r="E244" s="1">
+        <v>4</v>
+      </c>
       <c r="F244" s="1"/>
       <c r="G244" s="1"/>
       <c r="H244" s="1"/>
@@ -6388,7 +6413,9 @@
       <c r="D245" s="1">
         <v>4</v>
       </c>
-      <c r="E245" s="1"/>
+      <c r="E245" s="1">
+        <v>2</v>
+      </c>
       <c r="F245" s="1"/>
       <c r="G245" s="1"/>
       <c r="H245" s="1"/>
@@ -6406,7 +6433,9 @@
       <c r="D246" s="1">
         <v>4</v>
       </c>
-      <c r="E246" s="1"/>
+      <c r="E246" s="1">
+        <v>4</v>
+      </c>
       <c r="F246" s="1"/>
       <c r="G246" s="1"/>
       <c r="H246" s="1"/>
@@ -6424,7 +6453,9 @@
       <c r="D247" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="E247" s="1"/>
+      <c r="E247" s="1" t="s">
+        <v>26</v>
+      </c>
       <c r="F247" s="1"/>
       <c r="G247" s="1" t="s">
         <v>26</v>
@@ -6435,6 +6466,14 @@
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="B159:H159"/>
+    <mergeCell ref="A59:H59"/>
+    <mergeCell ref="B102:H102"/>
+    <mergeCell ref="A138:H138"/>
+    <mergeCell ref="B139:H139"/>
+    <mergeCell ref="A101:H101"/>
+    <mergeCell ref="A79:H79"/>
+    <mergeCell ref="B80:H80"/>
     <mergeCell ref="B196:H196"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A60:H60"/>
@@ -6451,14 +6490,6 @@
     <mergeCell ref="B61:H61"/>
     <mergeCell ref="A119:H119"/>
     <mergeCell ref="B120:H120"/>
-    <mergeCell ref="B159:H159"/>
-    <mergeCell ref="A59:H59"/>
-    <mergeCell ref="B102:H102"/>
-    <mergeCell ref="A138:H138"/>
-    <mergeCell ref="B139:H139"/>
-    <mergeCell ref="A101:H101"/>
-    <mergeCell ref="A79:H79"/>
-    <mergeCell ref="B80:H80"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>

</xml_diff>

<commit_message>
vault backup: 2026-04-10 09:12:17
</commit_message>
<xml_diff>
--- a/睡眠日记_Sleep_Diary1.xlsx
+++ b/睡眠日记_Sleep_Diary1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My_like\My_like\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E534FA5B-942F-4861-B279-9AA1E98EA56A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA4A72FE-CB1F-4328-9231-8D93B42F86BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="746" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="752" uniqueCount="180">
   <si>
     <t>睡眠日记 Sleep Diary</t>
   </si>
@@ -629,6 +629,9 @@
   </si>
   <si>
     <t>6：00</t>
+  </si>
+  <si>
+    <t>3 min</t>
   </si>
 </sst>
 </file>
@@ -6196,7 +6199,9 @@
       <c r="E234" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="F234" s="6"/>
+      <c r="F234" s="6" t="s">
+        <v>125</v>
+      </c>
       <c r="G234" s="6"/>
       <c r="H234" s="6"/>
     </row>
@@ -6216,7 +6221,9 @@
       <c r="E235" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="F235" s="6"/>
+      <c r="F235" s="6" t="s">
+        <v>16</v>
+      </c>
       <c r="G235" s="6"/>
       <c r="H235" s="13"/>
     </row>
@@ -6236,7 +6243,9 @@
       <c r="E236" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="F236" s="6"/>
+      <c r="F236" s="6" t="s">
+        <v>67</v>
+      </c>
       <c r="G236" s="6"/>
       <c r="H236" s="13"/>
     </row>
@@ -6276,7 +6285,9 @@
       <c r="E238" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="F238" s="1"/>
+      <c r="F238" s="1" t="s">
+        <v>179</v>
+      </c>
       <c r="G238" s="1"/>
       <c r="H238" s="1"/>
     </row>
@@ -6296,7 +6307,9 @@
       <c r="E239" s="1">
         <v>0</v>
       </c>
-      <c r="F239" s="1"/>
+      <c r="F239" s="1">
+        <v>0</v>
+      </c>
       <c r="G239" s="1"/>
       <c r="H239" s="1"/>
     </row>
@@ -6316,7 +6329,9 @@
       <c r="E240" s="1">
         <v>0</v>
       </c>
-      <c r="F240" s="1"/>
+      <c r="F240" s="1">
+        <v>0</v>
+      </c>
       <c r="G240" s="1"/>
       <c r="H240" s="1"/>
     </row>
@@ -6331,12 +6346,14 @@
         <v>480</v>
       </c>
       <c r="D241" s="1">
-        <v>480</v>
+        <v>430</v>
       </c>
       <c r="E241" s="1">
-        <v>480</v>
-      </c>
-      <c r="F241" s="1"/>
+        <v>420</v>
+      </c>
+      <c r="F241" s="1">
+        <v>420</v>
+      </c>
       <c r="G241" s="1"/>
       <c r="H241" s="6"/>
     </row>
@@ -6356,7 +6373,9 @@
       <c r="E242" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="F242" s="1"/>
+      <c r="F242" s="1" t="s">
+        <v>26</v>
+      </c>
       <c r="G242" s="1"/>
       <c r="H242" s="1"/>
     </row>
@@ -6376,7 +6395,9 @@
       <c r="E243" s="1">
         <v>60</v>
       </c>
-      <c r="F243" s="1"/>
+      <c r="F243" s="1">
+        <v>40</v>
+      </c>
       <c r="G243" s="1"/>
       <c r="H243" s="1"/>
     </row>
@@ -6396,7 +6417,9 @@
       <c r="E244" s="1">
         <v>4</v>
       </c>
-      <c r="F244" s="1"/>
+      <c r="F244" s="1">
+        <v>4</v>
+      </c>
       <c r="G244" s="1"/>
       <c r="H244" s="1"/>
     </row>
@@ -6416,7 +6439,9 @@
       <c r="E245" s="1">
         <v>2</v>
       </c>
-      <c r="F245" s="1"/>
+      <c r="F245" s="1">
+        <v>3</v>
+      </c>
       <c r="G245" s="1"/>
       <c r="H245" s="1"/>
     </row>
@@ -6436,7 +6461,9 @@
       <c r="E246" s="1">
         <v>4</v>
       </c>
-      <c r="F246" s="1"/>
+      <c r="F246" s="1">
+        <v>4</v>
+      </c>
       <c r="G246" s="1"/>
       <c r="H246" s="1"/>
     </row>
@@ -6456,7 +6483,9 @@
       <c r="E247" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="F247" s="1"/>
+      <c r="F247" s="1" t="s">
+        <v>26</v>
+      </c>
       <c r="G247" s="1" t="s">
         <v>26</v>
       </c>
@@ -6466,14 +6495,6 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="B159:H159"/>
-    <mergeCell ref="A59:H59"/>
-    <mergeCell ref="B102:H102"/>
-    <mergeCell ref="A138:H138"/>
-    <mergeCell ref="B139:H139"/>
-    <mergeCell ref="A101:H101"/>
-    <mergeCell ref="A79:H79"/>
-    <mergeCell ref="B80:H80"/>
     <mergeCell ref="B196:H196"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A60:H60"/>
@@ -6490,6 +6511,14 @@
     <mergeCell ref="B61:H61"/>
     <mergeCell ref="A119:H119"/>
     <mergeCell ref="B120:H120"/>
+    <mergeCell ref="B159:H159"/>
+    <mergeCell ref="A59:H59"/>
+    <mergeCell ref="B102:H102"/>
+    <mergeCell ref="A138:H138"/>
+    <mergeCell ref="B139:H139"/>
+    <mergeCell ref="A101:H101"/>
+    <mergeCell ref="A79:H79"/>
+    <mergeCell ref="B80:H80"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>

</xml_diff>

<commit_message>
vault backup: 2026-04-11 13:40:28
</commit_message>
<xml_diff>
--- a/睡眠日记_Sleep_Diary1.xlsx
+++ b/睡眠日记_Sleep_Diary1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My_like\My_like\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA4A72FE-CB1F-4328-9231-8D93B42F86BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DAFFE8D-7DFF-4163-B3C4-2FC34A9659BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="752" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="757" uniqueCount="183">
   <si>
     <t>睡眠日记 Sleep Diary</t>
   </si>
@@ -632,6 +632,15 @@
   </si>
   <si>
     <t>3 min</t>
+  </si>
+  <si>
+    <t>11：40</t>
+  </si>
+  <si>
+    <t>0：40</t>
+  </si>
+  <si>
+    <t>1：30</t>
   </si>
 </sst>
 </file>
@@ -6202,7 +6211,9 @@
       <c r="F234" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="G234" s="6"/>
+      <c r="G234" s="6" t="s">
+        <v>180</v>
+      </c>
       <c r="H234" s="6"/>
     </row>
     <row r="235" spans="1:8" ht="16.5">
@@ -6224,7 +6235,9 @@
       <c r="F235" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G235" s="6"/>
+      <c r="G235" s="6" t="s">
+        <v>180</v>
+      </c>
       <c r="H235" s="13"/>
     </row>
     <row r="236" spans="1:8" ht="16.5">
@@ -6246,7 +6259,9 @@
       <c r="F236" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="G236" s="6"/>
+      <c r="G236" s="6" t="s">
+        <v>181</v>
+      </c>
       <c r="H236" s="13"/>
     </row>
     <row r="237" spans="1:8" ht="16.5">
@@ -6266,7 +6281,9 @@
         <v>30</v>
       </c>
       <c r="F237" s="6"/>
-      <c r="G237" s="6"/>
+      <c r="G237" s="6" t="s">
+        <v>182</v>
+      </c>
       <c r="H237" s="13"/>
     </row>
     <row r="238" spans="1:8" ht="49.5">
@@ -6288,7 +6305,9 @@
       <c r="F238" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="G238" s="1"/>
+      <c r="G238" s="1">
+        <v>0</v>
+      </c>
       <c r="H238" s="1"/>
     </row>
     <row r="239" spans="1:8" ht="16.5">
@@ -6310,7 +6329,9 @@
       <c r="F239" s="1">
         <v>0</v>
       </c>
-      <c r="G239" s="1"/>
+      <c r="G239" s="1">
+        <v>1</v>
+      </c>
       <c r="H239" s="1"/>
     </row>
     <row r="240" spans="1:8" ht="33">
@@ -6332,7 +6353,9 @@
       <c r="F240" s="1">
         <v>0</v>
       </c>
-      <c r="G240" s="1"/>
+      <c r="G240" s="1">
+        <v>30</v>
+      </c>
       <c r="H240" s="1"/>
     </row>
     <row r="241" spans="1:8" ht="33">
@@ -6354,7 +6377,9 @@
       <c r="F241" s="1">
         <v>420</v>
       </c>
-      <c r="G241" s="1"/>
+      <c r="G241" s="1">
+        <v>540</v>
+      </c>
       <c r="H241" s="6"/>
     </row>
     <row r="242" spans="1:8" ht="82.5">
@@ -6376,7 +6401,9 @@
       <c r="F242" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="G242" s="1"/>
+      <c r="G242" s="1" t="s">
+        <v>26</v>
+      </c>
       <c r="H242" s="1"/>
     </row>
     <row r="243" spans="1:8" ht="66">
@@ -6398,7 +6425,9 @@
       <c r="F243" s="1">
         <v>40</v>
       </c>
-      <c r="G243" s="1"/>
+      <c r="G243" s="1">
+        <v>0</v>
+      </c>
       <c r="H243" s="1"/>
     </row>
     <row r="244" spans="1:8" ht="49.5">
@@ -6420,7 +6449,9 @@
       <c r="F244" s="1">
         <v>4</v>
       </c>
-      <c r="G244" s="1"/>
+      <c r="G244" s="1">
+        <v>4</v>
+      </c>
       <c r="H244" s="1"/>
     </row>
     <row r="245" spans="1:8" ht="99">
@@ -6442,7 +6473,9 @@
       <c r="F245" s="1">
         <v>3</v>
       </c>
-      <c r="G245" s="1"/>
+      <c r="G245" s="1">
+        <v>4</v>
+      </c>
       <c r="H245" s="1"/>
     </row>
     <row r="246" spans="1:8" ht="115.5">
@@ -6464,7 +6497,9 @@
       <c r="F246" s="1">
         <v>4</v>
       </c>
-      <c r="G246" s="1"/>
+      <c r="G246" s="1">
+        <v>3</v>
+      </c>
       <c r="H246" s="1"/>
     </row>
     <row r="247" spans="1:8" ht="66">
@@ -6495,6 +6530,14 @@
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="B159:H159"/>
+    <mergeCell ref="A59:H59"/>
+    <mergeCell ref="B102:H102"/>
+    <mergeCell ref="A138:H138"/>
+    <mergeCell ref="B139:H139"/>
+    <mergeCell ref="A101:H101"/>
+    <mergeCell ref="A79:H79"/>
+    <mergeCell ref="B80:H80"/>
     <mergeCell ref="B196:H196"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A60:H60"/>
@@ -6511,14 +6554,6 @@
     <mergeCell ref="B61:H61"/>
     <mergeCell ref="A119:H119"/>
     <mergeCell ref="B120:H120"/>
-    <mergeCell ref="B159:H159"/>
-    <mergeCell ref="A59:H59"/>
-    <mergeCell ref="B102:H102"/>
-    <mergeCell ref="A138:H138"/>
-    <mergeCell ref="B139:H139"/>
-    <mergeCell ref="A101:H101"/>
-    <mergeCell ref="A79:H79"/>
-    <mergeCell ref="B80:H80"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>

</xml_diff>

<commit_message>
vault backup: 2026-04-12 11:08:25
</commit_message>
<xml_diff>
--- a/睡眠日记_Sleep_Diary1.xlsx
+++ b/睡眠日记_Sleep_Diary1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My_like\My_like\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DAFFE8D-7DFF-4163-B3C4-2FC34A9659BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63165B8A-A26A-4C7C-B148-CE7A6995B68D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="757" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="790" uniqueCount="187">
   <si>
     <t>睡眠日记 Sleep Diary</t>
   </si>
@@ -641,6 +641,18 @@
   </si>
   <si>
     <t>1：30</t>
+  </si>
+  <si>
+    <t>9：47</t>
+  </si>
+  <si>
+    <t>9：50</t>
+  </si>
+  <si>
+    <t>00：20</t>
+  </si>
+  <si>
+    <t>540 min</t>
   </si>
 </sst>
 </file>
@@ -1141,7 +1153,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H247"/>
+  <dimension ref="A1:H265"/>
   <sheetFormatPr defaultColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="8" width="20" customWidth="1"/>
@@ -6214,7 +6226,9 @@
       <c r="G234" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="H234" s="6"/>
+      <c r="H234" s="6" t="s">
+        <v>183</v>
+      </c>
     </row>
     <row r="235" spans="1:8" ht="16.5">
       <c r="A235" s="1" t="s">
@@ -6238,7 +6252,9 @@
       <c r="G235" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="H235" s="13"/>
+      <c r="H235" s="13" t="s">
+        <v>184</v>
+      </c>
     </row>
     <row r="236" spans="1:8" ht="16.5">
       <c r="A236" s="1" t="s">
@@ -6262,7 +6278,9 @@
       <c r="G236" s="6" t="s">
         <v>181</v>
       </c>
-      <c r="H236" s="13"/>
+      <c r="H236" s="13" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="237" spans="1:8" ht="16.5">
       <c r="A237" s="1" t="s">
@@ -6284,7 +6302,9 @@
       <c r="G237" s="6" t="s">
         <v>182</v>
       </c>
-      <c r="H237" s="13"/>
+      <c r="H237" s="13" t="s">
+        <v>185</v>
+      </c>
     </row>
     <row r="238" spans="1:8" ht="49.5">
       <c r="A238" s="1" t="s">
@@ -6308,7 +6328,9 @@
       <c r="G238" s="1">
         <v>0</v>
       </c>
-      <c r="H238" s="1"/>
+      <c r="H238" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="239" spans="1:8" ht="16.5">
       <c r="A239" s="1" t="s">
@@ -6332,7 +6354,9 @@
       <c r="G239" s="1">
         <v>1</v>
       </c>
-      <c r="H239" s="1"/>
+      <c r="H239" s="1">
+        <v>1</v>
+      </c>
     </row>
     <row r="240" spans="1:8" ht="33">
       <c r="A240" s="1" t="s">
@@ -6356,7 +6380,9 @@
       <c r="G240" s="1">
         <v>30</v>
       </c>
-      <c r="H240" s="1"/>
+      <c r="H240" s="1">
+        <v>30</v>
+      </c>
     </row>
     <row r="241" spans="1:8" ht="33">
       <c r="A241" s="1" t="s">
@@ -6380,7 +6406,9 @@
       <c r="G241" s="1">
         <v>540</v>
       </c>
-      <c r="H241" s="6"/>
+      <c r="H241" s="6" t="s">
+        <v>186</v>
+      </c>
     </row>
     <row r="242" spans="1:8" ht="82.5">
       <c r="A242" s="1" t="s">
@@ -6404,7 +6432,9 @@
       <c r="G242" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="H242" s="1"/>
+      <c r="H242" s="1" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="243" spans="1:8" ht="66">
       <c r="A243" s="1" t="s">
@@ -6428,7 +6458,9 @@
       <c r="G243" s="1">
         <v>0</v>
       </c>
-      <c r="H243" s="1"/>
+      <c r="H243" s="1">
+        <v>60</v>
+      </c>
     </row>
     <row r="244" spans="1:8" ht="49.5">
       <c r="A244" s="1" t="s">
@@ -6452,7 +6484,9 @@
       <c r="G244" s="1">
         <v>4</v>
       </c>
-      <c r="H244" s="1"/>
+      <c r="H244" s="1">
+        <v>4</v>
+      </c>
     </row>
     <row r="245" spans="1:8" ht="99">
       <c r="A245" s="1" t="s">
@@ -6476,7 +6510,9 @@
       <c r="G245" s="1">
         <v>4</v>
       </c>
-      <c r="H245" s="1"/>
+      <c r="H245" s="1">
+        <v>4</v>
+      </c>
     </row>
     <row r="246" spans="1:8" ht="115.5">
       <c r="A246" s="1" t="s">
@@ -6500,7 +6536,9 @@
       <c r="G246" s="1">
         <v>3</v>
       </c>
-      <c r="H246" s="1"/>
+      <c r="H246" s="1">
+        <v>4</v>
+      </c>
     </row>
     <row r="247" spans="1:8" ht="66">
       <c r="A247" s="1" t="s">
@@ -6524,20 +6562,248 @@
       <c r="G247" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="H247" s="1" t="s">
+      <c r="H247" s="1">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="250" spans="1:8" ht="16.5">
+      <c r="A250" s="1"/>
+      <c r="B250" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="C250" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="D250" s="9" t="s">
+        <v>149</v>
+      </c>
+      <c r="E250" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="F250" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="G250" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="H250" s="10" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="251" spans="1:8" ht="18">
+      <c r="A251" s="2"/>
+      <c r="B251" s="11">
+        <v>46125</v>
+      </c>
+      <c r="C251" s="11">
+        <f>B251+1</f>
+        <v>46126</v>
+      </c>
+      <c r="D251" s="11">
+        <f t="shared" ref="D251" si="26">C251+1</f>
+        <v>46127</v>
+      </c>
+      <c r="E251" s="11">
+        <f t="shared" ref="E251" si="27">D251+1</f>
+        <v>46128</v>
+      </c>
+      <c r="F251" s="11">
+        <f t="shared" ref="F251" si="28">E251+1</f>
+        <v>46129</v>
+      </c>
+      <c r="G251" s="11">
+        <f t="shared" ref="G251" si="29">F251+1</f>
+        <v>46130</v>
+      </c>
+      <c r="H251" s="11">
+        <f t="shared" ref="H251" si="30">G251+1</f>
+        <v>46131</v>
+      </c>
+    </row>
+    <row r="252" spans="1:8" ht="33">
+      <c r="A252" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B252" s="12"/>
+      <c r="C252" s="6"/>
+      <c r="D252" s="6"/>
+      <c r="E252" s="6"/>
+      <c r="F252" s="6"/>
+      <c r="G252" s="6"/>
+      <c r="H252" s="6"/>
+    </row>
+    <row r="253" spans="1:8" ht="16.5">
+      <c r="A253" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B253" s="6"/>
+      <c r="C253" s="6"/>
+      <c r="D253" s="6"/>
+      <c r="E253" s="6"/>
+      <c r="F253" s="6"/>
+      <c r="G253" s="6"/>
+      <c r="H253" s="13"/>
+    </row>
+    <row r="254" spans="1:8" ht="16.5">
+      <c r="A254" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B254" s="6"/>
+      <c r="C254" s="6"/>
+      <c r="D254" s="6"/>
+      <c r="E254" s="7"/>
+      <c r="F254" s="6"/>
+      <c r="G254" s="6"/>
+      <c r="H254" s="13"/>
+    </row>
+    <row r="255" spans="1:8" ht="16.5">
+      <c r="A255" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B255" s="6"/>
+      <c r="C255" s="6"/>
+      <c r="D255" s="6"/>
+      <c r="E255" s="7"/>
+      <c r="F255" s="6"/>
+      <c r="G255" s="6"/>
+      <c r="H255" s="13"/>
+    </row>
+    <row r="256" spans="1:8" ht="49.5">
+      <c r="A256" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B256" s="6"/>
+      <c r="C256" s="1"/>
+      <c r="D256" s="7"/>
+      <c r="E256" s="1"/>
+      <c r="F256" s="1"/>
+      <c r="G256" s="1"/>
+      <c r="H256" s="1"/>
+    </row>
+    <row r="257" spans="1:8" ht="16.5">
+      <c r="A257" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B257" s="1"/>
+      <c r="C257" s="1"/>
+      <c r="D257" s="1"/>
+      <c r="E257" s="1"/>
+      <c r="F257" s="1"/>
+      <c r="G257" s="1"/>
+      <c r="H257" s="1"/>
+    </row>
+    <row r="258" spans="1:8" ht="33">
+      <c r="A258" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B258" s="1"/>
+      <c r="C258" s="1"/>
+      <c r="D258" s="1"/>
+      <c r="E258" s="1"/>
+      <c r="F258" s="1"/>
+      <c r="G258" s="1"/>
+      <c r="H258" s="1"/>
+    </row>
+    <row r="259" spans="1:8" ht="33">
+      <c r="A259" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B259" s="1"/>
+      <c r="C259" s="1"/>
+      <c r="D259" s="1"/>
+      <c r="E259" s="1"/>
+      <c r="F259" s="1"/>
+      <c r="G259" s="1"/>
+      <c r="H259" s="6"/>
+    </row>
+    <row r="260" spans="1:8" ht="82.5">
+      <c r="A260" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B260" s="1"/>
+      <c r="C260" s="1"/>
+      <c r="D260" s="1"/>
+      <c r="E260" s="1"/>
+      <c r="F260" s="1"/>
+      <c r="G260" s="1"/>
+      <c r="H260" s="1"/>
+    </row>
+    <row r="261" spans="1:8" ht="66">
+      <c r="A261" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B261" s="1"/>
+      <c r="C261" s="1"/>
+      <c r="D261" s="1"/>
+      <c r="E261" s="1"/>
+      <c r="F261" s="1"/>
+      <c r="G261" s="1"/>
+      <c r="H261" s="1"/>
+    </row>
+    <row r="262" spans="1:8" ht="49.5">
+      <c r="A262" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B262" s="1"/>
+      <c r="C262" s="1"/>
+      <c r="D262" s="1"/>
+      <c r="E262" s="1"/>
+      <c r="F262" s="1"/>
+      <c r="G262" s="1"/>
+      <c r="H262" s="1"/>
+    </row>
+    <row r="263" spans="1:8" ht="99">
+      <c r="A263" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B263" s="1"/>
+      <c r="C263" s="1"/>
+      <c r="D263" s="1"/>
+      <c r="E263" s="1"/>
+      <c r="F263" s="1"/>
+      <c r="G263" s="1"/>
+      <c r="H263" s="1"/>
+    </row>
+    <row r="264" spans="1:8" ht="115.5">
+      <c r="A264" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B264" s="1"/>
+      <c r="C264" s="1"/>
+      <c r="D264" s="1"/>
+      <c r="E264" s="1"/>
+      <c r="F264" s="1"/>
+      <c r="G264" s="1"/>
+      <c r="H264" s="1"/>
+    </row>
+    <row r="265" spans="1:8" ht="66">
+      <c r="A265" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B265" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C265" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D265" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E265" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F265" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="G265" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="H265" s="1" t="s">
         <v>26</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="B159:H159"/>
-    <mergeCell ref="A59:H59"/>
-    <mergeCell ref="B102:H102"/>
-    <mergeCell ref="A138:H138"/>
-    <mergeCell ref="B139:H139"/>
-    <mergeCell ref="A101:H101"/>
-    <mergeCell ref="A79:H79"/>
-    <mergeCell ref="B80:H80"/>
     <mergeCell ref="B196:H196"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A60:H60"/>
@@ -6554,6 +6820,14 @@
     <mergeCell ref="B61:H61"/>
     <mergeCell ref="A119:H119"/>
     <mergeCell ref="B120:H120"/>
+    <mergeCell ref="B159:H159"/>
+    <mergeCell ref="A59:H59"/>
+    <mergeCell ref="B102:H102"/>
+    <mergeCell ref="A138:H138"/>
+    <mergeCell ref="B139:H139"/>
+    <mergeCell ref="A101:H101"/>
+    <mergeCell ref="A79:H79"/>
+    <mergeCell ref="B80:H80"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>

</xml_diff>

<commit_message>
vault backup: 2026-04-13 09:53:28
</commit_message>
<xml_diff>
--- a/睡眠日记_Sleep_Diary1.xlsx
+++ b/睡眠日记_Sleep_Diary1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My_like\My_like\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\My_lovwly\test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63165B8A-A26A-4C7C-B148-CE7A6995B68D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFD703BE-79E1-4BFC-847C-C943BF9289B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="790" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="803" uniqueCount="188">
   <si>
     <t>睡眠日记 Sleep Diary</t>
   </si>
@@ -653,6 +653,9 @@
   </si>
   <si>
     <t>540 min</t>
+  </si>
+  <si>
+    <t>有点被流浪汉吓到</t>
   </si>
 </sst>
 </file>
@@ -1153,7 +1156,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H265"/>
+  <dimension ref="A1:H266"/>
   <sheetFormatPr defaultColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="8" width="20" customWidth="1"/>
@@ -6624,7 +6627,9 @@
       <c r="A252" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B252" s="12"/>
+      <c r="B252" s="12" t="s">
+        <v>78</v>
+      </c>
       <c r="C252" s="6"/>
       <c r="D252" s="6"/>
       <c r="E252" s="6"/>
@@ -6636,7 +6641,9 @@
       <c r="A253" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B253" s="6"/>
+      <c r="B253" s="6" t="s">
+        <v>78</v>
+      </c>
       <c r="C253" s="6"/>
       <c r="D253" s="6"/>
       <c r="E253" s="6"/>
@@ -6648,7 +6655,9 @@
       <c r="A254" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B254" s="6"/>
+      <c r="B254" s="6" t="s">
+        <v>30</v>
+      </c>
       <c r="C254" s="6"/>
       <c r="D254" s="6"/>
       <c r="E254" s="7"/>
@@ -6660,7 +6669,9 @@
       <c r="A255" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B255" s="6"/>
+      <c r="B255" s="6" t="s">
+        <v>38</v>
+      </c>
       <c r="C255" s="6"/>
       <c r="D255" s="6"/>
       <c r="E255" s="7"/>
@@ -6672,7 +6683,9 @@
       <c r="A256" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B256" s="6"/>
+      <c r="B256" s="6" t="s">
+        <v>141</v>
+      </c>
       <c r="C256" s="1"/>
       <c r="D256" s="7"/>
       <c r="E256" s="1"/>
@@ -6684,7 +6697,9 @@
       <c r="A257" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B257" s="1"/>
+      <c r="B257" s="1">
+        <v>1</v>
+      </c>
       <c r="C257" s="1"/>
       <c r="D257" s="1"/>
       <c r="E257" s="1"/>
@@ -6696,7 +6711,9 @@
       <c r="A258" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B258" s="1"/>
+      <c r="B258" s="1">
+        <v>60</v>
+      </c>
       <c r="C258" s="1"/>
       <c r="D258" s="1"/>
       <c r="E258" s="1"/>
@@ -6708,7 +6725,9 @@
       <c r="A259" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B259" s="1"/>
+      <c r="B259" s="1">
+        <v>480</v>
+      </c>
       <c r="C259" s="1"/>
       <c r="D259" s="1"/>
       <c r="E259" s="1"/>
@@ -6720,19 +6739,35 @@
       <c r="A260" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B260" s="1"/>
-      <c r="C260" s="1"/>
-      <c r="D260" s="1"/>
-      <c r="E260" s="1"/>
-      <c r="F260" s="1"/>
-      <c r="G260" s="1"/>
-      <c r="H260" s="1"/>
+      <c r="B260" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C260" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D260" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E260" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F260" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="G260" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="H260" s="1" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="261" spans="1:8" ht="66">
       <c r="A261" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B261" s="1"/>
+      <c r="B261" s="1">
+        <v>40</v>
+      </c>
       <c r="C261" s="1"/>
       <c r="D261" s="1"/>
       <c r="E261" s="1"/>
@@ -6744,7 +6779,9 @@
       <c r="A262" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B262" s="1"/>
+      <c r="B262" s="1">
+        <v>4</v>
+      </c>
       <c r="C262" s="1"/>
       <c r="D262" s="1"/>
       <c r="E262" s="1"/>
@@ -6756,7 +6793,9 @@
       <c r="A263" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B263" s="1"/>
+      <c r="B263" s="1">
+        <v>4</v>
+      </c>
       <c r="C263" s="1"/>
       <c r="D263" s="1"/>
       <c r="E263" s="1"/>
@@ -6768,7 +6807,9 @@
       <c r="A264" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B264" s="1"/>
+      <c r="B264" s="1">
+        <v>4</v>
+      </c>
       <c r="C264" s="1"/>
       <c r="D264" s="1"/>
       <c r="E264" s="1"/>
@@ -6802,8 +6843,21 @@
         <v>26</v>
       </c>
     </row>
+    <row r="266" spans="1:8">
+      <c r="B266" t="s">
+        <v>187</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="B159:H159"/>
+    <mergeCell ref="A59:H59"/>
+    <mergeCell ref="B102:H102"/>
+    <mergeCell ref="A138:H138"/>
+    <mergeCell ref="B139:H139"/>
+    <mergeCell ref="A101:H101"/>
+    <mergeCell ref="A79:H79"/>
+    <mergeCell ref="B80:H80"/>
     <mergeCell ref="B196:H196"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A60:H60"/>
@@ -6820,14 +6874,6 @@
     <mergeCell ref="B61:H61"/>
     <mergeCell ref="A119:H119"/>
     <mergeCell ref="B120:H120"/>
-    <mergeCell ref="B159:H159"/>
-    <mergeCell ref="A59:H59"/>
-    <mergeCell ref="B102:H102"/>
-    <mergeCell ref="A138:H138"/>
-    <mergeCell ref="B139:H139"/>
-    <mergeCell ref="A101:H101"/>
-    <mergeCell ref="A79:H79"/>
-    <mergeCell ref="B80:H80"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>

</xml_diff>

<commit_message>
vault backup: 2026-04-27 17:38:08
</commit_message>
<xml_diff>
--- a/睡眠日记_Sleep_Diary1.xlsx
+++ b/睡眠日记_Sleep_Diary1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\My_lovwly\test\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My_like\My_like\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFD703BE-79E1-4BFC-847C-C943BF9289B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6952AF17-AF7E-4B2B-ABE4-D22C95FE7AC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7095" yWindow="0" windowWidth="17085" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="睡眠日记 Sleep Diary" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="803" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="808" uniqueCount="192">
   <si>
     <t>睡眠日记 Sleep Diary</t>
   </si>
@@ -656,6 +656,18 @@
   </si>
   <si>
     <t>有点被流浪汉吓到</t>
+  </si>
+  <si>
+    <t>12：00</t>
+  </si>
+  <si>
+    <t>240 min</t>
+  </si>
+  <si>
+    <t>止疼药</t>
+  </si>
+  <si>
+    <t>300 min</t>
   </si>
 </sst>
 </file>
@@ -6633,7 +6645,9 @@
       <c r="C252" s="6"/>
       <c r="D252" s="6"/>
       <c r="E252" s="6"/>
-      <c r="F252" s="6"/>
+      <c r="F252" s="6" t="s">
+        <v>43</v>
+      </c>
       <c r="G252" s="6"/>
       <c r="H252" s="6"/>
     </row>
@@ -6647,7 +6661,9 @@
       <c r="C253" s="6"/>
       <c r="D253" s="6"/>
       <c r="E253" s="6"/>
-      <c r="F253" s="6"/>
+      <c r="F253" s="6" t="s">
+        <v>184</v>
+      </c>
       <c r="G253" s="6"/>
       <c r="H253" s="13"/>
     </row>
@@ -6661,7 +6677,9 @@
       <c r="C254" s="6"/>
       <c r="D254" s="6"/>
       <c r="E254" s="7"/>
-      <c r="F254" s="6"/>
+      <c r="F254" s="6" t="s">
+        <v>127</v>
+      </c>
       <c r="G254" s="6"/>
       <c r="H254" s="13"/>
     </row>
@@ -6675,7 +6693,9 @@
       <c r="C255" s="6"/>
       <c r="D255" s="6"/>
       <c r="E255" s="7"/>
-      <c r="F255" s="6"/>
+      <c r="F255" s="6" t="s">
+        <v>188</v>
+      </c>
       <c r="G255" s="6"/>
       <c r="H255" s="13"/>
     </row>
@@ -6689,7 +6709,9 @@
       <c r="C256" s="1"/>
       <c r="D256" s="7"/>
       <c r="E256" s="1"/>
-      <c r="F256" s="1"/>
+      <c r="F256" s="1" t="s">
+        <v>189</v>
+      </c>
       <c r="G256" s="1"/>
       <c r="H256" s="1"/>
     </row>
@@ -6703,7 +6725,9 @@
       <c r="C257" s="1"/>
       <c r="D257" s="1"/>
       <c r="E257" s="1"/>
-      <c r="F257" s="1"/>
+      <c r="F257">
+        <v>0</v>
+      </c>
       <c r="G257" s="1"/>
       <c r="H257" s="1"/>
     </row>
@@ -6717,7 +6741,9 @@
       <c r="C258" s="1"/>
       <c r="D258" s="1"/>
       <c r="E258" s="1"/>
-      <c r="F258" s="1"/>
+      <c r="F258" s="1">
+        <v>0</v>
+      </c>
       <c r="G258" s="1"/>
       <c r="H258" s="1"/>
     </row>
@@ -6731,7 +6757,9 @@
       <c r="C259" s="1"/>
       <c r="D259" s="1"/>
       <c r="E259" s="1"/>
-      <c r="F259" s="1"/>
+      <c r="F259" s="1">
+        <v>210</v>
+      </c>
       <c r="G259" s="1"/>
       <c r="H259" s="6"/>
     </row>
@@ -6752,7 +6780,7 @@
         <v>26</v>
       </c>
       <c r="F260" s="1" t="s">
-        <v>26</v>
+        <v>190</v>
       </c>
       <c r="G260" s="1" t="s">
         <v>26</v>
@@ -6771,7 +6799,9 @@
       <c r="C261" s="1"/>
       <c r="D261" s="1"/>
       <c r="E261" s="1"/>
-      <c r="F261" s="1"/>
+      <c r="F261" s="1">
+        <v>240</v>
+      </c>
       <c r="G261" s="1"/>
       <c r="H261" s="1"/>
     </row>
@@ -6785,7 +6815,9 @@
       <c r="C262" s="1"/>
       <c r="D262" s="1"/>
       <c r="E262" s="1"/>
-      <c r="F262" s="1"/>
+      <c r="F262" s="1">
+        <v>3</v>
+      </c>
       <c r="G262" s="1"/>
       <c r="H262" s="1"/>
     </row>
@@ -6799,7 +6831,9 @@
       <c r="C263" s="1"/>
       <c r="D263" s="1"/>
       <c r="E263" s="1"/>
-      <c r="F263" s="1"/>
+      <c r="F263" s="1">
+        <v>1</v>
+      </c>
       <c r="G263" s="1"/>
       <c r="H263" s="1"/>
     </row>
@@ -6813,7 +6847,9 @@
       <c r="C264" s="1"/>
       <c r="D264" s="1"/>
       <c r="E264" s="1"/>
-      <c r="F264" s="1"/>
+      <c r="F264" s="1">
+        <v>4</v>
+      </c>
       <c r="G264" s="1"/>
       <c r="H264" s="1"/>
     </row>
@@ -6834,7 +6870,7 @@
         <v>26</v>
       </c>
       <c r="F265" s="1" t="s">
-        <v>26</v>
+        <v>191</v>
       </c>
       <c r="G265" s="1" t="s">
         <v>26</v>
@@ -6850,14 +6886,6 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="B159:H159"/>
-    <mergeCell ref="A59:H59"/>
-    <mergeCell ref="B102:H102"/>
-    <mergeCell ref="A138:H138"/>
-    <mergeCell ref="B139:H139"/>
-    <mergeCell ref="A101:H101"/>
-    <mergeCell ref="A79:H79"/>
-    <mergeCell ref="B80:H80"/>
     <mergeCell ref="B196:H196"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A60:H60"/>
@@ -6874,6 +6902,14 @@
     <mergeCell ref="B61:H61"/>
     <mergeCell ref="A119:H119"/>
     <mergeCell ref="B120:H120"/>
+    <mergeCell ref="B159:H159"/>
+    <mergeCell ref="A59:H59"/>
+    <mergeCell ref="B102:H102"/>
+    <mergeCell ref="A138:H138"/>
+    <mergeCell ref="B139:H139"/>
+    <mergeCell ref="A101:H101"/>
+    <mergeCell ref="A79:H79"/>
+    <mergeCell ref="B80:H80"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>

</xml_diff>

<commit_message>
vault backup: 2026-04-29 10:13:56
</commit_message>
<xml_diff>
--- a/睡眠日记_Sleep_Diary1.xlsx
+++ b/睡眠日记_Sleep_Diary1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My_like\My_like\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6952AF17-AF7E-4B2B-ABE4-D22C95FE7AC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A2A2EF5-7A59-481C-8942-7B40F0E7ABA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7095" yWindow="0" windowWidth="17085" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="睡眠日记 Sleep Diary" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="808" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="849" uniqueCount="195">
   <si>
     <t>睡眠日记 Sleep Diary</t>
   </si>
@@ -668,6 +668,15 @@
   </si>
   <si>
     <t>300 min</t>
+  </si>
+  <si>
+    <t>100 min</t>
+  </si>
+  <si>
+    <t>被猫挠门叫醒</t>
+  </si>
+  <si>
+    <t>每天六点起 10点睡 午休40 min</t>
   </si>
 </sst>
 </file>
@@ -677,7 +686,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="h:mm"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -715,6 +724,17 @@
       <b/>
       <sz val="11"/>
       <name val="微软雅黑"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -808,7 +828,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -865,6 +885,33 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="46" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1168,7 +1215,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H266"/>
+  <dimension ref="A1:H285"/>
   <sheetFormatPr defaultColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="8" width="20" customWidth="1"/>
@@ -6884,8 +6931,303 @@
         <v>187</v>
       </c>
     </row>
+    <row r="268" spans="1:8">
+      <c r="A268" s="5"/>
+      <c r="B268" s="21" t="s">
+        <v>147</v>
+      </c>
+      <c r="C268" s="22" t="s">
+        <v>148</v>
+      </c>
+      <c r="D268" s="22" t="s">
+        <v>149</v>
+      </c>
+      <c r="E268" s="22" t="s">
+        <v>150</v>
+      </c>
+      <c r="F268" s="22" t="s">
+        <v>151</v>
+      </c>
+      <c r="G268" s="22" t="s">
+        <v>152</v>
+      </c>
+      <c r="H268" s="23" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="269" spans="1:8" ht="18">
+      <c r="A269" s="2"/>
+      <c r="B269" s="11">
+        <v>46139</v>
+      </c>
+      <c r="C269" s="11">
+        <f>B269+1</f>
+        <v>46140</v>
+      </c>
+      <c r="D269" s="11">
+        <f t="shared" ref="D269" si="31">C269+1</f>
+        <v>46141</v>
+      </c>
+      <c r="E269" s="11">
+        <f t="shared" ref="E269" si="32">D269+1</f>
+        <v>46142</v>
+      </c>
+      <c r="F269" s="11">
+        <f t="shared" ref="F269" si="33">E269+1</f>
+        <v>46143</v>
+      </c>
+      <c r="G269" s="11">
+        <f t="shared" ref="G269" si="34">F269+1</f>
+        <v>46144</v>
+      </c>
+      <c r="H269" s="11">
+        <f t="shared" ref="H269" si="35">G269+1</f>
+        <v>46145</v>
+      </c>
+    </row>
+    <row r="270" spans="1:8" ht="30">
+      <c r="A270" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B270" s="24"/>
+      <c r="C270" s="25" t="s">
+        <v>178</v>
+      </c>
+      <c r="D270" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="E270" s="25"/>
+      <c r="F270" s="25"/>
+      <c r="G270" s="25"/>
+      <c r="H270" s="25"/>
+    </row>
+    <row r="271" spans="1:8">
+      <c r="A271" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B271" s="25"/>
+      <c r="C271" s="25"/>
+      <c r="D271" s="25" t="s">
+        <v>72</v>
+      </c>
+      <c r="E271" s="25"/>
+      <c r="F271" s="25"/>
+      <c r="G271" s="25"/>
+      <c r="H271" s="26"/>
+    </row>
+    <row r="272" spans="1:8">
+      <c r="A272" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B272" s="25"/>
+      <c r="C272" s="25"/>
+      <c r="D272" s="25" t="s">
+        <v>157</v>
+      </c>
+      <c r="E272" s="27"/>
+      <c r="F272" s="25"/>
+      <c r="G272" s="25"/>
+      <c r="H272" s="26"/>
+    </row>
+    <row r="273" spans="1:8">
+      <c r="A273" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B273" s="25"/>
+      <c r="C273" s="25"/>
+      <c r="D273" s="25" t="s">
+        <v>91</v>
+      </c>
+      <c r="E273" s="27"/>
+      <c r="F273" s="25"/>
+      <c r="G273" s="25"/>
+      <c r="H273" s="26"/>
+    </row>
+    <row r="274" spans="1:8" ht="45">
+      <c r="A274" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B274" s="25"/>
+      <c r="C274" s="5"/>
+      <c r="D274">
+        <v>0</v>
+      </c>
+      <c r="E274" s="5"/>
+      <c r="F274" s="5"/>
+      <c r="G274" s="5"/>
+      <c r="H274" s="5"/>
+    </row>
+    <row r="275" spans="1:8">
+      <c r="A275" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B275" s="5"/>
+      <c r="C275" s="5"/>
+      <c r="D275">
+        <v>1</v>
+      </c>
+      <c r="E275" s="5"/>
+      <c r="F275" s="28"/>
+      <c r="G275" s="5"/>
+      <c r="H275" s="5"/>
+    </row>
+    <row r="276" spans="1:8" ht="30">
+      <c r="A276" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B276" s="5"/>
+      <c r="C276" s="5"/>
+      <c r="D276" s="27" t="s">
+        <v>192</v>
+      </c>
+      <c r="E276" s="5"/>
+      <c r="F276" s="5"/>
+      <c r="G276" s="5"/>
+      <c r="H276" s="5"/>
+    </row>
+    <row r="277" spans="1:8" ht="30">
+      <c r="A277" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B277" s="5"/>
+      <c r="C277" s="5"/>
+      <c r="D277" s="5"/>
+      <c r="E277" s="5"/>
+      <c r="F277" s="5"/>
+      <c r="G277" s="5"/>
+      <c r="H277" s="25"/>
+    </row>
+    <row r="278" spans="1:8" ht="75">
+      <c r="A278" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B278" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C278" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D278" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E278" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F278" s="5"/>
+      <c r="G278" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="H278" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="279" spans="1:8" ht="60">
+      <c r="A279" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B279" s="5"/>
+      <c r="C279" s="5"/>
+      <c r="D279" s="5">
+        <v>10</v>
+      </c>
+      <c r="E279" s="5"/>
+      <c r="F279" s="5"/>
+      <c r="G279" s="5"/>
+      <c r="H279" s="5"/>
+    </row>
+    <row r="280" spans="1:8" ht="45">
+      <c r="A280" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B280" s="5"/>
+      <c r="C280" s="5"/>
+      <c r="D280" s="5">
+        <v>4</v>
+      </c>
+      <c r="E280" s="5"/>
+      <c r="F280" s="5"/>
+      <c r="G280" s="5"/>
+      <c r="H280" s="5"/>
+    </row>
+    <row r="281" spans="1:8" ht="90">
+      <c r="A281" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B281" s="5"/>
+      <c r="C281" s="5"/>
+      <c r="D281" s="5">
+        <v>3</v>
+      </c>
+      <c r="E281" s="5"/>
+      <c r="F281" s="5"/>
+      <c r="G281" s="5"/>
+      <c r="H281" s="5"/>
+    </row>
+    <row r="282" spans="1:8" ht="105">
+      <c r="A282" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B282" s="5"/>
+      <c r="C282" s="5"/>
+      <c r="D282" s="5">
+        <v>4</v>
+      </c>
+      <c r="E282" s="5"/>
+      <c r="F282" s="5"/>
+      <c r="G282" s="5"/>
+      <c r="H282" s="5"/>
+    </row>
+    <row r="283" spans="1:8" ht="60">
+      <c r="A283" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B283" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C283" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D283" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="E283" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F283" s="5"/>
+      <c r="G283" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="H283" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="284" spans="1:8">
+      <c r="A284" s="28"/>
+      <c r="B284" s="28"/>
+      <c r="C284" s="28"/>
+      <c r="D284" s="28" t="s">
+        <v>193</v>
+      </c>
+      <c r="E284" s="28"/>
+      <c r="F284" s="28"/>
+      <c r="G284" s="28"/>
+      <c r="H284" s="28"/>
+    </row>
+    <row r="285" spans="1:8">
+      <c r="D285" s="29" t="s">
+        <v>194</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="B159:H159"/>
+    <mergeCell ref="A59:H59"/>
+    <mergeCell ref="B102:H102"/>
+    <mergeCell ref="A138:H138"/>
+    <mergeCell ref="B139:H139"/>
+    <mergeCell ref="A101:H101"/>
+    <mergeCell ref="A79:H79"/>
+    <mergeCell ref="B80:H80"/>
     <mergeCell ref="B196:H196"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A60:H60"/>
@@ -6902,14 +7244,6 @@
     <mergeCell ref="B61:H61"/>
     <mergeCell ref="A119:H119"/>
     <mergeCell ref="B120:H120"/>
-    <mergeCell ref="B159:H159"/>
-    <mergeCell ref="A59:H59"/>
-    <mergeCell ref="B102:H102"/>
-    <mergeCell ref="A138:H138"/>
-    <mergeCell ref="B139:H139"/>
-    <mergeCell ref="A101:H101"/>
-    <mergeCell ref="A79:H79"/>
-    <mergeCell ref="B80:H80"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>

</xml_diff>

<commit_message>
vault backup: 2026-04-30 06:34:02
</commit_message>
<xml_diff>
--- a/睡眠日记_Sleep_Diary1.xlsx
+++ b/睡眠日记_Sleep_Diary1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My_like\My_like\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A2A2EF5-7A59-481C-8942-7B40F0E7ABA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B693C8D2-6FCB-4E47-8986-FE9A721986A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="睡眠日记 Sleep Diary" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="849" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="850" uniqueCount="196">
   <si>
     <t>睡眠日记 Sleep Diary</t>
   </si>
@@ -677,6 +677,9 @@
   </si>
   <si>
     <t>每天六点起 10点睡 午休40 min</t>
+  </si>
+  <si>
+    <t>睡觉手机不在卧室，早上听到闹钟来关，但是清醒了</t>
   </si>
 </sst>
 </file>
@@ -869,23 +872,6 @@
     <xf numFmtId="20" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -912,6 +898,23 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1222,42 +1225,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="22.5">
-      <c r="A1" s="17" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="19"/>
+      <c r="A1" s="26" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="28"/>
     </row>
     <row r="2" spans="1:8" ht="17.25">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="18"/>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-      <c r="H2" s="19"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="28"/>
     </row>
     <row r="3" spans="1:8" ht="16.5">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="15"/>
-      <c r="D3" s="15"/>
-      <c r="E3" s="15"/>
-      <c r="F3" s="15"/>
-      <c r="G3" s="15"/>
-      <c r="H3" s="16"/>
+      <c r="C3" s="24"/>
+      <c r="D3" s="24"/>
+      <c r="E3" s="24"/>
+      <c r="F3" s="24"/>
+      <c r="G3" s="24"/>
+      <c r="H3" s="25"/>
     </row>
     <row r="4" spans="1:8" ht="54">
       <c r="A4" s="2"/>
@@ -1651,42 +1654,42 @@
       <c r="A20" s="3"/>
     </row>
     <row r="21" spans="1:8" ht="22.5">
-      <c r="A21" s="17" t="s">
-        <v>0</v>
-      </c>
-      <c r="B21" s="18"/>
-      <c r="C21" s="18"/>
-      <c r="D21" s="18"/>
-      <c r="E21" s="18"/>
-      <c r="F21" s="18"/>
-      <c r="G21" s="18"/>
-      <c r="H21" s="19"/>
+      <c r="A21" s="26" t="s">
+        <v>0</v>
+      </c>
+      <c r="B21" s="27"/>
+      <c r="C21" s="27"/>
+      <c r="D21" s="27"/>
+      <c r="E21" s="27"/>
+      <c r="F21" s="27"/>
+      <c r="G21" s="27"/>
+      <c r="H21" s="28"/>
     </row>
     <row r="22" spans="1:8" ht="17.25">
-      <c r="A22" s="20" t="s">
+      <c r="A22" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="B22" s="18"/>
-      <c r="C22" s="18"/>
-      <c r="D22" s="18"/>
-      <c r="E22" s="18"/>
-      <c r="F22" s="18"/>
-      <c r="G22" s="18"/>
-      <c r="H22" s="19"/>
+      <c r="B22" s="27"/>
+      <c r="C22" s="27"/>
+      <c r="D22" s="27"/>
+      <c r="E22" s="27"/>
+      <c r="F22" s="27"/>
+      <c r="G22" s="27"/>
+      <c r="H22" s="28"/>
     </row>
     <row r="23" spans="1:8" ht="16.5">
       <c r="A23" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B23" s="14" t="s">
+      <c r="B23" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="C23" s="15"/>
-      <c r="D23" s="15"/>
-      <c r="E23" s="15"/>
-      <c r="F23" s="15"/>
-      <c r="G23" s="15"/>
-      <c r="H23" s="16"/>
+      <c r="C23" s="24"/>
+      <c r="D23" s="24"/>
+      <c r="E23" s="24"/>
+      <c r="F23" s="24"/>
+      <c r="G23" s="24"/>
+      <c r="H23" s="25"/>
     </row>
     <row r="24" spans="1:8" ht="54">
       <c r="A24" s="2"/>
@@ -2077,42 +2080,42 @@
       </c>
     </row>
     <row r="40" spans="1:8" ht="22.5">
-      <c r="A40" s="17" t="s">
-        <v>0</v>
-      </c>
-      <c r="B40" s="18"/>
-      <c r="C40" s="18"/>
-      <c r="D40" s="18"/>
-      <c r="E40" s="18"/>
-      <c r="F40" s="18"/>
-      <c r="G40" s="18"/>
-      <c r="H40" s="19"/>
+      <c r="A40" s="26" t="s">
+        <v>0</v>
+      </c>
+      <c r="B40" s="27"/>
+      <c r="C40" s="27"/>
+      <c r="D40" s="27"/>
+      <c r="E40" s="27"/>
+      <c r="F40" s="27"/>
+      <c r="G40" s="27"/>
+      <c r="H40" s="28"/>
     </row>
     <row r="41" spans="1:8" ht="17.25">
-      <c r="A41" s="20" t="s">
+      <c r="A41" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="B41" s="18"/>
-      <c r="C41" s="18"/>
-      <c r="D41" s="18"/>
-      <c r="E41" s="18"/>
-      <c r="F41" s="18"/>
-      <c r="G41" s="18"/>
-      <c r="H41" s="19"/>
+      <c r="B41" s="27"/>
+      <c r="C41" s="27"/>
+      <c r="D41" s="27"/>
+      <c r="E41" s="27"/>
+      <c r="F41" s="27"/>
+      <c r="G41" s="27"/>
+      <c r="H41" s="28"/>
     </row>
     <row r="42" spans="1:8" ht="16.5">
       <c r="A42" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B42" s="14" t="s">
+      <c r="B42" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="C42" s="15"/>
-      <c r="D42" s="15"/>
-      <c r="E42" s="15"/>
-      <c r="F42" s="15"/>
-      <c r="G42" s="15"/>
-      <c r="H42" s="16"/>
+      <c r="C42" s="24"/>
+      <c r="D42" s="24"/>
+      <c r="E42" s="24"/>
+      <c r="F42" s="24"/>
+      <c r="G42" s="24"/>
+      <c r="H42" s="25"/>
     </row>
     <row r="43" spans="1:8" ht="54">
       <c r="A43" s="2"/>
@@ -2503,42 +2506,42 @@
       </c>
     </row>
     <row r="59" spans="1:8" ht="22.5">
-      <c r="A59" s="17" t="s">
-        <v>0</v>
-      </c>
-      <c r="B59" s="18"/>
-      <c r="C59" s="18"/>
-      <c r="D59" s="18"/>
-      <c r="E59" s="18"/>
-      <c r="F59" s="18"/>
-      <c r="G59" s="18"/>
-      <c r="H59" s="19"/>
+      <c r="A59" s="26" t="s">
+        <v>0</v>
+      </c>
+      <c r="B59" s="27"/>
+      <c r="C59" s="27"/>
+      <c r="D59" s="27"/>
+      <c r="E59" s="27"/>
+      <c r="F59" s="27"/>
+      <c r="G59" s="27"/>
+      <c r="H59" s="28"/>
     </row>
     <row r="60" spans="1:8" ht="17.25">
-      <c r="A60" s="20" t="s">
+      <c r="A60" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="B60" s="18"/>
-      <c r="C60" s="18"/>
-      <c r="D60" s="18"/>
-      <c r="E60" s="18"/>
-      <c r="F60" s="18"/>
-      <c r="G60" s="18"/>
-      <c r="H60" s="19"/>
+      <c r="B60" s="27"/>
+      <c r="C60" s="27"/>
+      <c r="D60" s="27"/>
+      <c r="E60" s="27"/>
+      <c r="F60" s="27"/>
+      <c r="G60" s="27"/>
+      <c r="H60" s="28"/>
     </row>
     <row r="61" spans="1:8" ht="16.5">
       <c r="A61" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B61" s="14" t="s">
+      <c r="B61" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="C61" s="15"/>
-      <c r="D61" s="15"/>
-      <c r="E61" s="15"/>
-      <c r="F61" s="15"/>
-      <c r="G61" s="15"/>
-      <c r="H61" s="16"/>
+      <c r="C61" s="24"/>
+      <c r="D61" s="24"/>
+      <c r="E61" s="24"/>
+      <c r="F61" s="24"/>
+      <c r="G61" s="24"/>
+      <c r="H61" s="25"/>
     </row>
     <row r="62" spans="1:8" ht="54">
       <c r="A62" s="2"/>
@@ -2929,30 +2932,30 @@
       </c>
     </row>
     <row r="79" spans="1:8" ht="17.25">
-      <c r="A79" s="20" t="s">
+      <c r="A79" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="B79" s="18"/>
-      <c r="C79" s="18"/>
-      <c r="D79" s="18"/>
-      <c r="E79" s="18"/>
-      <c r="F79" s="18"/>
-      <c r="G79" s="18"/>
-      <c r="H79" s="19"/>
+      <c r="B79" s="27"/>
+      <c r="C79" s="27"/>
+      <c r="D79" s="27"/>
+      <c r="E79" s="27"/>
+      <c r="F79" s="27"/>
+      <c r="G79" s="27"/>
+      <c r="H79" s="28"/>
     </row>
     <row r="80" spans="1:8" ht="16.5">
       <c r="A80" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B80" s="14" t="s">
+      <c r="B80" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="C80" s="15"/>
-      <c r="D80" s="15"/>
-      <c r="E80" s="15"/>
-      <c r="F80" s="15"/>
-      <c r="G80" s="15"/>
-      <c r="H80" s="16"/>
+      <c r="C80" s="24"/>
+      <c r="D80" s="24"/>
+      <c r="E80" s="24"/>
+      <c r="F80" s="24"/>
+      <c r="G80" s="24"/>
+      <c r="H80" s="25"/>
     </row>
     <row r="81" spans="1:8" ht="54">
       <c r="A81" s="2"/>
@@ -3348,30 +3351,30 @@
       </c>
     </row>
     <row r="101" spans="1:8" ht="17.25">
-      <c r="A101" s="20" t="s">
+      <c r="A101" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="B101" s="18"/>
-      <c r="C101" s="18"/>
-      <c r="D101" s="18"/>
-      <c r="E101" s="18"/>
-      <c r="F101" s="18"/>
-      <c r="G101" s="18"/>
-      <c r="H101" s="19"/>
+      <c r="B101" s="27"/>
+      <c r="C101" s="27"/>
+      <c r="D101" s="27"/>
+      <c r="E101" s="27"/>
+      <c r="F101" s="27"/>
+      <c r="G101" s="27"/>
+      <c r="H101" s="28"/>
     </row>
     <row r="102" spans="1:8" ht="16.5">
       <c r="A102" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B102" s="14" t="s">
+      <c r="B102" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="C102" s="15"/>
-      <c r="D102" s="15"/>
-      <c r="E102" s="15"/>
-      <c r="F102" s="15"/>
-      <c r="G102" s="15"/>
-      <c r="H102" s="16"/>
+      <c r="C102" s="24"/>
+      <c r="D102" s="24"/>
+      <c r="E102" s="24"/>
+      <c r="F102" s="24"/>
+      <c r="G102" s="24"/>
+      <c r="H102" s="25"/>
     </row>
     <row r="103" spans="1:8" ht="54">
       <c r="A103" s="2"/>
@@ -3762,30 +3765,30 @@
       </c>
     </row>
     <row r="119" spans="1:8" ht="17.25">
-      <c r="A119" s="20" t="s">
+      <c r="A119" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="B119" s="18"/>
-      <c r="C119" s="18"/>
-      <c r="D119" s="18"/>
-      <c r="E119" s="18"/>
-      <c r="F119" s="18"/>
-      <c r="G119" s="18"/>
-      <c r="H119" s="19"/>
+      <c r="B119" s="27"/>
+      <c r="C119" s="27"/>
+      <c r="D119" s="27"/>
+      <c r="E119" s="27"/>
+      <c r="F119" s="27"/>
+      <c r="G119" s="27"/>
+      <c r="H119" s="28"/>
     </row>
     <row r="120" spans="1:8" ht="16.5">
       <c r="A120" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B120" s="14" t="s">
+      <c r="B120" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="C120" s="15"/>
-      <c r="D120" s="15"/>
-      <c r="E120" s="15"/>
-      <c r="F120" s="15"/>
-      <c r="G120" s="15"/>
-      <c r="H120" s="16"/>
+      <c r="C120" s="24"/>
+      <c r="D120" s="24"/>
+      <c r="E120" s="24"/>
+      <c r="F120" s="24"/>
+      <c r="G120" s="24"/>
+      <c r="H120" s="25"/>
     </row>
     <row r="121" spans="1:8" ht="36">
       <c r="A121" s="2"/>
@@ -4176,30 +4179,30 @@
       </c>
     </row>
     <row r="138" spans="1:8" ht="17.25">
-      <c r="A138" s="20" t="s">
+      <c r="A138" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="B138" s="18"/>
-      <c r="C138" s="18"/>
-      <c r="D138" s="18"/>
-      <c r="E138" s="18"/>
-      <c r="F138" s="18"/>
-      <c r="G138" s="18"/>
-      <c r="H138" s="19"/>
+      <c r="B138" s="27"/>
+      <c r="C138" s="27"/>
+      <c r="D138" s="27"/>
+      <c r="E138" s="27"/>
+      <c r="F138" s="27"/>
+      <c r="G138" s="27"/>
+      <c r="H138" s="28"/>
     </row>
     <row r="139" spans="1:8" ht="16.5">
       <c r="A139" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B139" s="14" t="s">
+      <c r="B139" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="C139" s="15"/>
-      <c r="D139" s="15"/>
-      <c r="E139" s="15"/>
-      <c r="F139" s="15"/>
-      <c r="G139" s="15"/>
-      <c r="H139" s="16"/>
+      <c r="C139" s="24"/>
+      <c r="D139" s="24"/>
+      <c r="E139" s="24"/>
+      <c r="F139" s="24"/>
+      <c r="G139" s="24"/>
+      <c r="H139" s="25"/>
     </row>
     <row r="140" spans="1:8" ht="16.5">
       <c r="A140" s="1"/>
@@ -4625,30 +4628,30 @@
       </c>
     </row>
     <row r="158" spans="1:8" ht="17.25">
-      <c r="A158" s="20" t="s">
+      <c r="A158" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="B158" s="18"/>
-      <c r="C158" s="18"/>
-      <c r="D158" s="18"/>
-      <c r="E158" s="18"/>
-      <c r="F158" s="18"/>
-      <c r="G158" s="18"/>
-      <c r="H158" s="19"/>
+      <c r="B158" s="27"/>
+      <c r="C158" s="27"/>
+      <c r="D158" s="27"/>
+      <c r="E158" s="27"/>
+      <c r="F158" s="27"/>
+      <c r="G158" s="27"/>
+      <c r="H158" s="28"/>
     </row>
     <row r="159" spans="1:8" ht="16.5">
       <c r="A159" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B159" s="14" t="s">
+      <c r="B159" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="C159" s="15"/>
-      <c r="D159" s="15"/>
-      <c r="E159" s="15"/>
-      <c r="F159" s="15"/>
-      <c r="G159" s="15"/>
-      <c r="H159" s="16"/>
+      <c r="C159" s="24"/>
+      <c r="D159" s="24"/>
+      <c r="E159" s="24"/>
+      <c r="F159" s="24"/>
+      <c r="G159" s="24"/>
+      <c r="H159" s="25"/>
     </row>
     <row r="160" spans="1:8" ht="16.5">
       <c r="A160" s="1"/>
@@ -5072,15 +5075,15 @@
       <c r="A177" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B177" s="14" t="s">
+      <c r="B177" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="C177" s="15"/>
-      <c r="D177" s="15"/>
-      <c r="E177" s="15"/>
-      <c r="F177" s="15"/>
-      <c r="G177" s="15"/>
-      <c r="H177" s="16"/>
+      <c r="C177" s="24"/>
+      <c r="D177" s="24"/>
+      <c r="E177" s="24"/>
+      <c r="F177" s="24"/>
+      <c r="G177" s="24"/>
+      <c r="H177" s="25"/>
     </row>
     <row r="178" spans="1:8" ht="16.5">
       <c r="A178" s="1"/>
@@ -5470,15 +5473,15 @@
       <c r="A196" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B196" s="14" t="s">
+      <c r="B196" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="C196" s="15"/>
-      <c r="D196" s="15"/>
-      <c r="E196" s="15"/>
-      <c r="F196" s="15"/>
-      <c r="G196" s="15"/>
-      <c r="H196" s="16"/>
+      <c r="C196" s="24"/>
+      <c r="D196" s="24"/>
+      <c r="E196" s="24"/>
+      <c r="F196" s="24"/>
+      <c r="G196" s="24"/>
+      <c r="H196" s="25"/>
     </row>
     <row r="197" spans="1:8" ht="16.5">
       <c r="A197" s="1"/>
@@ -6933,25 +6936,25 @@
     </row>
     <row r="268" spans="1:8">
       <c r="A268" s="5"/>
-      <c r="B268" s="21" t="s">
+      <c r="B268" s="14" t="s">
         <v>147</v>
       </c>
-      <c r="C268" s="22" t="s">
+      <c r="C268" s="15" t="s">
         <v>148</v>
       </c>
-      <c r="D268" s="22" t="s">
+      <c r="D268" s="15" t="s">
         <v>149</v>
       </c>
-      <c r="E268" s="22" t="s">
+      <c r="E268" s="15" t="s">
         <v>150</v>
       </c>
-      <c r="F268" s="22" t="s">
+      <c r="F268" s="15" t="s">
         <v>151</v>
       </c>
-      <c r="G268" s="22" t="s">
+      <c r="G268" s="15" t="s">
         <v>152</v>
       </c>
-      <c r="H268" s="23" t="s">
+      <c r="H268" s="16" t="s">
         <v>153</v>
       </c>
     </row>
@@ -6989,70 +6992,80 @@
       <c r="A270" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B270" s="24"/>
-      <c r="C270" s="25" t="s">
+      <c r="B270" s="17"/>
+      <c r="C270" s="18" t="s">
         <v>178</v>
       </c>
-      <c r="D270" s="25" t="s">
+      <c r="D270" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="E270" s="25"/>
-      <c r="F270" s="25"/>
-      <c r="G270" s="25"/>
-      <c r="H270" s="25"/>
+      <c r="E270" s="18">
+        <v>0.25347222222222221</v>
+      </c>
+      <c r="F270" s="18"/>
+      <c r="G270" s="18"/>
+      <c r="H270" s="18"/>
     </row>
     <row r="271" spans="1:8">
       <c r="A271" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B271" s="25"/>
-      <c r="C271" s="25"/>
-      <c r="D271" s="25" t="s">
+      <c r="B271" s="18"/>
+      <c r="C271" s="18"/>
+      <c r="D271" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="E271" s="25"/>
-      <c r="F271" s="25"/>
-      <c r="G271" s="25"/>
-      <c r="H271" s="26"/>
+      <c r="E271" s="18">
+        <v>0.25347222222222221</v>
+      </c>
+      <c r="F271" s="18"/>
+      <c r="G271" s="18"/>
+      <c r="H271" s="19"/>
     </row>
     <row r="272" spans="1:8">
       <c r="A272" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B272" s="25"/>
-      <c r="C272" s="25"/>
-      <c r="D272" s="25" t="s">
+      <c r="B272" s="18"/>
+      <c r="C272" s="18"/>
+      <c r="D272" s="18" t="s">
         <v>157</v>
       </c>
-      <c r="E272" s="27"/>
-      <c r="F272" s="25"/>
-      <c r="G272" s="25"/>
-      <c r="H272" s="26"/>
+      <c r="E272" s="20">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="F272" s="18"/>
+      <c r="G272" s="18"/>
+      <c r="H272" s="19"/>
     </row>
     <row r="273" spans="1:8">
       <c r="A273" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B273" s="25"/>
-      <c r="C273" s="25"/>
-      <c r="D273" s="25" t="s">
+      <c r="B273" s="18"/>
+      <c r="C273" s="18"/>
+      <c r="D273" s="18" t="s">
         <v>91</v>
       </c>
-      <c r="E273" s="27"/>
-      <c r="F273" s="25"/>
-      <c r="G273" s="25"/>
-      <c r="H273" s="26"/>
+      <c r="E273" s="20">
+        <v>0.9375</v>
+      </c>
+      <c r="F273" s="18"/>
+      <c r="G273" s="18"/>
+      <c r="H273" s="19"/>
     </row>
     <row r="274" spans="1:8" ht="45">
       <c r="A274" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B274" s="25"/>
+      <c r="B274" s="18"/>
       <c r="C274" s="5"/>
       <c r="D274">
         <v>0</v>
       </c>
-      <c r="E274" s="5"/>
+      <c r="E274" s="5">
+        <v>0</v>
+      </c>
       <c r="F274" s="5"/>
       <c r="G274" s="5"/>
       <c r="H274" s="5"/>
@@ -7066,8 +7079,10 @@
       <c r="D275">
         <v>1</v>
       </c>
-      <c r="E275" s="5"/>
-      <c r="F275" s="28"/>
+      <c r="E275" s="5">
+        <v>0</v>
+      </c>
+      <c r="F275" s="21"/>
       <c r="G275" s="5"/>
       <c r="H275" s="5"/>
     </row>
@@ -7077,10 +7092,12 @@
       </c>
       <c r="B276" s="5"/>
       <c r="C276" s="5"/>
-      <c r="D276" s="27" t="s">
+      <c r="D276" s="20" t="s">
         <v>192</v>
       </c>
-      <c r="E276" s="5"/>
+      <c r="E276" s="5">
+        <v>0</v>
+      </c>
       <c r="F276" s="5"/>
       <c r="G276" s="5"/>
       <c r="H276" s="5"/>
@@ -7091,11 +7108,15 @@
       </c>
       <c r="B277" s="5"/>
       <c r="C277" s="5"/>
-      <c r="D277" s="5"/>
-      <c r="E277" s="5"/>
+      <c r="D277" s="5">
+        <v>470</v>
+      </c>
+      <c r="E277" s="5">
+        <v>450</v>
+      </c>
       <c r="F277" s="5"/>
       <c r="G277" s="5"/>
-      <c r="H277" s="25"/>
+      <c r="H277" s="18"/>
     </row>
     <row r="278" spans="1:8" ht="75">
       <c r="A278" s="5" t="s">
@@ -7130,7 +7151,9 @@
       <c r="D279" s="5">
         <v>10</v>
       </c>
-      <c r="E279" s="5"/>
+      <c r="E279" s="5">
+        <v>0</v>
+      </c>
       <c r="F279" s="5"/>
       <c r="G279" s="5"/>
       <c r="H279" s="5"/>
@@ -7144,7 +7167,9 @@
       <c r="D280" s="5">
         <v>4</v>
       </c>
-      <c r="E280" s="5"/>
+      <c r="E280" s="5">
+        <v>4</v>
+      </c>
       <c r="F280" s="5"/>
       <c r="G280" s="5"/>
       <c r="H280" s="5"/>
@@ -7158,8 +7183,12 @@
       <c r="D281" s="5">
         <v>3</v>
       </c>
-      <c r="E281" s="5"/>
-      <c r="F281" s="5"/>
+      <c r="E281" s="5">
+        <v>4</v>
+      </c>
+      <c r="F281" s="5">
+        <v>0</v>
+      </c>
       <c r="G281" s="5"/>
       <c r="H281" s="5"/>
     </row>
@@ -7172,7 +7201,9 @@
       <c r="D282" s="5">
         <v>4</v>
       </c>
-      <c r="E282" s="5"/>
+      <c r="E282" s="5">
+        <v>4</v>
+      </c>
       <c r="F282" s="5"/>
       <c r="G282" s="5"/>
       <c r="H282" s="5"/>
@@ -7202,32 +7233,26 @@
       </c>
     </row>
     <row r="284" spans="1:8">
-      <c r="A284" s="28"/>
-      <c r="B284" s="28"/>
-      <c r="C284" s="28"/>
-      <c r="D284" s="28" t="s">
+      <c r="A284" s="21"/>
+      <c r="B284" s="21"/>
+      <c r="C284" s="21"/>
+      <c r="D284" s="21" t="s">
         <v>193</v>
       </c>
-      <c r="E284" s="28"/>
-      <c r="F284" s="28"/>
-      <c r="G284" s="28"/>
-      <c r="H284" s="28"/>
+      <c r="E284" s="21" t="s">
+        <v>195</v>
+      </c>
+      <c r="F284" s="21"/>
+      <c r="G284" s="21"/>
+      <c r="H284" s="21"/>
     </row>
     <row r="285" spans="1:8">
-      <c r="D285" s="29" t="s">
+      <c r="D285" s="22" t="s">
         <v>194</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="B159:H159"/>
-    <mergeCell ref="A59:H59"/>
-    <mergeCell ref="B102:H102"/>
-    <mergeCell ref="A138:H138"/>
-    <mergeCell ref="B139:H139"/>
-    <mergeCell ref="A101:H101"/>
-    <mergeCell ref="A79:H79"/>
-    <mergeCell ref="B80:H80"/>
     <mergeCell ref="B196:H196"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A60:H60"/>
@@ -7244,6 +7269,14 @@
     <mergeCell ref="B61:H61"/>
     <mergeCell ref="A119:H119"/>
     <mergeCell ref="B120:H120"/>
+    <mergeCell ref="B159:H159"/>
+    <mergeCell ref="A59:H59"/>
+    <mergeCell ref="B102:H102"/>
+    <mergeCell ref="A138:H138"/>
+    <mergeCell ref="B139:H139"/>
+    <mergeCell ref="A101:H101"/>
+    <mergeCell ref="A79:H79"/>
+    <mergeCell ref="B80:H80"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>

</xml_diff>

<commit_message>
vault backup: 2026-05-01 06:38:40
</commit_message>
<xml_diff>
--- a/睡眠日记_Sleep_Diary1.xlsx
+++ b/睡眠日记_Sleep_Diary1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My_like\My_like\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B693C8D2-6FCB-4E47-8986-FE9A721986A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2537E963-C1A0-4B6B-B488-5C02489D5E65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="睡眠日记 Sleep Diary" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="850" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="857" uniqueCount="199">
   <si>
     <t>睡眠日记 Sleep Diary</t>
   </si>
@@ -680,6 +680,15 @@
   </si>
   <si>
     <t>睡觉手机不在卧室，早上听到闹钟来关，但是清醒了</t>
+  </si>
+  <si>
+    <t>6：01</t>
+  </si>
+  <si>
+    <t>22：05</t>
+  </si>
+  <si>
+    <t>一觉睡到天亮</t>
   </si>
 </sst>
 </file>
@@ -7002,7 +7011,9 @@
       <c r="E270" s="18">
         <v>0.25347222222222221</v>
       </c>
-      <c r="F270" s="18"/>
+      <c r="F270" s="18" t="s">
+        <v>196</v>
+      </c>
       <c r="G270" s="18"/>
       <c r="H270" s="18"/>
     </row>
@@ -7018,7 +7029,9 @@
       <c r="E271" s="18">
         <v>0.25347222222222221</v>
       </c>
-      <c r="F271" s="18"/>
+      <c r="F271" s="18" t="s">
+        <v>196</v>
+      </c>
       <c r="G271" s="18"/>
       <c r="H271" s="19"/>
     </row>
@@ -7034,7 +7047,9 @@
       <c r="E272" s="20">
         <v>0.91666666666666663</v>
       </c>
-      <c r="F272" s="18"/>
+      <c r="F272" s="18" t="s">
+        <v>197</v>
+      </c>
       <c r="G272" s="18"/>
       <c r="H272" s="19"/>
     </row>
@@ -7050,7 +7065,9 @@
       <c r="E273" s="20">
         <v>0.9375</v>
       </c>
-      <c r="F273" s="18"/>
+      <c r="F273" s="18" t="s">
+        <v>91</v>
+      </c>
       <c r="G273" s="18"/>
       <c r="H273" s="19"/>
     </row>
@@ -7066,7 +7083,9 @@
       <c r="E274" s="5">
         <v>0</v>
       </c>
-      <c r="F274" s="5"/>
+      <c r="F274" s="5">
+        <v>0</v>
+      </c>
       <c r="G274" s="5"/>
       <c r="H274" s="5"/>
     </row>
@@ -7082,7 +7101,9 @@
       <c r="E275" s="5">
         <v>0</v>
       </c>
-      <c r="F275" s="21"/>
+      <c r="F275" s="21">
+        <v>0</v>
+      </c>
       <c r="G275" s="5"/>
       <c r="H275" s="5"/>
     </row>
@@ -7098,7 +7119,9 @@
       <c r="E276" s="5">
         <v>0</v>
       </c>
-      <c r="F276" s="5"/>
+      <c r="F276" s="5">
+        <v>0</v>
+      </c>
       <c r="G276" s="5"/>
       <c r="H276" s="5"/>
     </row>
@@ -7114,7 +7137,9 @@
       <c r="E277" s="5">
         <v>450</v>
       </c>
-      <c r="F277" s="5"/>
+      <c r="F277" s="5">
+        <v>450</v>
+      </c>
       <c r="G277" s="5"/>
       <c r="H277" s="18"/>
     </row>
@@ -7134,7 +7159,9 @@
       <c r="E278" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="F278" s="5"/>
+      <c r="F278" s="5" t="s">
+        <v>26</v>
+      </c>
       <c r="G278" s="5" t="s">
         <v>26</v>
       </c>
@@ -7154,7 +7181,9 @@
       <c r="E279" s="5">
         <v>0</v>
       </c>
-      <c r="F279" s="5"/>
+      <c r="F279" s="5">
+        <v>0</v>
+      </c>
       <c r="G279" s="5"/>
       <c r="H279" s="5"/>
     </row>
@@ -7170,7 +7199,9 @@
       <c r="E280" s="5">
         <v>4</v>
       </c>
-      <c r="F280" s="5"/>
+      <c r="F280" s="5">
+        <v>4</v>
+      </c>
       <c r="G280" s="5"/>
       <c r="H280" s="5"/>
     </row>
@@ -7187,7 +7218,7 @@
         <v>4</v>
       </c>
       <c r="F281" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G281" s="5"/>
       <c r="H281" s="5"/>
@@ -7204,7 +7235,9 @@
       <c r="E282" s="5">
         <v>4</v>
       </c>
-      <c r="F282" s="5"/>
+      <c r="F282" s="5">
+        <v>3</v>
+      </c>
       <c r="G282" s="5"/>
       <c r="H282" s="5"/>
     </row>
@@ -7224,7 +7257,9 @@
       <c r="E283" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="F283" s="5"/>
+      <c r="F283" s="5" t="s">
+        <v>141</v>
+      </c>
       <c r="G283" s="5" t="s">
         <v>26</v>
       </c>
@@ -7242,7 +7277,9 @@
       <c r="E284" s="21" t="s">
         <v>195</v>
       </c>
-      <c r="F284" s="21"/>
+      <c r="F284" s="21" t="s">
+        <v>198</v>
+      </c>
       <c r="G284" s="21"/>
       <c r="H284" s="21"/>
     </row>
@@ -7253,6 +7290,14 @@
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="B159:H159"/>
+    <mergeCell ref="A59:H59"/>
+    <mergeCell ref="B102:H102"/>
+    <mergeCell ref="A138:H138"/>
+    <mergeCell ref="B139:H139"/>
+    <mergeCell ref="A101:H101"/>
+    <mergeCell ref="A79:H79"/>
+    <mergeCell ref="B80:H80"/>
     <mergeCell ref="B196:H196"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A60:H60"/>
@@ -7269,14 +7314,6 @@
     <mergeCell ref="B61:H61"/>
     <mergeCell ref="A119:H119"/>
     <mergeCell ref="B120:H120"/>
-    <mergeCell ref="B159:H159"/>
-    <mergeCell ref="A59:H59"/>
-    <mergeCell ref="B102:H102"/>
-    <mergeCell ref="A138:H138"/>
-    <mergeCell ref="B139:H139"/>
-    <mergeCell ref="A101:H101"/>
-    <mergeCell ref="A79:H79"/>
-    <mergeCell ref="B80:H80"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>

</xml_diff>

<commit_message>
vault backup: 2026-05-02 07:59:24
</commit_message>
<xml_diff>
--- a/睡眠日记_Sleep_Diary1.xlsx
+++ b/睡眠日记_Sleep_Diary1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My_like\My_like\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2537E963-C1A0-4B6B-B488-5C02489D5E65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52DC1D08-C3BD-40BB-B596-D153BA1A2FA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="857" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="863" uniqueCount="203">
   <si>
     <t>睡眠日记 Sleep Diary</t>
   </si>
@@ -689,6 +689,18 @@
   </si>
   <si>
     <t>一觉睡到天亮</t>
+  </si>
+  <si>
+    <t>6：03</t>
+  </si>
+  <si>
+    <t>15 min</t>
+  </si>
+  <si>
+    <t>昨日睡前脑子里在想最近的事情</t>
+  </si>
+  <si>
+    <t>我发现半睡半醒之间，人会陷入潜意识</t>
   </si>
 </sst>
 </file>
@@ -7014,7 +7026,9 @@
       <c r="F270" s="18" t="s">
         <v>196</v>
       </c>
-      <c r="G270" s="18"/>
+      <c r="G270" s="18" t="s">
+        <v>178</v>
+      </c>
       <c r="H270" s="18"/>
     </row>
     <row r="271" spans="1:8">
@@ -7032,7 +7046,9 @@
       <c r="F271" s="18" t="s">
         <v>196</v>
       </c>
-      <c r="G271" s="18"/>
+      <c r="G271" s="18" t="s">
+        <v>199</v>
+      </c>
       <c r="H271" s="19"/>
     </row>
     <row r="272" spans="1:8">
@@ -7050,7 +7066,9 @@
       <c r="F272" s="18" t="s">
         <v>197</v>
       </c>
-      <c r="G272" s="18"/>
+      <c r="G272" s="18" t="s">
+        <v>64</v>
+      </c>
       <c r="H272" s="19"/>
     </row>
     <row r="273" spans="1:8">
@@ -7068,7 +7086,9 @@
       <c r="F273" s="18" t="s">
         <v>91</v>
       </c>
-      <c r="G273" s="18"/>
+      <c r="G273" s="18" t="s">
+        <v>91</v>
+      </c>
       <c r="H273" s="19"/>
     </row>
     <row r="274" spans="1:8" ht="45">
@@ -7086,7 +7106,9 @@
       <c r="F274" s="5">
         <v>0</v>
       </c>
-      <c r="G274" s="5"/>
+      <c r="G274" s="5">
+        <v>3</v>
+      </c>
       <c r="H274" s="5"/>
     </row>
     <row r="275" spans="1:8">
@@ -7104,7 +7126,9 @@
       <c r="F275" s="21">
         <v>0</v>
       </c>
-      <c r="G275" s="5"/>
+      <c r="G275" s="5">
+        <v>1</v>
+      </c>
       <c r="H275" s="5"/>
     </row>
     <row r="276" spans="1:8" ht="30">
@@ -7122,7 +7146,9 @@
       <c r="F276" s="5">
         <v>0</v>
       </c>
-      <c r="G276" s="5"/>
+      <c r="G276" s="5">
+        <v>10</v>
+      </c>
       <c r="H276" s="5"/>
     </row>
     <row r="277" spans="1:8" ht="30">
@@ -7140,7 +7166,9 @@
       <c r="F277" s="5">
         <v>450</v>
       </c>
-      <c r="G277" s="5"/>
+      <c r="G277" s="5">
+        <v>440</v>
+      </c>
       <c r="H277" s="18"/>
     </row>
     <row r="278" spans="1:8" ht="75">
@@ -7184,7 +7212,9 @@
       <c r="F279" s="5">
         <v>0</v>
       </c>
-      <c r="G279" s="5"/>
+      <c r="G279" s="5">
+        <v>0</v>
+      </c>
       <c r="H279" s="5"/>
     </row>
     <row r="280" spans="1:8" ht="45">
@@ -7202,7 +7232,9 @@
       <c r="F280" s="5">
         <v>4</v>
       </c>
-      <c r="G280" s="5"/>
+      <c r="G280" s="5">
+        <v>4</v>
+      </c>
       <c r="H280" s="5"/>
     </row>
     <row r="281" spans="1:8" ht="90">
@@ -7220,7 +7252,9 @@
       <c r="F281" s="5">
         <v>4</v>
       </c>
-      <c r="G281" s="5"/>
+      <c r="G281" s="5">
+        <v>4</v>
+      </c>
       <c r="H281" s="5"/>
     </row>
     <row r="282" spans="1:8" ht="105">
@@ -7238,7 +7272,9 @@
       <c r="F282" s="5">
         <v>3</v>
       </c>
-      <c r="G282" s="5"/>
+      <c r="G282" s="5">
+        <v>3</v>
+      </c>
       <c r="H282" s="5"/>
     </row>
     <row r="283" spans="1:8" ht="60">
@@ -7261,7 +7297,7 @@
         <v>141</v>
       </c>
       <c r="G283" s="5" t="s">
-        <v>26</v>
+        <v>200</v>
       </c>
       <c r="H283" s="5" t="s">
         <v>26</v>
@@ -7280,24 +7316,21 @@
       <c r="F284" s="21" t="s">
         <v>198</v>
       </c>
-      <c r="G284" s="21"/>
+      <c r="G284" s="21" t="s">
+        <v>201</v>
+      </c>
       <c r="H284" s="21"/>
     </row>
     <row r="285" spans="1:8">
       <c r="D285" s="22" t="s">
         <v>194</v>
       </c>
+      <c r="G285" t="s">
+        <v>202</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="B159:H159"/>
-    <mergeCell ref="A59:H59"/>
-    <mergeCell ref="B102:H102"/>
-    <mergeCell ref="A138:H138"/>
-    <mergeCell ref="B139:H139"/>
-    <mergeCell ref="A101:H101"/>
-    <mergeCell ref="A79:H79"/>
-    <mergeCell ref="B80:H80"/>
     <mergeCell ref="B196:H196"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A60:H60"/>
@@ -7314,6 +7347,14 @@
     <mergeCell ref="B61:H61"/>
     <mergeCell ref="A119:H119"/>
     <mergeCell ref="B120:H120"/>
+    <mergeCell ref="B159:H159"/>
+    <mergeCell ref="A59:H59"/>
+    <mergeCell ref="B102:H102"/>
+    <mergeCell ref="A138:H138"/>
+    <mergeCell ref="B139:H139"/>
+    <mergeCell ref="A101:H101"/>
+    <mergeCell ref="A79:H79"/>
+    <mergeCell ref="B80:H80"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>

</xml_diff>

<commit_message>
vault backup: 2026-05-05 12:05:57
</commit_message>
<xml_diff>
--- a/睡眠日记_Sleep_Diary1.xlsx
+++ b/睡眠日记_Sleep_Diary1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My_like\My_like\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52DC1D08-C3BD-40BB-B596-D153BA1A2FA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DED28C9E-DEAC-48D2-8BC7-F4539B6639F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="863" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="904" uniqueCount="206">
   <si>
     <t>睡眠日记 Sleep Diary</t>
   </si>
@@ -701,6 +701,15 @@
   </si>
   <si>
     <t>我发现半睡半醒之间，人会陷入潜意识</t>
+  </si>
+  <si>
+    <t>30 min</t>
+  </si>
+  <si>
+    <t>6：02</t>
+  </si>
+  <si>
+    <t>90min</t>
   </si>
 </sst>
 </file>
@@ -1239,7 +1248,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H285"/>
+  <dimension ref="A1:H301"/>
   <sheetFormatPr defaultColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="8" width="20" customWidth="1"/>
@@ -7029,7 +7038,9 @@
       <c r="G270" s="18" t="s">
         <v>178</v>
       </c>
-      <c r="H270" s="18"/>
+      <c r="H270" s="18" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="271" spans="1:8">
       <c r="A271" s="5" t="s">
@@ -7049,7 +7060,9 @@
       <c r="G271" s="18" t="s">
         <v>199</v>
       </c>
-      <c r="H271" s="19"/>
+      <c r="H271" s="19" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="272" spans="1:8">
       <c r="A272" s="5" t="s">
@@ -7069,7 +7082,9 @@
       <c r="G272" s="18" t="s">
         <v>64</v>
       </c>
-      <c r="H272" s="19"/>
+      <c r="H272" s="19" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="273" spans="1:8">
       <c r="A273" s="5" t="s">
@@ -7089,7 +7104,9 @@
       <c r="G273" s="18" t="s">
         <v>91</v>
       </c>
-      <c r="H273" s="19"/>
+      <c r="H273" s="19" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="274" spans="1:8" ht="45">
       <c r="A274" s="5" t="s">
@@ -7109,7 +7126,9 @@
       <c r="G274" s="5">
         <v>3</v>
       </c>
-      <c r="H274" s="5"/>
+      <c r="H274" s="5">
+        <v>5</v>
+      </c>
     </row>
     <row r="275" spans="1:8">
       <c r="A275" s="5" t="s">
@@ -7129,7 +7148,9 @@
       <c r="G275" s="5">
         <v>1</v>
       </c>
-      <c r="H275" s="5"/>
+      <c r="H275" s="5">
+        <v>1</v>
+      </c>
     </row>
     <row r="276" spans="1:8" ht="30">
       <c r="A276" s="5" t="s">
@@ -7149,7 +7170,9 @@
       <c r="G276" s="5">
         <v>10</v>
       </c>
-      <c r="H276" s="5"/>
+      <c r="H276" s="5">
+        <v>30</v>
+      </c>
     </row>
     <row r="277" spans="1:8" ht="30">
       <c r="A277" s="5" t="s">
@@ -7169,7 +7192,9 @@
       <c r="G277" s="5">
         <v>440</v>
       </c>
-      <c r="H277" s="18"/>
+      <c r="H277" s="18">
+        <v>570</v>
+      </c>
     </row>
     <row r="278" spans="1:8" ht="75">
       <c r="A278" s="5" t="s">
@@ -7215,7 +7240,9 @@
       <c r="G279" s="5">
         <v>0</v>
       </c>
-      <c r="H279" s="5"/>
+      <c r="H279" s="5">
+        <v>20</v>
+      </c>
     </row>
     <row r="280" spans="1:8" ht="45">
       <c r="A280" s="5" t="s">
@@ -7235,7 +7262,9 @@
       <c r="G280" s="5">
         <v>4</v>
       </c>
-      <c r="H280" s="5"/>
+      <c r="H280" s="5">
+        <v>4</v>
+      </c>
     </row>
     <row r="281" spans="1:8" ht="90">
       <c r="A281" s="5" t="s">
@@ -7255,7 +7284,9 @@
       <c r="G281" s="5">
         <v>4</v>
       </c>
-      <c r="H281" s="5"/>
+      <c r="H281" s="5">
+        <v>4</v>
+      </c>
     </row>
     <row r="282" spans="1:8" ht="105">
       <c r="A282" s="5" t="s">
@@ -7275,7 +7306,9 @@
       <c r="G282" s="5">
         <v>3</v>
       </c>
-      <c r="H282" s="5"/>
+      <c r="H282" s="5">
+        <v>3</v>
+      </c>
     </row>
     <row r="283" spans="1:8" ht="60">
       <c r="A283" s="5" t="s">
@@ -7300,7 +7333,7 @@
         <v>200</v>
       </c>
       <c r="H283" s="5" t="s">
-        <v>26</v>
+        <v>203</v>
       </c>
     </row>
     <row r="284" spans="1:8">
@@ -7329,8 +7362,302 @@
         <v>202</v>
       </c>
     </row>
+    <row r="286" spans="1:8">
+      <c r="A286" s="5"/>
+      <c r="B286" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="C286" s="15" t="s">
+        <v>148</v>
+      </c>
+      <c r="D286" s="15" t="s">
+        <v>149</v>
+      </c>
+      <c r="E286" s="15" t="s">
+        <v>150</v>
+      </c>
+      <c r="F286" s="15" t="s">
+        <v>151</v>
+      </c>
+      <c r="G286" s="15" t="s">
+        <v>152</v>
+      </c>
+      <c r="H286" s="16" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="287" spans="1:8" ht="18">
+      <c r="A287" s="2"/>
+      <c r="B287" s="11">
+        <v>46146</v>
+      </c>
+      <c r="C287" s="11">
+        <f>B287+1</f>
+        <v>46147</v>
+      </c>
+      <c r="D287" s="11">
+        <f t="shared" ref="D287" si="36">C287+1</f>
+        <v>46148</v>
+      </c>
+      <c r="E287" s="11">
+        <f t="shared" ref="E287" si="37">D287+1</f>
+        <v>46149</v>
+      </c>
+      <c r="F287" s="11">
+        <f t="shared" ref="F287" si="38">E287+1</f>
+        <v>46150</v>
+      </c>
+      <c r="G287" s="11">
+        <f t="shared" ref="G287" si="39">F287+1</f>
+        <v>46151</v>
+      </c>
+      <c r="H287" s="11">
+        <f t="shared" ref="H287" si="40">G287+1</f>
+        <v>46152</v>
+      </c>
+    </row>
+    <row r="288" spans="1:8" ht="30">
+      <c r="A288" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B288" s="17" t="s">
+        <v>204</v>
+      </c>
+      <c r="C288" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="D288" s="18"/>
+      <c r="E288" s="18"/>
+      <c r="F288" s="18"/>
+      <c r="G288" s="18"/>
+      <c r="H288" s="18"/>
+    </row>
+    <row r="289" spans="1:8">
+      <c r="A289" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B289" s="18" t="s">
+        <v>199</v>
+      </c>
+      <c r="C289" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="D289" s="18"/>
+      <c r="E289" s="18"/>
+      <c r="F289" s="18"/>
+      <c r="G289" s="18"/>
+      <c r="H289" s="19"/>
+    </row>
+    <row r="290" spans="1:8">
+      <c r="A290" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B290" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="C290" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="D290" s="18"/>
+      <c r="E290" s="20"/>
+      <c r="F290" s="18"/>
+      <c r="G290" s="18"/>
+      <c r="H290" s="19"/>
+    </row>
+    <row r="291" spans="1:8">
+      <c r="A291" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B291" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="C291" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="D291" s="18"/>
+      <c r="E291" s="20"/>
+      <c r="F291" s="18"/>
+      <c r="G291" s="18"/>
+      <c r="H291" s="19"/>
+    </row>
+    <row r="292" spans="1:8" ht="45">
+      <c r="A292" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B292" s="18">
+        <v>0</v>
+      </c>
+      <c r="C292" s="5">
+        <v>0</v>
+      </c>
+      <c r="E292" s="5"/>
+      <c r="F292" s="5"/>
+      <c r="G292" s="5"/>
+      <c r="H292" s="5"/>
+    </row>
+    <row r="293" spans="1:8">
+      <c r="A293" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B293" s="5">
+        <v>0</v>
+      </c>
+      <c r="C293" s="5">
+        <v>1</v>
+      </c>
+      <c r="E293" s="5"/>
+      <c r="F293" s="21"/>
+      <c r="G293" s="5"/>
+      <c r="H293" s="5"/>
+    </row>
+    <row r="294" spans="1:8" ht="30">
+      <c r="A294" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B294" s="5">
+        <v>0</v>
+      </c>
+      <c r="C294" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="D294" s="20"/>
+      <c r="E294" s="5"/>
+      <c r="F294" s="5"/>
+      <c r="G294" s="5"/>
+      <c r="H294" s="5"/>
+    </row>
+    <row r="295" spans="1:8" ht="30">
+      <c r="A295" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B295" s="5">
+        <v>450</v>
+      </c>
+      <c r="C295" s="5">
+        <v>450</v>
+      </c>
+      <c r="D295" s="5"/>
+      <c r="E295" s="5"/>
+      <c r="F295" s="5"/>
+      <c r="G295" s="5"/>
+      <c r="H295" s="18"/>
+    </row>
+    <row r="296" spans="1:8" ht="75">
+      <c r="A296" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B296" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C296" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D296" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E296" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F296" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="G296" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="H296" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="297" spans="1:8" ht="60">
+      <c r="A297" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B297" s="5">
+        <v>0</v>
+      </c>
+      <c r="C297" s="5">
+        <v>20</v>
+      </c>
+      <c r="D297" s="5"/>
+      <c r="E297" s="5"/>
+      <c r="F297" s="5"/>
+      <c r="G297" s="5"/>
+      <c r="H297" s="5"/>
+    </row>
+    <row r="298" spans="1:8" ht="45">
+      <c r="A298" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B298" s="5">
+        <v>4</v>
+      </c>
+      <c r="C298" s="5">
+        <v>4</v>
+      </c>
+      <c r="D298" s="5"/>
+      <c r="E298" s="5"/>
+      <c r="F298" s="5"/>
+      <c r="G298" s="5"/>
+      <c r="H298" s="5"/>
+    </row>
+    <row r="299" spans="1:8" ht="90">
+      <c r="A299" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B299" s="5">
+        <v>4</v>
+      </c>
+      <c r="C299" s="5">
+        <v>3</v>
+      </c>
+      <c r="D299" s="5"/>
+      <c r="E299" s="5"/>
+      <c r="F299" s="5"/>
+      <c r="G299" s="5"/>
+      <c r="H299" s="5"/>
+    </row>
+    <row r="300" spans="1:8" ht="105">
+      <c r="A300" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B300" s="5">
+        <v>3</v>
+      </c>
+      <c r="C300" s="5">
+        <v>4</v>
+      </c>
+      <c r="D300" s="5"/>
+      <c r="E300" s="5"/>
+      <c r="F300" s="5"/>
+      <c r="G300" s="5"/>
+      <c r="H300" s="5"/>
+    </row>
+    <row r="301" spans="1:8" ht="60">
+      <c r="A301" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B301" s="5">
+        <v>0</v>
+      </c>
+      <c r="C301" s="5">
+        <v>30</v>
+      </c>
+      <c r="D301" s="5"/>
+      <c r="E301" s="5"/>
+      <c r="F301" s="5"/>
+      <c r="G301" s="5"/>
+      <c r="H301" s="5"/>
+    </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="B159:H159"/>
+    <mergeCell ref="A59:H59"/>
+    <mergeCell ref="B102:H102"/>
+    <mergeCell ref="A138:H138"/>
+    <mergeCell ref="B139:H139"/>
+    <mergeCell ref="A101:H101"/>
+    <mergeCell ref="A79:H79"/>
+    <mergeCell ref="B80:H80"/>
     <mergeCell ref="B196:H196"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A60:H60"/>
@@ -7347,14 +7674,6 @@
     <mergeCell ref="B61:H61"/>
     <mergeCell ref="A119:H119"/>
     <mergeCell ref="B120:H120"/>
-    <mergeCell ref="B159:H159"/>
-    <mergeCell ref="A59:H59"/>
-    <mergeCell ref="B102:H102"/>
-    <mergeCell ref="A138:H138"/>
-    <mergeCell ref="B139:H139"/>
-    <mergeCell ref="A101:H101"/>
-    <mergeCell ref="A79:H79"/>
-    <mergeCell ref="B80:H80"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>

</xml_diff>

<commit_message>
vault backup: 2026-05-06 15:36:54
</commit_message>
<xml_diff>
--- a/睡眠日记_Sleep_Diary1.xlsx
+++ b/睡眠日记_Sleep_Diary1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My_like\My_like\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DED28C9E-DEAC-48D2-8BC7-F4539B6639F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AADE8D99-F823-4C6F-BD14-46848A63D6DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="904" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="909" uniqueCount="208">
   <si>
     <t>睡眠日记 Sleep Diary</t>
   </si>
@@ -710,6 +710,12 @@
   </si>
   <si>
     <t>90min</t>
+  </si>
+  <si>
+    <t>5：34</t>
+  </si>
+  <si>
+    <t>5：35</t>
   </si>
 </sst>
 </file>
@@ -7426,7 +7432,9 @@
       <c r="C288" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="D288" s="18"/>
+      <c r="D288" s="18" t="s">
+        <v>206</v>
+      </c>
       <c r="E288" s="18"/>
       <c r="F288" s="18"/>
       <c r="G288" s="18"/>
@@ -7442,7 +7450,9 @@
       <c r="C289" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="D289" s="18"/>
+      <c r="D289" s="18" t="s">
+        <v>207</v>
+      </c>
       <c r="E289" s="18"/>
       <c r="F289" s="18"/>
       <c r="G289" s="18"/>
@@ -7458,7 +7468,9 @@
       <c r="C290" s="18" t="s">
         <v>64</v>
       </c>
-      <c r="D290" s="18"/>
+      <c r="D290" s="18" t="s">
+        <v>64</v>
+      </c>
       <c r="E290" s="20"/>
       <c r="F290" s="18"/>
       <c r="G290" s="18"/>
@@ -7474,7 +7486,9 @@
       <c r="C291" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="D291" s="18"/>
+      <c r="D291" s="18" t="s">
+        <v>33</v>
+      </c>
       <c r="E291" s="20"/>
       <c r="F291" s="18"/>
       <c r="G291" s="18"/>
@@ -7490,6 +7504,9 @@
       <c r="C292" s="5">
         <v>0</v>
       </c>
+      <c r="D292">
+        <v>0</v>
+      </c>
       <c r="E292" s="5"/>
       <c r="F292" s="5"/>
       <c r="G292" s="5"/>
@@ -7505,6 +7522,9 @@
       <c r="C293" s="5">
         <v>1</v>
       </c>
+      <c r="D293">
+        <v>0</v>
+      </c>
       <c r="E293" s="5"/>
       <c r="F293" s="21"/>
       <c r="G293" s="5"/>
@@ -7520,7 +7540,9 @@
       <c r="C294" s="5" t="s">
         <v>205</v>
       </c>
-      <c r="D294" s="20"/>
+      <c r="D294" s="20">
+        <v>0</v>
+      </c>
       <c r="E294" s="5"/>
       <c r="F294" s="5"/>
       <c r="G294" s="5"/>
@@ -7536,7 +7558,9 @@
       <c r="C295" s="5">
         <v>450</v>
       </c>
-      <c r="D295" s="5"/>
+      <c r="D295" s="5">
+        <v>450</v>
+      </c>
       <c r="E295" s="5"/>
       <c r="F295" s="5"/>
       <c r="G295" s="5"/>
@@ -7578,7 +7602,9 @@
       <c r="C297" s="5">
         <v>20</v>
       </c>
-      <c r="D297" s="5"/>
+      <c r="D297" s="5">
+        <v>0</v>
+      </c>
       <c r="E297" s="5"/>
       <c r="F297" s="5"/>
       <c r="G297" s="5"/>
@@ -7594,7 +7620,9 @@
       <c r="C298" s="5">
         <v>4</v>
       </c>
-      <c r="D298" s="5"/>
+      <c r="D298" s="5">
+        <v>4</v>
+      </c>
       <c r="E298" s="5"/>
       <c r="F298" s="5"/>
       <c r="G298" s="5"/>
@@ -7610,7 +7638,9 @@
       <c r="C299" s="5">
         <v>3</v>
       </c>
-      <c r="D299" s="5"/>
+      <c r="D299" s="5">
+        <v>3</v>
+      </c>
       <c r="E299" s="5"/>
       <c r="F299" s="5"/>
       <c r="G299" s="5"/>
@@ -7626,7 +7656,9 @@
       <c r="C300" s="5">
         <v>4</v>
       </c>
-      <c r="D300" s="5"/>
+      <c r="D300" s="5">
+        <v>4</v>
+      </c>
       <c r="E300" s="5"/>
       <c r="F300" s="5"/>
       <c r="G300" s="5"/>
@@ -7642,7 +7674,9 @@
       <c r="C301" s="5">
         <v>30</v>
       </c>
-      <c r="D301" s="5"/>
+      <c r="D301" s="5" t="s">
+        <v>26</v>
+      </c>
       <c r="E301" s="5"/>
       <c r="F301" s="5"/>
       <c r="G301" s="5"/>
@@ -7650,14 +7684,6 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="B159:H159"/>
-    <mergeCell ref="A59:H59"/>
-    <mergeCell ref="B102:H102"/>
-    <mergeCell ref="A138:H138"/>
-    <mergeCell ref="B139:H139"/>
-    <mergeCell ref="A101:H101"/>
-    <mergeCell ref="A79:H79"/>
-    <mergeCell ref="B80:H80"/>
     <mergeCell ref="B196:H196"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A60:H60"/>
@@ -7674,6 +7700,14 @@
     <mergeCell ref="B61:H61"/>
     <mergeCell ref="A119:H119"/>
     <mergeCell ref="B120:H120"/>
+    <mergeCell ref="B159:H159"/>
+    <mergeCell ref="A59:H59"/>
+    <mergeCell ref="B102:H102"/>
+    <mergeCell ref="A138:H138"/>
+    <mergeCell ref="B139:H139"/>
+    <mergeCell ref="A101:H101"/>
+    <mergeCell ref="A79:H79"/>
+    <mergeCell ref="B80:H80"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>

</xml_diff>

<commit_message>
vault backup: 2026-05-10 06:46:07
</commit_message>
<xml_diff>
--- a/睡眠日记_Sleep_Diary1.xlsx
+++ b/睡眠日记_Sleep_Diary1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My_like\My_like\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AADE8D99-F823-4C6F-BD14-46848A63D6DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC4D662E-D732-4ACB-9C71-CBC4757E5A8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="909" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="998" uniqueCount="212">
   <si>
     <t>睡眠日记 Sleep Diary</t>
   </si>
@@ -716,6 +716,18 @@
   </si>
   <si>
     <t>5：35</t>
+  </si>
+  <si>
+    <t>周三白天精神比较紧张</t>
+  </si>
+  <si>
+    <t>6：13</t>
+  </si>
+  <si>
+    <t>周五周六白天比较容易困</t>
+  </si>
+  <si>
+    <t>自然在6点醒的习惯已经养成了，花了11天</t>
   </si>
 </sst>
 </file>
@@ -1254,7 +1266,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H301"/>
+  <dimension ref="A1:H337"/>
   <sheetFormatPr defaultColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="8" width="20" customWidth="1"/>
@@ -7435,10 +7447,14 @@
       <c r="D288" s="18" t="s">
         <v>206</v>
       </c>
-      <c r="E288" s="18"/>
+      <c r="E288" s="18" t="s">
+        <v>172</v>
+      </c>
       <c r="F288" s="18"/>
       <c r="G288" s="18"/>
-      <c r="H288" s="18"/>
+      <c r="H288" s="18" t="s">
+        <v>209</v>
+      </c>
     </row>
     <row r="289" spans="1:8">
       <c r="A289" s="5" t="s">
@@ -7453,10 +7469,14 @@
       <c r="D289" s="18" t="s">
         <v>207</v>
       </c>
-      <c r="E289" s="18"/>
+      <c r="E289" s="18" t="s">
+        <v>178</v>
+      </c>
       <c r="F289" s="18"/>
       <c r="G289" s="18"/>
-      <c r="H289" s="19"/>
+      <c r="H289" s="19" t="s">
+        <v>209</v>
+      </c>
     </row>
     <row r="290" spans="1:8">
       <c r="A290" s="5" t="s">
@@ -7471,10 +7491,14 @@
       <c r="D290" s="18" t="s">
         <v>64</v>
       </c>
-      <c r="E290" s="20"/>
+      <c r="E290" s="20" t="s">
+        <v>64</v>
+      </c>
       <c r="F290" s="18"/>
       <c r="G290" s="18"/>
-      <c r="H290" s="19"/>
+      <c r="H290" s="19" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="291" spans="1:8">
       <c r="A291" s="5" t="s">
@@ -7489,10 +7513,14 @@
       <c r="D291" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="E291" s="20"/>
+      <c r="E291" s="20" t="s">
+        <v>30</v>
+      </c>
       <c r="F291" s="18"/>
       <c r="G291" s="18"/>
-      <c r="H291" s="19"/>
+      <c r="H291" s="19" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="292" spans="1:8" ht="45">
       <c r="A292" s="5" t="s">
@@ -7507,10 +7535,14 @@
       <c r="D292">
         <v>0</v>
       </c>
-      <c r="E292" s="5"/>
+      <c r="E292" s="5">
+        <v>5</v>
+      </c>
       <c r="F292" s="5"/>
       <c r="G292" s="5"/>
-      <c r="H292" s="5"/>
+      <c r="H292" s="5">
+        <v>0</v>
+      </c>
     </row>
     <row r="293" spans="1:8">
       <c r="A293" s="5" t="s">
@@ -7525,10 +7557,14 @@
       <c r="D293">
         <v>0</v>
       </c>
-      <c r="E293" s="5"/>
+      <c r="E293" s="5">
+        <v>0</v>
+      </c>
       <c r="F293" s="21"/>
       <c r="G293" s="5"/>
-      <c r="H293" s="5"/>
+      <c r="H293" s="5">
+        <v>0</v>
+      </c>
     </row>
     <row r="294" spans="1:8" ht="30">
       <c r="A294" s="5" t="s">
@@ -7543,10 +7579,14 @@
       <c r="D294" s="20">
         <v>0</v>
       </c>
-      <c r="E294" s="5"/>
+      <c r="E294" s="5">
+        <v>0</v>
+      </c>
       <c r="F294" s="5"/>
       <c r="G294" s="5"/>
-      <c r="H294" s="5"/>
+      <c r="H294" s="5">
+        <v>0</v>
+      </c>
     </row>
     <row r="295" spans="1:8" ht="30">
       <c r="A295" s="5" t="s">
@@ -7561,10 +7601,14 @@
       <c r="D295" s="5">
         <v>450</v>
       </c>
-      <c r="E295" s="5"/>
+      <c r="E295" s="5">
+        <v>390</v>
+      </c>
       <c r="F295" s="5"/>
       <c r="G295" s="5"/>
-      <c r="H295" s="18"/>
+      <c r="H295" s="18">
+        <v>420</v>
+      </c>
     </row>
     <row r="296" spans="1:8" ht="75">
       <c r="A296" s="5" t="s">
@@ -7605,10 +7649,14 @@
       <c r="D297" s="5">
         <v>0</v>
       </c>
-      <c r="E297" s="5"/>
+      <c r="E297" s="5">
+        <v>60</v>
+      </c>
       <c r="F297" s="5"/>
       <c r="G297" s="5"/>
-      <c r="H297" s="5"/>
+      <c r="H297" s="5">
+        <v>0</v>
+      </c>
     </row>
     <row r="298" spans="1:8" ht="45">
       <c r="A298" s="5" t="s">
@@ -7623,10 +7671,14 @@
       <c r="D298" s="5">
         <v>4</v>
       </c>
-      <c r="E298" s="5"/>
+      <c r="E298" s="5">
+        <v>4</v>
+      </c>
       <c r="F298" s="5"/>
       <c r="G298" s="5"/>
-      <c r="H298" s="5"/>
+      <c r="H298" s="5">
+        <v>4</v>
+      </c>
     </row>
     <row r="299" spans="1:8" ht="90">
       <c r="A299" s="5" t="s">
@@ -7641,10 +7693,14 @@
       <c r="D299" s="5">
         <v>3</v>
       </c>
-      <c r="E299" s="5"/>
+      <c r="E299" s="5">
+        <v>4</v>
+      </c>
       <c r="F299" s="5"/>
       <c r="G299" s="5"/>
-      <c r="H299" s="5"/>
+      <c r="H299" s="5">
+        <v>4</v>
+      </c>
     </row>
     <row r="300" spans="1:8" ht="105">
       <c r="A300" s="5" t="s">
@@ -7659,10 +7715,14 @@
       <c r="D300" s="5">
         <v>4</v>
       </c>
-      <c r="E300" s="5"/>
+      <c r="E300" s="5">
+        <v>4</v>
+      </c>
       <c r="F300" s="5"/>
       <c r="G300" s="5"/>
-      <c r="H300" s="5"/>
+      <c r="H300" s="5">
+        <v>4</v>
+      </c>
     </row>
     <row r="301" spans="1:8" ht="60">
       <c r="A301" s="5" t="s">
@@ -7677,10 +7737,625 @@
       <c r="D301" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="E301" s="5"/>
+      <c r="E301" s="5">
+        <v>30</v>
+      </c>
       <c r="F301" s="5"/>
       <c r="G301" s="5"/>
-      <c r="H301" s="5"/>
+      <c r="H301" s="5">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="302" spans="1:8">
+      <c r="E302" t="s">
+        <v>208</v>
+      </c>
+      <c r="G302" t="s">
+        <v>210</v>
+      </c>
+      <c r="H302" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="304" spans="1:8">
+      <c r="A304" s="5"/>
+      <c r="B304" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="C304" s="15" t="s">
+        <v>148</v>
+      </c>
+      <c r="D304" s="15" t="s">
+        <v>149</v>
+      </c>
+      <c r="E304" s="15" t="s">
+        <v>150</v>
+      </c>
+      <c r="F304" s="15" t="s">
+        <v>151</v>
+      </c>
+      <c r="G304" s="15" t="s">
+        <v>152</v>
+      </c>
+      <c r="H304" s="16" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="305" spans="1:8" ht="18">
+      <c r="A305" s="2"/>
+      <c r="B305" s="11">
+        <v>46146</v>
+      </c>
+      <c r="C305" s="11">
+        <f>B305+1</f>
+        <v>46147</v>
+      </c>
+      <c r="D305" s="11">
+        <f t="shared" ref="D305" si="41">C305+1</f>
+        <v>46148</v>
+      </c>
+      <c r="E305" s="11">
+        <f t="shared" ref="E305" si="42">D305+1</f>
+        <v>46149</v>
+      </c>
+      <c r="F305" s="11">
+        <f t="shared" ref="F305" si="43">E305+1</f>
+        <v>46150</v>
+      </c>
+      <c r="G305" s="11">
+        <f t="shared" ref="G305" si="44">F305+1</f>
+        <v>46151</v>
+      </c>
+      <c r="H305" s="11">
+        <f t="shared" ref="H305" si="45">G305+1</f>
+        <v>46152</v>
+      </c>
+    </row>
+    <row r="306" spans="1:8" ht="30">
+      <c r="A306" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B306" s="17" t="s">
+        <v>204</v>
+      </c>
+      <c r="C306" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="D306" s="18" t="s">
+        <v>206</v>
+      </c>
+      <c r="E306" s="18" t="s">
+        <v>172</v>
+      </c>
+      <c r="F306" s="18"/>
+      <c r="G306" s="18"/>
+      <c r="H306" s="18" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="307" spans="1:8">
+      <c r="A307" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B307" s="18" t="s">
+        <v>199</v>
+      </c>
+      <c r="C307" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="D307" s="18" t="s">
+        <v>207</v>
+      </c>
+      <c r="E307" s="18" t="s">
+        <v>178</v>
+      </c>
+      <c r="F307" s="18"/>
+      <c r="G307" s="18"/>
+      <c r="H307" s="19" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="308" spans="1:8">
+      <c r="A308" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B308" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="C308" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="D308" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="E308" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="F308" s="18"/>
+      <c r="G308" s="18"/>
+      <c r="H308" s="19" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="309" spans="1:8">
+      <c r="A309" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B309" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="C309" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="D309" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="E309" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="F309" s="18"/>
+      <c r="G309" s="18"/>
+      <c r="H309" s="19" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="310" spans="1:8" ht="45">
+      <c r="A310" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B310" s="18">
+        <v>0</v>
+      </c>
+      <c r="C310" s="5">
+        <v>0</v>
+      </c>
+      <c r="D310">
+        <v>0</v>
+      </c>
+      <c r="E310" s="5">
+        <v>5</v>
+      </c>
+      <c r="F310" s="5"/>
+      <c r="G310" s="5"/>
+      <c r="H310" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="311" spans="1:8">
+      <c r="A311" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B311" s="5">
+        <v>0</v>
+      </c>
+      <c r="C311" s="5">
+        <v>1</v>
+      </c>
+      <c r="D311">
+        <v>0</v>
+      </c>
+      <c r="E311" s="5">
+        <v>0</v>
+      </c>
+      <c r="F311" s="21"/>
+      <c r="G311" s="5"/>
+      <c r="H311" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="312" spans="1:8" ht="30">
+      <c r="A312" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B312" s="5">
+        <v>0</v>
+      </c>
+      <c r="C312" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="D312" s="20">
+        <v>0</v>
+      </c>
+      <c r="E312" s="5">
+        <v>0</v>
+      </c>
+      <c r="F312" s="5"/>
+      <c r="G312" s="5"/>
+      <c r="H312" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="313" spans="1:8" ht="30">
+      <c r="A313" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B313" s="5">
+        <v>450</v>
+      </c>
+      <c r="C313" s="5">
+        <v>450</v>
+      </c>
+      <c r="D313" s="5">
+        <v>450</v>
+      </c>
+      <c r="E313" s="5">
+        <v>390</v>
+      </c>
+      <c r="F313" s="5"/>
+      <c r="G313" s="5"/>
+      <c r="H313" s="18">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="314" spans="1:8" ht="75">
+      <c r="A314" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B314" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C314" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D314" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E314" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F314" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="G314" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="H314" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="315" spans="1:8" ht="60">
+      <c r="A315" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B315" s="5">
+        <v>0</v>
+      </c>
+      <c r="C315" s="5">
+        <v>20</v>
+      </c>
+      <c r="D315" s="5">
+        <v>0</v>
+      </c>
+      <c r="E315" s="5">
+        <v>60</v>
+      </c>
+      <c r="F315" s="5"/>
+      <c r="G315" s="5"/>
+      <c r="H315" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="316" spans="1:8" ht="45">
+      <c r="A316" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B316" s="5">
+        <v>4</v>
+      </c>
+      <c r="C316" s="5">
+        <v>4</v>
+      </c>
+      <c r="D316" s="5">
+        <v>4</v>
+      </c>
+      <c r="E316" s="5">
+        <v>4</v>
+      </c>
+      <c r="F316" s="5"/>
+      <c r="G316" s="5"/>
+      <c r="H316" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="317" spans="1:8" ht="90">
+      <c r="A317" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B317" s="5">
+        <v>4</v>
+      </c>
+      <c r="C317" s="5">
+        <v>3</v>
+      </c>
+      <c r="D317" s="5">
+        <v>3</v>
+      </c>
+      <c r="E317" s="5">
+        <v>4</v>
+      </c>
+      <c r="F317" s="5"/>
+      <c r="G317" s="5"/>
+      <c r="H317" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="318" spans="1:8" ht="105">
+      <c r="A318" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B318" s="5">
+        <v>3</v>
+      </c>
+      <c r="C318" s="5">
+        <v>4</v>
+      </c>
+      <c r="D318" s="5">
+        <v>4</v>
+      </c>
+      <c r="E318" s="5">
+        <v>4</v>
+      </c>
+      <c r="F318" s="5"/>
+      <c r="G318" s="5"/>
+      <c r="H318" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="319" spans="1:8" ht="60">
+      <c r="A319" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B319" s="5">
+        <v>0</v>
+      </c>
+      <c r="C319" s="5">
+        <v>30</v>
+      </c>
+      <c r="D319" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E319" s="5">
+        <v>30</v>
+      </c>
+      <c r="F319" s="5"/>
+      <c r="G319" s="5"/>
+      <c r="H319" s="5">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="322" spans="1:8">
+      <c r="A322" s="5"/>
+      <c r="B322" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="C322" s="15" t="s">
+        <v>148</v>
+      </c>
+      <c r="D322" s="15" t="s">
+        <v>149</v>
+      </c>
+      <c r="E322" s="15" t="s">
+        <v>150</v>
+      </c>
+      <c r="F322" s="15" t="s">
+        <v>151</v>
+      </c>
+      <c r="G322" s="15" t="s">
+        <v>152</v>
+      </c>
+      <c r="H322" s="16" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="323" spans="1:8" ht="18">
+      <c r="A323" s="2"/>
+      <c r="B323" s="11">
+        <v>46153</v>
+      </c>
+      <c r="C323" s="11">
+        <f>B323+1</f>
+        <v>46154</v>
+      </c>
+      <c r="D323" s="11">
+        <f t="shared" ref="D323" si="46">C323+1</f>
+        <v>46155</v>
+      </c>
+      <c r="E323" s="11">
+        <f t="shared" ref="E323" si="47">D323+1</f>
+        <v>46156</v>
+      </c>
+      <c r="F323" s="11">
+        <f t="shared" ref="F323" si="48">E323+1</f>
+        <v>46157</v>
+      </c>
+      <c r="G323" s="11">
+        <f t="shared" ref="G323" si="49">F323+1</f>
+        <v>46158</v>
+      </c>
+      <c r="H323" s="11">
+        <f t="shared" ref="H323" si="50">G323+1</f>
+        <v>46159</v>
+      </c>
+    </row>
+    <row r="324" spans="1:8" ht="30">
+      <c r="A324" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B324" s="17"/>
+      <c r="C324" s="18"/>
+      <c r="D324" s="18"/>
+      <c r="E324" s="18"/>
+      <c r="F324" s="18"/>
+      <c r="G324" s="18"/>
+      <c r="H324" s="18"/>
+    </row>
+    <row r="325" spans="1:8">
+      <c r="A325" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B325" s="18"/>
+      <c r="C325" s="18"/>
+      <c r="D325" s="18"/>
+      <c r="E325" s="18"/>
+      <c r="F325" s="18"/>
+      <c r="G325" s="18"/>
+      <c r="H325" s="19"/>
+    </row>
+    <row r="326" spans="1:8">
+      <c r="A326" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B326" s="18"/>
+      <c r="C326" s="18"/>
+      <c r="D326" s="18"/>
+      <c r="E326" s="20"/>
+      <c r="F326" s="18"/>
+      <c r="G326" s="18"/>
+      <c r="H326" s="19"/>
+    </row>
+    <row r="327" spans="1:8">
+      <c r="A327" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B327" s="18"/>
+      <c r="C327" s="18"/>
+      <c r="D327" s="18"/>
+      <c r="E327" s="20"/>
+      <c r="F327" s="18"/>
+      <c r="G327" s="18"/>
+      <c r="H327" s="19"/>
+    </row>
+    <row r="328" spans="1:8" ht="45">
+      <c r="A328" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B328" s="18"/>
+      <c r="C328" s="5"/>
+      <c r="E328" s="5"/>
+      <c r="F328" s="5"/>
+      <c r="G328" s="5"/>
+      <c r="H328" s="5"/>
+    </row>
+    <row r="329" spans="1:8">
+      <c r="A329" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B329" s="5"/>
+      <c r="C329" s="5"/>
+      <c r="E329" s="5"/>
+      <c r="F329" s="21"/>
+      <c r="G329" s="5"/>
+      <c r="H329" s="5"/>
+    </row>
+    <row r="330" spans="1:8" ht="30">
+      <c r="A330" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B330" s="5"/>
+      <c r="C330" s="5"/>
+      <c r="D330" s="20"/>
+      <c r="E330" s="5"/>
+      <c r="F330" s="5"/>
+      <c r="G330" s="5"/>
+      <c r="H330" s="5"/>
+    </row>
+    <row r="331" spans="1:8" ht="30">
+      <c r="A331" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B331" s="5"/>
+      <c r="C331" s="5"/>
+      <c r="D331" s="5"/>
+      <c r="E331" s="5"/>
+      <c r="F331" s="5"/>
+      <c r="G331" s="5"/>
+      <c r="H331" s="18"/>
+    </row>
+    <row r="332" spans="1:8" ht="75">
+      <c r="A332" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B332" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C332" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D332" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E332" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F332" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="G332" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="H332" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="333" spans="1:8" ht="60">
+      <c r="A333" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B333" s="5"/>
+      <c r="C333" s="5"/>
+      <c r="D333" s="5"/>
+      <c r="E333" s="5"/>
+      <c r="F333" s="5"/>
+      <c r="G333" s="5"/>
+      <c r="H333" s="5"/>
+    </row>
+    <row r="334" spans="1:8" ht="45">
+      <c r="A334" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B334" s="5"/>
+      <c r="C334" s="5"/>
+      <c r="D334" s="5"/>
+      <c r="E334" s="5"/>
+      <c r="F334" s="5"/>
+      <c r="G334" s="5"/>
+      <c r="H334" s="5"/>
+    </row>
+    <row r="335" spans="1:8" ht="90">
+      <c r="A335" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B335" s="5"/>
+      <c r="C335" s="5"/>
+      <c r="D335" s="5"/>
+      <c r="E335" s="5"/>
+      <c r="F335" s="5"/>
+      <c r="G335" s="5"/>
+      <c r="H335" s="5"/>
+    </row>
+    <row r="336" spans="1:8" ht="105">
+      <c r="A336" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B336" s="5"/>
+      <c r="C336" s="5"/>
+      <c r="D336" s="5"/>
+      <c r="E336" s="5"/>
+      <c r="F336" s="5"/>
+      <c r="G336" s="5"/>
+      <c r="H336" s="5"/>
+    </row>
+    <row r="337" spans="1:8" ht="60">
+      <c r="A337" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B337" s="5"/>
+      <c r="C337" s="5"/>
+      <c r="D337" s="5"/>
+      <c r="E337" s="5"/>
+      <c r="F337" s="5"/>
+      <c r="G337" s="5"/>
+      <c r="H337" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="24">

</xml_diff>

<commit_message>
vault backup: 2026-05-11 07:07:05
</commit_message>
<xml_diff>
--- a/睡眠日记_Sleep_Diary1.xlsx
+++ b/睡眠日记_Sleep_Diary1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My_like\My_like\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC4D662E-D732-4ACB-9C71-CBC4757E5A8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{691AE4B6-0EBF-4B07-B786-7C797D7EF823}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3075" yWindow="0" windowWidth="15660" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="睡眠日记 Sleep Diary" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="998" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1004" uniqueCount="214">
   <si>
     <t>睡眠日记 Sleep Diary</t>
   </si>
@@ -728,6 +728,12 @@
   </si>
   <si>
     <t>自然在6点醒的习惯已经养成了，花了11天</t>
+  </si>
+  <si>
+    <t>6：45</t>
+  </si>
+  <si>
+    <t>开始控制饮食第一天</t>
   </si>
 </sst>
 </file>
@@ -1266,7 +1272,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H337"/>
+  <dimension ref="A1:H338"/>
   <sheetFormatPr defaultColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="8" width="20" customWidth="1"/>
@@ -8181,7 +8187,9 @@
       <c r="A324" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B324" s="17"/>
+      <c r="B324" s="17" t="s">
+        <v>212</v>
+      </c>
       <c r="C324" s="18"/>
       <c r="D324" s="18"/>
       <c r="E324" s="18"/>
@@ -8193,7 +8201,9 @@
       <c r="A325" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B325" s="18"/>
+      <c r="B325" s="18" t="s">
+        <v>212</v>
+      </c>
       <c r="C325" s="18"/>
       <c r="D325" s="18"/>
       <c r="E325" s="18"/>
@@ -8205,7 +8215,9 @@
       <c r="A326" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B326" s="18"/>
+      <c r="B326" t="s">
+        <v>105</v>
+      </c>
       <c r="C326" s="18"/>
       <c r="D326" s="18"/>
       <c r="E326" s="20"/>
@@ -8217,7 +8229,9 @@
       <c r="A327" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B327" s="18"/>
+      <c r="B327" s="18" t="s">
+        <v>44</v>
+      </c>
       <c r="C327" s="18"/>
       <c r="D327" s="18"/>
       <c r="E327" s="20"/>
@@ -8229,7 +8243,9 @@
       <c r="A328" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B328" s="18"/>
+      <c r="B328" s="18">
+        <v>0</v>
+      </c>
       <c r="C328" s="5"/>
       <c r="E328" s="5"/>
       <c r="F328" s="5"/>
@@ -8240,7 +8256,9 @@
       <c r="A329" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B329" s="5"/>
+      <c r="B329" s="5">
+        <v>1</v>
+      </c>
       <c r="C329" s="5"/>
       <c r="E329" s="5"/>
       <c r="F329" s="21"/>
@@ -8251,7 +8269,9 @@
       <c r="A330" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B330" s="5"/>
+      <c r="B330" s="5">
+        <v>5</v>
+      </c>
       <c r="C330" s="5"/>
       <c r="D330" s="20"/>
       <c r="E330" s="5"/>
@@ -8263,7 +8283,9 @@
       <c r="A331" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B331" s="5"/>
+      <c r="B331" s="5">
+        <v>450</v>
+      </c>
       <c r="C331" s="5"/>
       <c r="D331" s="5"/>
       <c r="E331" s="5"/>
@@ -8301,7 +8323,9 @@
       <c r="A333" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B333" s="5"/>
+      <c r="B333" s="5">
+        <v>0</v>
+      </c>
       <c r="C333" s="5"/>
       <c r="D333" s="5"/>
       <c r="E333" s="5"/>
@@ -8313,7 +8337,9 @@
       <c r="A334" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="B334" s="5"/>
+      <c r="B334" s="5">
+        <v>4</v>
+      </c>
       <c r="C334" s="5"/>
       <c r="D334" s="5"/>
       <c r="E334" s="5"/>
@@ -8325,7 +8351,9 @@
       <c r="A335" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B335" s="5"/>
+      <c r="B335" s="5">
+        <v>4</v>
+      </c>
       <c r="C335" s="5"/>
       <c r="D335" s="5"/>
       <c r="E335" s="5"/>
@@ -8337,7 +8365,9 @@
       <c r="A336" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B336" s="5"/>
+      <c r="B336" s="5">
+        <v>4</v>
+      </c>
       <c r="C336" s="5"/>
       <c r="D336" s="5"/>
       <c r="E336" s="5"/>
@@ -8349,7 +8379,9 @@
       <c r="A337" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B337" s="5"/>
+      <c r="B337" s="5" t="s">
+        <v>26</v>
+      </c>
       <c r="C337" s="5"/>
       <c r="D337" s="5"/>
       <c r="E337" s="5"/>
@@ -8357,8 +8389,21 @@
       <c r="G337" s="5"/>
       <c r="H337" s="5"/>
     </row>
+    <row r="338" spans="1:8">
+      <c r="B338" t="s">
+        <v>213</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="B159:H159"/>
+    <mergeCell ref="A59:H59"/>
+    <mergeCell ref="B102:H102"/>
+    <mergeCell ref="A138:H138"/>
+    <mergeCell ref="B139:H139"/>
+    <mergeCell ref="A101:H101"/>
+    <mergeCell ref="A79:H79"/>
+    <mergeCell ref="B80:H80"/>
     <mergeCell ref="B196:H196"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A60:H60"/>
@@ -8375,14 +8420,6 @@
     <mergeCell ref="B61:H61"/>
     <mergeCell ref="A119:H119"/>
     <mergeCell ref="B120:H120"/>
-    <mergeCell ref="B159:H159"/>
-    <mergeCell ref="A59:H59"/>
-    <mergeCell ref="B102:H102"/>
-    <mergeCell ref="A138:H138"/>
-    <mergeCell ref="B139:H139"/>
-    <mergeCell ref="A101:H101"/>
-    <mergeCell ref="A79:H79"/>
-    <mergeCell ref="B80:H80"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>

</xml_diff>

<commit_message>
vault backup: 2026-05-12 06:42:44
</commit_message>
<xml_diff>
--- a/睡眠日记_Sleep_Diary1.xlsx
+++ b/睡眠日记_Sleep_Diary1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My_like\My_like\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{691AE4B6-0EBF-4B07-B786-7C797D7EF823}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B776624C-C529-4581-91E8-76DE8BF44EEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3075" yWindow="0" windowWidth="15660" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-135" yWindow="0" windowWidth="12600" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="睡眠日记 Sleep Diary" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1004" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1009" uniqueCount="215">
   <si>
     <t>睡眠日记 Sleep Diary</t>
   </si>
@@ -734,6 +734,9 @@
   </si>
   <si>
     <t>开始控制饮食第一天</t>
+  </si>
+  <si>
+    <t>6：12</t>
   </si>
 </sst>
 </file>
@@ -8190,7 +8193,9 @@
       <c r="B324" s="17" t="s">
         <v>212</v>
       </c>
-      <c r="C324" s="18"/>
+      <c r="C324" s="18" t="s">
+        <v>71</v>
+      </c>
       <c r="D324" s="18"/>
       <c r="E324" s="18"/>
       <c r="F324" s="18"/>
@@ -8204,7 +8209,9 @@
       <c r="B325" s="18" t="s">
         <v>212</v>
       </c>
-      <c r="C325" s="18"/>
+      <c r="C325" s="18" t="s">
+        <v>214</v>
+      </c>
       <c r="D325" s="18"/>
       <c r="E325" s="18"/>
       <c r="F325" s="18"/>
@@ -8218,7 +8225,9 @@
       <c r="B326" t="s">
         <v>105</v>
       </c>
-      <c r="C326" s="18"/>
+      <c r="C326" s="18" t="s">
+        <v>64</v>
+      </c>
       <c r="D326" s="18"/>
       <c r="E326" s="20"/>
       <c r="F326" s="18"/>
@@ -8232,7 +8241,9 @@
       <c r="B327" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="C327" s="18"/>
+      <c r="C327" s="18" t="s">
+        <v>91</v>
+      </c>
       <c r="D327" s="18"/>
       <c r="E327" s="20"/>
       <c r="F327" s="18"/>
@@ -8246,7 +8257,9 @@
       <c r="B328" s="18">
         <v>0</v>
       </c>
-      <c r="C328" s="5"/>
+      <c r="C328" s="5">
+        <v>0</v>
+      </c>
       <c r="E328" s="5"/>
       <c r="F328" s="5"/>
       <c r="G328" s="5"/>
@@ -8259,7 +8272,9 @@
       <c r="B329" s="5">
         <v>1</v>
       </c>
-      <c r="C329" s="5"/>
+      <c r="C329" s="5">
+        <v>1</v>
+      </c>
       <c r="E329" s="5"/>
       <c r="F329" s="21"/>
       <c r="G329" s="5"/>
@@ -8272,7 +8287,9 @@
       <c r="B330" s="5">
         <v>5</v>
       </c>
-      <c r="C330" s="5"/>
+      <c r="C330" s="5">
+        <v>5</v>
+      </c>
       <c r="D330" s="20"/>
       <c r="E330" s="5"/>
       <c r="F330" s="5"/>
@@ -8286,7 +8303,9 @@
       <c r="B331" s="5">
         <v>450</v>
       </c>
-      <c r="C331" s="5"/>
+      <c r="C331" s="5">
+        <v>450</v>
+      </c>
       <c r="D331" s="5"/>
       <c r="E331" s="5"/>
       <c r="F331" s="5"/>
@@ -8326,7 +8345,9 @@
       <c r="B333" s="5">
         <v>0</v>
       </c>
-      <c r="C333" s="5"/>
+      <c r="C333" s="5">
+        <v>0</v>
+      </c>
       <c r="D333" s="5"/>
       <c r="E333" s="5"/>
       <c r="F333" s="5"/>
@@ -8340,7 +8361,9 @@
       <c r="B334" s="5">
         <v>4</v>
       </c>
-      <c r="C334" s="5"/>
+      <c r="C334" s="5">
+        <v>4</v>
+      </c>
       <c r="D334" s="5"/>
       <c r="E334" s="5"/>
       <c r="F334" s="5"/>
@@ -8354,7 +8377,9 @@
       <c r="B335" s="5">
         <v>4</v>
       </c>
-      <c r="C335" s="5"/>
+      <c r="C335" s="5">
+        <v>3</v>
+      </c>
       <c r="D335" s="5"/>
       <c r="E335" s="5"/>
       <c r="F335" s="5"/>
@@ -8368,7 +8393,9 @@
       <c r="B336" s="5">
         <v>4</v>
       </c>
-      <c r="C336" s="5"/>
+      <c r="C336" s="5">
+        <v>4</v>
+      </c>
       <c r="D336" s="5"/>
       <c r="E336" s="5"/>
       <c r="F336" s="5"/>
@@ -8382,7 +8409,9 @@
       <c r="B337" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C337" s="5"/>
+      <c r="C337" s="5" t="s">
+        <v>26</v>
+      </c>
       <c r="D337" s="5"/>
       <c r="E337" s="5"/>
       <c r="F337" s="5"/>
@@ -8393,17 +8422,12 @@
       <c r="B338" t="s">
         <v>213</v>
       </c>
+      <c r="C338">
+        <v>2</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="B159:H159"/>
-    <mergeCell ref="A59:H59"/>
-    <mergeCell ref="B102:H102"/>
-    <mergeCell ref="A138:H138"/>
-    <mergeCell ref="B139:H139"/>
-    <mergeCell ref="A101:H101"/>
-    <mergeCell ref="A79:H79"/>
-    <mergeCell ref="B80:H80"/>
     <mergeCell ref="B196:H196"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A60:H60"/>
@@ -8420,6 +8444,14 @@
     <mergeCell ref="B61:H61"/>
     <mergeCell ref="A119:H119"/>
     <mergeCell ref="B120:H120"/>
+    <mergeCell ref="B159:H159"/>
+    <mergeCell ref="A59:H59"/>
+    <mergeCell ref="B102:H102"/>
+    <mergeCell ref="A138:H138"/>
+    <mergeCell ref="B139:H139"/>
+    <mergeCell ref="A101:H101"/>
+    <mergeCell ref="A79:H79"/>
+    <mergeCell ref="B80:H80"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>

</xml_diff>

<commit_message>
vault backup: 2026-05-14 10:18:42
</commit_message>
<xml_diff>
--- a/睡眠日记_Sleep_Diary1.xlsx
+++ b/睡眠日记_Sleep_Diary1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My_like\My_like\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B776624C-C529-4581-91E8-76DE8BF44EEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B36B83B7-A01B-4876-B895-D6CF3E87A40D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-135" yWindow="0" windowWidth="12600" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="睡眠日记 Sleep Diary" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1009" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1019" uniqueCount="219">
   <si>
     <t>睡眠日记 Sleep Diary</t>
   </si>
@@ -737,6 +737,18 @@
   </si>
   <si>
     <t>6：12</t>
+  </si>
+  <si>
+    <t>6：57</t>
+  </si>
+  <si>
+    <t>停止控制饮食</t>
+  </si>
+  <si>
+    <t>9：29</t>
+  </si>
+  <si>
+    <t>恢复饮食</t>
   </si>
 </sst>
 </file>
@@ -8196,8 +8208,12 @@
       <c r="C324" s="18" t="s">
         <v>71</v>
       </c>
-      <c r="D324" s="18"/>
-      <c r="E324" s="18"/>
+      <c r="D324" s="18" t="s">
+        <v>215</v>
+      </c>
+      <c r="E324" s="18" t="s">
+        <v>70</v>
+      </c>
       <c r="F324" s="18"/>
       <c r="G324" s="18"/>
       <c r="H324" s="18"/>
@@ -8212,8 +8228,12 @@
       <c r="C325" s="18" t="s">
         <v>214</v>
       </c>
-      <c r="D325" s="18"/>
-      <c r="E325" s="18"/>
+      <c r="D325" s="18" t="s">
+        <v>215</v>
+      </c>
+      <c r="E325" s="18" t="s">
+        <v>217</v>
+      </c>
       <c r="F325" s="18"/>
       <c r="G325" s="18"/>
       <c r="H325" s="19"/>
@@ -8228,8 +8248,12 @@
       <c r="C326" s="18" t="s">
         <v>64</v>
       </c>
-      <c r="D326" s="18"/>
-      <c r="E326" s="20"/>
+      <c r="D326" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="E326" s="20" t="s">
+        <v>30</v>
+      </c>
       <c r="F326" s="18"/>
       <c r="G326" s="18"/>
       <c r="H326" s="19"/>
@@ -8244,8 +8268,12 @@
       <c r="C327" s="18" t="s">
         <v>91</v>
       </c>
-      <c r="D327" s="18"/>
-      <c r="E327" s="20"/>
+      <c r="D327" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="E327" s="20" t="s">
+        <v>69</v>
+      </c>
       <c r="F327" s="18"/>
       <c r="G327" s="18"/>
       <c r="H327" s="19"/>
@@ -8260,7 +8288,12 @@
       <c r="C328" s="5">
         <v>0</v>
       </c>
-      <c r="E328" s="5"/>
+      <c r="D328">
+        <v>0</v>
+      </c>
+      <c r="E328">
+        <v>0</v>
+      </c>
       <c r="F328" s="5"/>
       <c r="G328" s="5"/>
       <c r="H328" s="5"/>
@@ -8275,7 +8308,12 @@
       <c r="C329" s="5">
         <v>1</v>
       </c>
-      <c r="E329" s="5"/>
+      <c r="D329">
+        <v>0</v>
+      </c>
+      <c r="E329" s="5">
+        <v>1</v>
+      </c>
       <c r="F329" s="21"/>
       <c r="G329" s="5"/>
       <c r="H329" s="5"/>
@@ -8290,8 +8328,12 @@
       <c r="C330" s="5">
         <v>5</v>
       </c>
-      <c r="D330" s="20"/>
-      <c r="E330" s="5"/>
+      <c r="D330" s="20">
+        <v>0</v>
+      </c>
+      <c r="E330" s="5">
+        <v>70</v>
+      </c>
       <c r="F330" s="5"/>
       <c r="G330" s="5"/>
       <c r="H330" s="5"/>
@@ -8306,8 +8348,12 @@
       <c r="C331" s="5">
         <v>450</v>
       </c>
-      <c r="D331" s="5"/>
-      <c r="E331" s="5"/>
+      <c r="D331" s="5">
+        <v>510</v>
+      </c>
+      <c r="E331" s="5">
+        <v>480</v>
+      </c>
       <c r="F331" s="5"/>
       <c r="G331" s="5"/>
       <c r="H331" s="18"/>
@@ -8348,8 +8394,12 @@
       <c r="C333" s="5">
         <v>0</v>
       </c>
-      <c r="D333" s="5"/>
-      <c r="E333" s="5"/>
+      <c r="D333" s="5">
+        <v>20</v>
+      </c>
+      <c r="E333" s="5">
+        <v>15</v>
+      </c>
       <c r="F333" s="5"/>
       <c r="G333" s="5"/>
       <c r="H333" s="5"/>
@@ -8364,8 +8414,12 @@
       <c r="C334" s="5">
         <v>4</v>
       </c>
-      <c r="D334" s="5"/>
-      <c r="E334" s="5"/>
+      <c r="D334" s="5">
+        <v>4</v>
+      </c>
+      <c r="E334" s="5">
+        <v>4</v>
+      </c>
       <c r="F334" s="5"/>
       <c r="G334" s="5"/>
       <c r="H334" s="5"/>
@@ -8380,8 +8434,12 @@
       <c r="C335" s="5">
         <v>3</v>
       </c>
-      <c r="D335" s="5"/>
-      <c r="E335" s="5"/>
+      <c r="D335" s="5">
+        <v>4</v>
+      </c>
+      <c r="E335" s="5">
+        <v>4</v>
+      </c>
       <c r="F335" s="5"/>
       <c r="G335" s="5"/>
       <c r="H335" s="5"/>
@@ -8396,8 +8454,12 @@
       <c r="C336" s="5">
         <v>4</v>
       </c>
-      <c r="D336" s="5"/>
-      <c r="E336" s="5"/>
+      <c r="D336" s="5">
+        <v>4</v>
+      </c>
+      <c r="E336" s="5">
+        <v>3</v>
+      </c>
       <c r="F336" s="5"/>
       <c r="G336" s="5"/>
       <c r="H336" s="5"/>
@@ -8412,8 +8474,12 @@
       <c r="C337" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D337" s="5"/>
-      <c r="E337" s="5"/>
+      <c r="D337" s="5">
+        <v>70</v>
+      </c>
+      <c r="E337" s="5">
+        <v>0</v>
+      </c>
       <c r="F337" s="5"/>
       <c r="G337" s="5"/>
       <c r="H337" s="5"/>
@@ -8424,6 +8490,12 @@
       </c>
       <c r="C338">
         <v>2</v>
+      </c>
+      <c r="D338" t="s">
+        <v>216</v>
+      </c>
+      <c r="E338" t="s">
+        <v>218</v>
       </c>
     </row>
   </sheetData>

</xml_diff>